<commit_message>
Bug sheet: 56 verified defects (11 grouped rows from the coverage-unlock run); README numbers
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
+++ b/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
@@ -221,8 +221,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:L46" headerRowCount="1">
-  <autoFilter ref="A1:L46"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:L57" headerRowCount="1">
+  <autoFilter ref="A1:L57"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Bug #"/>
     <tableColumn id="2" name="Area"/>
@@ -589,10 +589,11 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>COUNTA(Bugs!A2:A46)</f>
+        <f>COUNTA(Bugs!A2:A57)</f>
         <v/>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
@@ -607,7 +608,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF(Bugs!I2:I46,A7)</f>
+        <f>COUNTIF(Bugs!I2:I57,A7)</f>
         <v/>
       </c>
     </row>
@@ -618,7 +619,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF(Bugs!I2:I46,A8)</f>
+        <f>COUNTIF(Bugs!I2:I57,A8)</f>
         <v/>
       </c>
     </row>
@@ -629,7 +630,7 @@
         </is>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIF(Bugs!I2:I46,A9)</f>
+        <f>COUNTIF(Bugs!I2:I57,A9)</f>
         <v/>
       </c>
     </row>
@@ -640,10 +641,11 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIF(Bugs!I2:I46,A10)</f>
+        <f>COUNTIF(Bugs!I2:I57,A10)</f>
         <v/>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
@@ -658,7 +660,7 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF(Bugs!J2:J46,A13)</f>
+        <f>COUNTIF(Bugs!J2:J57,A13)</f>
         <v/>
       </c>
     </row>
@@ -669,7 +671,7 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF(Bugs!J2:J46,A14)</f>
+        <f>COUNTIF(Bugs!J2:J57,A14)</f>
         <v/>
       </c>
     </row>
@@ -680,7 +682,7 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF(Bugs!J2:J46,A15)</f>
+        <f>COUNTIF(Bugs!J2:J57,A15)</f>
         <v/>
       </c>
     </row>
@@ -691,7 +693,7 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF(Bugs!J2:J46,A16)</f>
+        <f>COUNTIF(Bugs!J2:J57,A16)</f>
         <v/>
       </c>
     </row>
@@ -702,7 +704,7 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF(Bugs!J2:J46,A17)</f>
+        <f>COUNTIF(Bugs!J2:J57,A17)</f>
         <v/>
       </c>
     </row>
@@ -713,7 +715,7 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF(Bugs!J2:J46,A18)</f>
+        <f>COUNTIF(Bugs!J2:J57,A18)</f>
         <v/>
       </c>
     </row>
@@ -724,7 +726,7 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF(Bugs!J2:J46,A19)</f>
+        <f>COUNTIF(Bugs!J2:J57,A19)</f>
         <v/>
       </c>
     </row>
@@ -735,7 +737,7 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF(Bugs!J2:J46,A20)</f>
+        <f>COUNTIF(Bugs!J2:J57,A20)</f>
         <v/>
       </c>
     </row>
@@ -746,10 +748,11 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF(Bugs!J2:J46,A21)</f>
+        <f>COUNTIF(Bugs!J2:J57,A21)</f>
         <v/>
       </c>
     </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
@@ -764,7 +767,7 @@
         </is>
       </c>
       <c r="B24" s="5">
-        <f>COUNTIF(Bugs!H2:H46,"*"&amp;A24&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H57,"*"&amp;A24&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -775,7 +778,7 @@
         </is>
       </c>
       <c r="B25" s="5">
-        <f>COUNTIF(Bugs!H2:H46,"*"&amp;A25&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H57,"*"&amp;A25&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -786,10 +789,11 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF(Bugs!H2:H46,"*"&amp;A26&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H57,"*"&amp;A26&amp;"*")</f>
         <v/>
       </c>
     </row>
+    <row r="27"/>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
@@ -833,7 +837,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L46"/>
+  <dimension ref="A1:L57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1630,7 +1634,7 @@
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Asking for something by an id that does not exist makes the server crash instead of answering 'not found'. Seen on: event details, the lots of an event (read, save draft, reset to smart lots), the auction leader board, the auction report, the counter-offer history, closing a bid and its approval flows, the surrogate-bid approval flows, quote-detail pages and the Master QCS for a proposal from another event. Another screen of the same product answers 'not found' correctly for the same kind of request.</t>
+          <t>Asking for something by an id that does not exist makes the server crash instead of answering 'not found'. Seen on: event details, the lots of an event (read, save draft, reset to smart lots), the auction leader board, the auction report, the counter-offer history, closing a bid and its approval flows, the surrogate-bid approval flows, quote-detail pages, the Master QCS for a proposal from another event, and a vendor opening a round that does not exist. Another screen of the same product answers 'not found' correctly for the same kind of request.</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
@@ -3727,6 +3731,690 @@
         </is>
       </c>
       <c r="L46" s="7" t="inlineStr">
+        <is>
+          <t>3 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
+          <t>BUG-46</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>Adding a round</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>Adding a technical round without a questionnaire crashes</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="inlineStr">
+        <is>
+          <t>A technical (RFP) round is the round where vendors answer a questionnaire. When such a round is added with no questionnaire at all, with an empty questionnaire list, or with a price sheet sent in place of the questionnaire, the server crashes instead of saying a questionnaire is required.</t>
+        </is>
+      </c>
+      <c r="E47" s="7" t="inlineStr">
+        <is>
+          <t>Add a technical round to a draft event and leave out its questionnaire (or send an empty one).</t>
+        </is>
+      </c>
+      <c r="F47" s="7" t="inlineStr">
+        <is>
+          <t>Refused with a clear message such as 'add at least one form to the technical round'. Nothing is saved.</t>
+        </is>
+      </c>
+      <c r="G47" s="7" t="inlineStr">
+        <is>
+          <t>The server crashes.</t>
+        </is>
+      </c>
+      <c r="H47" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I47" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J47" s="7" t="inlineStr">
+        <is>
+          <t>Server crash</t>
+        </is>
+      </c>
+      <c r="K47" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on PROCOL DEMO on 3 Oct 2026: every variant listed failed the same way twice, each time on its own fresh test event.</t>
+        </is>
+      </c>
+      <c r="L47" s="7" t="inlineStr">
+        <is>
+          <t>3 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="7" t="inlineStr">
+        <is>
+          <t>BUG-47</t>
+        </is>
+      </c>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>Adding a round</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>Adding a technical round with an incomplete questionnaire crashes</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="inlineStr">
+        <is>
+          <t>When the questionnaire of a technical round is incomplete, the server crashes instead of pointing at the missing part. Seen with: a vendor-assessment form that has no questions, a form whose pages have no headings, and a tab that has no sections.</t>
+        </is>
+      </c>
+      <c r="E48" s="7" t="inlineStr">
+        <is>
+          <t>Add a technical round to a draft event whose vendor-assessment form has no questions (or whose pages have no headings, or a tab with no sections).</t>
+        </is>
+      </c>
+      <c r="F48" s="7" t="inlineStr">
+        <is>
+          <t>Refused with a message naming what is missing.</t>
+        </is>
+      </c>
+      <c r="G48" s="7" t="inlineStr">
+        <is>
+          <t>The server crashes.</t>
+        </is>
+      </c>
+      <c r="H48" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I48" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J48" s="7" t="inlineStr">
+        <is>
+          <t>Server crash</t>
+        </is>
+      </c>
+      <c r="K48" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on PROCOL DEMO on 3 Oct 2026: every variant listed failed the same way twice, each time on its own fresh test event.</t>
+        </is>
+      </c>
+      <c r="L48" s="7" t="inlineStr">
+        <is>
+          <t>3 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="7" t="inlineStr">
+        <is>
+          <t>BUG-48</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>Adding a round</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>Adding a price round with an incomplete price sheet crashes</t>
+        </is>
+      </c>
+      <c r="D49" s="7" t="inlineStr">
+        <is>
+          <t>The price sheet of a price (RFQ) round lists the columns vendors fill in and the items they price. When it is incomplete, the server crashes instead of refusing it. Seen with: a sheet that has no columns, a drop-down column with no options to choose from, and an item row with no product variant.</t>
+        </is>
+      </c>
+      <c r="E49" s="7" t="inlineStr">
+        <is>
+          <t>Add a price round to a draft event whose price sheet has a drop-down column with no options (or no columns at all, or an item with no variant).</t>
+        </is>
+      </c>
+      <c r="F49" s="7" t="inlineStr">
+        <is>
+          <t>Refused with a message naming what is missing.</t>
+        </is>
+      </c>
+      <c r="G49" s="7" t="inlineStr">
+        <is>
+          <t>The server crashes.</t>
+        </is>
+      </c>
+      <c r="H49" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I49" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J49" s="7" t="inlineStr">
+        <is>
+          <t>Server crash</t>
+        </is>
+      </c>
+      <c r="K49" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on PROCOL DEMO on 3 Oct 2026: every variant listed failed the same way twice, each time on its own fresh test event.</t>
+        </is>
+      </c>
+      <c r="L49" s="7" t="inlineStr">
+        <is>
+          <t>3 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="7" t="inlineStr">
+        <is>
+          <t>BUG-49</t>
+        </is>
+      </c>
+      <c r="B50" s="7" t="inlineStr">
+        <is>
+          <t>Adding a round</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="inlineStr">
+        <is>
+          <t>Adding an auction round with an invalid auction setting crashes</t>
+        </is>
+      </c>
+      <c r="D50" s="7" t="inlineStr">
+        <is>
+          <t>When an auction round is added with an auction setting outside the allowed choices or in the wrong form, the server crashes instead of refusing the setting. Seen with: an auction strategy that does not exist, the knockout step written as text instead of a number, the time-extension trigger written as text or as a fraction (e.g. 2.5 minutes), the 'basket auction' switch written as the word "false" instead of off, and a basket auction whose items carry no per-item terms.</t>
+        </is>
+      </c>
+      <c r="E50" s="7" t="inlineStr">
+        <is>
+          <t>Add an auction round to a draft event with the auction strategy set to a value that does not exist (or the extension trigger set to 2.5).</t>
+        </is>
+      </c>
+      <c r="F50" s="7" t="inlineStr">
+        <is>
+          <t>Refused with a message such as 'invalid auction strategy' or 'extension trigger must be a whole number of minutes'.</t>
+        </is>
+      </c>
+      <c r="G50" s="7" t="inlineStr">
+        <is>
+          <t>The server crashes.</t>
+        </is>
+      </c>
+      <c r="H50" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I50" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J50" s="7" t="inlineStr">
+        <is>
+          <t>Server crash</t>
+        </is>
+      </c>
+      <c r="K50" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on PROCOL DEMO on 3 Oct 2026: every variant listed failed the same way twice, each time on its own fresh test event.</t>
+        </is>
+      </c>
+      <c r="L50" s="7" t="inlineStr">
+        <is>
+          <t>3 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="7" t="inlineStr">
+        <is>
+          <t>BUG-50</t>
+        </is>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>Adding a round</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="inlineStr">
+        <is>
+          <t>Adding a round with its timings in the wrong form crashes</t>
+        </is>
+      </c>
+      <c r="D51" s="7" t="inlineStr">
+        <is>
+          <t>When a round is added with a closing time that is not a real date-time, or as a staggered round (where each item closes at its own time) without the per-item times, the server crashes instead of asking for valid times.</t>
+        </is>
+      </c>
+      <c r="E51" s="7" t="inlineStr">
+        <is>
+          <t>Add a staggered round to a draft event without giving each item its own closing time.</t>
+        </is>
+      </c>
+      <c r="F51" s="7" t="inlineStr">
+        <is>
+          <t>Refused with a message asking for the missing or invalid times.</t>
+        </is>
+      </c>
+      <c r="G51" s="7" t="inlineStr">
+        <is>
+          <t>The server crashes.</t>
+        </is>
+      </c>
+      <c r="H51" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I51" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J51" s="7" t="inlineStr">
+        <is>
+          <t>Server crash</t>
+        </is>
+      </c>
+      <c r="K51" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on PROCOL DEMO on 3 Oct 2026: every variant listed failed the same way twice, each time on its own fresh test event.</t>
+        </is>
+      </c>
+      <c r="L51" s="7" t="inlineStr">
+        <is>
+          <t>3 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="7" t="inlineStr">
+        <is>
+          <t>BUG-51</t>
+        </is>
+      </c>
+      <c r="B52" s="7" t="inlineStr">
+        <is>
+          <t>Adding a round</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>Adding a round with invalid currency settings crashes</t>
+        </is>
+      </c>
+      <c r="D52" s="7" t="inlineStr">
+        <is>
+          <t>When a round's currency settings list no allowed currencies, or name a base currency that is not among the allowed ones, the server crashes. The second case should be a simple refusal: the base currency must be one the vendors are allowed to quote in.</t>
+        </is>
+      </c>
+      <c r="E52" s="7" t="inlineStr">
+        <is>
+          <t>Add a round to a draft event whose base currency is not in its list of allowed currencies.</t>
+        </is>
+      </c>
+      <c r="F52" s="7" t="inlineStr">
+        <is>
+          <t>Refused with a message such as 'base currency must be one of the allowed currencies'.</t>
+        </is>
+      </c>
+      <c r="G52" s="7" t="inlineStr">
+        <is>
+          <t>The server crashes.</t>
+        </is>
+      </c>
+      <c r="H52" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I52" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J52" s="7" t="inlineStr">
+        <is>
+          <t>Server crash</t>
+        </is>
+      </c>
+      <c r="K52" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on PROCOL DEMO on 3 Oct 2026: every variant listed failed the same way twice, each time on its own fresh test event.</t>
+        </is>
+      </c>
+      <c r="L52" s="7" t="inlineStr">
+        <is>
+          <t>3 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="7" t="inlineStr">
+        <is>
+          <t>BUG-52</t>
+        </is>
+      </c>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>Adding a round</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="inlineStr">
+        <is>
+          <t>Adding a round with other settings in the wrong form crashes</t>
+        </is>
+      </c>
+      <c r="D53" s="7" t="inlineStr">
+        <is>
+          <t>Several round settings crash the server when they arrive in the wrong form instead of being refused: an unknown round status, the evaluators written as plain text instead of a list of people, the savings options sent as a list, the auto-award settings sent as text, and the invited-vendor list sent as an empty value.</t>
+        </is>
+      </c>
+      <c r="E53" s="7" t="inlineStr">
+        <is>
+          <t>Add a round to a draft event with the evaluators written as plain text (or any other variant listed).</t>
+        </is>
+      </c>
+      <c r="F53" s="7" t="inlineStr">
+        <is>
+          <t>Refused with a clear message naming the setting.</t>
+        </is>
+      </c>
+      <c r="G53" s="7" t="inlineStr">
+        <is>
+          <t>The server crashes.</t>
+        </is>
+      </c>
+      <c r="H53" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I53" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J53" s="7" t="inlineStr">
+        <is>
+          <t>Server crash</t>
+        </is>
+      </c>
+      <c r="K53" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on PROCOL DEMO on 3 Oct 2026: every variant listed failed the same way twice, each time on its own fresh test event.</t>
+        </is>
+      </c>
+      <c r="L53" s="7" t="inlineStr">
+        <is>
+          <t>3 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="7" t="inlineStr">
+        <is>
+          <t>BUG-53</t>
+        </is>
+      </c>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>Adding a round</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="inlineStr">
+        <is>
+          <t>Adding a technical or auction round with a template that does not exist crashes</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="inlineStr">
+        <is>
+          <t>A price round that names a template that does not exist is wrongly accepted (see the row 'A round can be created with a template that does not exist'). A technical round or an auction round naming a template that does not exist goes further and crashes the server.</t>
+        </is>
+      </c>
+      <c r="E54" s="7" t="inlineStr">
+        <is>
+          <t>Add a technical round (or an auction round) to a draft event, naming a template that does not exist.</t>
+        </is>
+      </c>
+      <c r="F54" s="7" t="inlineStr">
+        <is>
+          <t>Refused with 'template not found'.</t>
+        </is>
+      </c>
+      <c r="G54" s="7" t="inlineStr">
+        <is>
+          <t>The server crashes.</t>
+        </is>
+      </c>
+      <c r="H54" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I54" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J54" s="7" t="inlineStr">
+        <is>
+          <t>Server crash</t>
+        </is>
+      </c>
+      <c r="K54" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on PROCOL DEMO on 3 Oct 2026: every variant listed failed the same way twice, each time on its own fresh test event.</t>
+        </is>
+      </c>
+      <c r="L54" s="7" t="inlineStr">
+        <is>
+          <t>3 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="7" t="inlineStr">
+        <is>
+          <t>BUG-54</t>
+        </is>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>Event update</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="inlineStr">
+        <is>
+          <t>Changing a round's status to an unknown value crashes</t>
+        </is>
+      </c>
+      <c r="D55" s="7" t="inlineStr">
+        <is>
+          <t>Updating a single round of an event with a status word that does not exist (for example 'banana') crashes the server instead of refusing the status. This is about a round; the open question about the same mistake on the whole event is on the 'To confirm' tab.</t>
+        </is>
+      </c>
+      <c r="E55" s="7" t="inlineStr">
+        <is>
+          <t>Publish a test event, then update one of its rounds with the status set to a word that does not exist.</t>
+        </is>
+      </c>
+      <c r="F55" s="7" t="inlineStr">
+        <is>
+          <t>Refused with a message such as 'invalid status'. The round is unchanged.</t>
+        </is>
+      </c>
+      <c r="G55" s="7" t="inlineStr">
+        <is>
+          <t>The server crashes.</t>
+        </is>
+      </c>
+      <c r="H55" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I55" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J55" s="7" t="inlineStr">
+        <is>
+          <t>Server crash</t>
+        </is>
+      </c>
+      <c r="K55" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on PROCOL DEMO on 3 Oct 2026: every variant listed failed the same way twice, each time on its own fresh test event.</t>
+        </is>
+      </c>
+      <c r="L55" s="7" t="inlineStr">
+        <is>
+          <t>3 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="7" t="inlineStr">
+        <is>
+          <t>BUG-55</t>
+        </is>
+      </c>
+      <c r="B56" s="7" t="inlineStr">
+        <is>
+          <t>Bidding &amp; vendor permissions</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="inlineStr">
+        <is>
+          <t>A vendor's answer to 'will you participate?' crashes on an unknown choice</t>
+        </is>
+      </c>
+      <c r="D56" s="7" t="inlineStr">
+        <is>
+          <t>An invited vendor tells the buyer whether they will take part (participate or decline). When the answer sent is not one of those choices (for example 'maybe'), the server crashes instead of refusing it.</t>
+        </is>
+      </c>
+      <c r="E56" s="7" t="inlineStr">
+        <is>
+          <t>1. Invite a QA vendor to a live event.
+2. As the vendor, answer the participation question with a choice that does not exist.</t>
+        </is>
+      </c>
+      <c r="F56" s="7" t="inlineStr">
+        <is>
+          <t>Refused with a message such as 'choose participate or decline'.</t>
+        </is>
+      </c>
+      <c r="G56" s="7" t="inlineStr">
+        <is>
+          <t>The server crashes.</t>
+        </is>
+      </c>
+      <c r="H56" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I56" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J56" s="7" t="inlineStr">
+        <is>
+          <t>Server crash</t>
+        </is>
+      </c>
+      <c r="K56" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on PROCOL DEMO on 3 Oct 2026: every variant listed failed the same way twice, each time on its own fresh test event.</t>
+        </is>
+      </c>
+      <c r="L56" s="7" t="inlineStr">
+        <is>
+          <t>3 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="7" t="inlineStr">
+        <is>
+          <t>BUG-56</t>
+        </is>
+      </c>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>Bidding &amp; vendor permissions</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="inlineStr">
+        <is>
+          <t>A vendor reaching the buyer's 'bid on behalf of a vendor' route crashes it</t>
+        </is>
+      </c>
+      <c r="D57" s="7" t="inlineStr">
+        <is>
+          <t>Entering a bid on a vendor's behalf is a buyer action. A vendor's own login can still reach that route, and with an ordinary request it crashes the server instead of being told it is not allowed. The row 'A vendor that was never invited can still put a bid into an event' shows the same route also lets vendors in.</t>
+        </is>
+      </c>
+      <c r="E57" s="7" t="inlineStr">
+        <is>
+          <t>1. Invite a QA vendor to a live event.
+2. Signed in as that vendor, send a bid through the buyer's 'bid on behalf of a vendor' route.</t>
+        </is>
+      </c>
+      <c r="F57" s="7" t="inlineStr">
+        <is>
+          <t>Refused with 'you are not allowed to perform this action'.</t>
+        </is>
+      </c>
+      <c r="G57" s="7" t="inlineStr">
+        <is>
+          <t>The server crashes.</t>
+        </is>
+      </c>
+      <c r="H57" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I57" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J57" s="7" t="inlineStr">
+        <is>
+          <t>Server crash</t>
+        </is>
+      </c>
+      <c r="K57" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on PROCOL DEMO on 3 Oct 2026: every variant listed failed the same way twice, each time on its own fresh test event.</t>
+        </is>
+      </c>
+      <c r="L57" s="7" t="inlineStr">
         <is>
           <t>3 Oct 2026</t>
         </is>

</xml_diff>

<commit_message>
Bug sheet: 56 verified defects; README numbers
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
+++ b/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
@@ -221,8 +221,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:L46" headerRowCount="1">
-  <autoFilter ref="A1:L46"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:L57" headerRowCount="1">
+  <autoFilter ref="A1:L57"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Bug #"/>
     <tableColumn id="2" name="Area"/>
@@ -589,10 +589,11 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>COUNTA(Bugs!A2:A46)</f>
+        <f>COUNTA(Bugs!A2:A57)</f>
         <v/>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
@@ -607,7 +608,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF(Bugs!I2:I46,A7)</f>
+        <f>COUNTIF(Bugs!I2:I57,A7)</f>
         <v/>
       </c>
     </row>
@@ -618,7 +619,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF(Bugs!I2:I46,A8)</f>
+        <f>COUNTIF(Bugs!I2:I57,A8)</f>
         <v/>
       </c>
     </row>
@@ -629,7 +630,7 @@
         </is>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIF(Bugs!I2:I46,A9)</f>
+        <f>COUNTIF(Bugs!I2:I57,A9)</f>
         <v/>
       </c>
     </row>
@@ -640,10 +641,11 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIF(Bugs!I2:I46,A10)</f>
+        <f>COUNTIF(Bugs!I2:I57,A10)</f>
         <v/>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
@@ -658,7 +660,7 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF(Bugs!J2:J46,A13)</f>
+        <f>COUNTIF(Bugs!J2:J57,A13)</f>
         <v/>
       </c>
     </row>
@@ -669,7 +671,7 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF(Bugs!J2:J46,A14)</f>
+        <f>COUNTIF(Bugs!J2:J57,A14)</f>
         <v/>
       </c>
     </row>
@@ -680,7 +682,7 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF(Bugs!J2:J46,A15)</f>
+        <f>COUNTIF(Bugs!J2:J57,A15)</f>
         <v/>
       </c>
     </row>
@@ -691,7 +693,7 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF(Bugs!J2:J46,A16)</f>
+        <f>COUNTIF(Bugs!J2:J57,A16)</f>
         <v/>
       </c>
     </row>
@@ -702,7 +704,7 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF(Bugs!J2:J46,A17)</f>
+        <f>COUNTIF(Bugs!J2:J57,A17)</f>
         <v/>
       </c>
     </row>
@@ -713,7 +715,7 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF(Bugs!J2:J46,A18)</f>
+        <f>COUNTIF(Bugs!J2:J57,A18)</f>
         <v/>
       </c>
     </row>
@@ -724,7 +726,7 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF(Bugs!J2:J46,A19)</f>
+        <f>COUNTIF(Bugs!J2:J57,A19)</f>
         <v/>
       </c>
     </row>
@@ -735,7 +737,7 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF(Bugs!J2:J46,A20)</f>
+        <f>COUNTIF(Bugs!J2:J57,A20)</f>
         <v/>
       </c>
     </row>
@@ -746,10 +748,11 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF(Bugs!J2:J46,A21)</f>
+        <f>COUNTIF(Bugs!J2:J57,A21)</f>
         <v/>
       </c>
     </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
@@ -764,7 +767,7 @@
         </is>
       </c>
       <c r="B24" s="5">
-        <f>COUNTIF(Bugs!H2:H46,"*"&amp;A24&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H57,"*"&amp;A24&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -775,7 +778,7 @@
         </is>
       </c>
       <c r="B25" s="5">
-        <f>COUNTIF(Bugs!H2:H46,"*"&amp;A25&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H57,"*"&amp;A25&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -786,10 +789,11 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF(Bugs!H2:H46,"*"&amp;A26&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H57,"*"&amp;A26&amp;"*")</f>
         <v/>
       </c>
     </row>
+    <row r="27"/>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
@@ -833,7 +837,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L46"/>
+  <dimension ref="A1:L57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1630,7 +1634,7 @@
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Asking for something by an id that does not exist makes the server crash instead of answering 'not found'. Seen on: event details, the lots of an event (read, save draft, reset to smart lots), the auction leader board, the auction report, the counter-offer history, closing a bid and its approval flows, the surrogate-bid approval flows, quote-detail pages and the Master QCS for a proposal from another event. Another screen of the same product answers 'not found' correctly for the same kind of request.</t>
+          <t>Asking for something by an id that does not exist makes the server crash instead of answering 'not found'. Seen on: event details, the lots of an event (read, save draft, reset to smart lots), the auction leader board, the auction report, the counter-offer history, closing a bid and its approval flows, the surrogate-bid approval flows, quote-detail pages, the Master QCS for a proposal from another event, and a vendor opening a round that does not exist. Another screen of the same product answers 'not found' correctly for the same kind of request.</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
@@ -3727,6 +3731,690 @@
         </is>
       </c>
       <c r="L46" s="7" t="inlineStr">
+        <is>
+          <t>3 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
+          <t>BUG-46</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>Adding a round</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>Adding a technical round without a questionnaire crashes</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="inlineStr">
+        <is>
+          <t>A technical (RFP) round is the round where vendors answer a questionnaire. When such a round is added with no questionnaire at all, with an empty questionnaire list, or with a price sheet sent in place of the questionnaire, the server crashes instead of saying a questionnaire is required.</t>
+        </is>
+      </c>
+      <c r="E47" s="7" t="inlineStr">
+        <is>
+          <t>Add a technical round to a draft event and leave out its questionnaire (or send an empty one).</t>
+        </is>
+      </c>
+      <c r="F47" s="7" t="inlineStr">
+        <is>
+          <t>Refused with a clear message such as 'add at least one form to the technical round'. Nothing is saved.</t>
+        </is>
+      </c>
+      <c r="G47" s="7" t="inlineStr">
+        <is>
+          <t>The server crashes.</t>
+        </is>
+      </c>
+      <c r="H47" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I47" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J47" s="7" t="inlineStr">
+        <is>
+          <t>Server crash</t>
+        </is>
+      </c>
+      <c r="K47" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on PROCOL DEMO on 3 Oct 2026: every variant listed failed the same way twice, each time on its own fresh test event.</t>
+        </is>
+      </c>
+      <c r="L47" s="7" t="inlineStr">
+        <is>
+          <t>3 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="7" t="inlineStr">
+        <is>
+          <t>BUG-47</t>
+        </is>
+      </c>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>Adding a round</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>Adding a technical round with an incomplete questionnaire crashes</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="inlineStr">
+        <is>
+          <t>When the questionnaire of a technical round is incomplete, the server crashes instead of pointing at the missing part. Seen with: a vendor-assessment form that has no questions, a form whose pages have no headings, and a tab that has no sections.</t>
+        </is>
+      </c>
+      <c r="E48" s="7" t="inlineStr">
+        <is>
+          <t>Add a technical round to a draft event whose vendor-assessment form has no questions (or whose pages have no headings, or a tab with no sections).</t>
+        </is>
+      </c>
+      <c r="F48" s="7" t="inlineStr">
+        <is>
+          <t>Refused with a message naming what is missing.</t>
+        </is>
+      </c>
+      <c r="G48" s="7" t="inlineStr">
+        <is>
+          <t>The server crashes.</t>
+        </is>
+      </c>
+      <c r="H48" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I48" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J48" s="7" t="inlineStr">
+        <is>
+          <t>Server crash</t>
+        </is>
+      </c>
+      <c r="K48" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on PROCOL DEMO on 3 Oct 2026: every variant listed failed the same way twice, each time on its own fresh test event.</t>
+        </is>
+      </c>
+      <c r="L48" s="7" t="inlineStr">
+        <is>
+          <t>3 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="7" t="inlineStr">
+        <is>
+          <t>BUG-48</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>Adding a round</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>Adding a price round with an incomplete price sheet crashes</t>
+        </is>
+      </c>
+      <c r="D49" s="7" t="inlineStr">
+        <is>
+          <t>The price sheet of a price (RFQ) round lists the columns vendors fill in and the items they price. When it is incomplete, the server crashes instead of refusing it. Seen with: a sheet that has no columns, a drop-down column with no options to choose from, and an item row with no product variant.</t>
+        </is>
+      </c>
+      <c r="E49" s="7" t="inlineStr">
+        <is>
+          <t>Add a price round to a draft event whose price sheet has a drop-down column with no options (or no columns at all, or an item with no variant).</t>
+        </is>
+      </c>
+      <c r="F49" s="7" t="inlineStr">
+        <is>
+          <t>Refused with a message naming what is missing.</t>
+        </is>
+      </c>
+      <c r="G49" s="7" t="inlineStr">
+        <is>
+          <t>The server crashes.</t>
+        </is>
+      </c>
+      <c r="H49" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I49" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J49" s="7" t="inlineStr">
+        <is>
+          <t>Server crash</t>
+        </is>
+      </c>
+      <c r="K49" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on PROCOL DEMO on 3 Oct 2026: every variant listed failed the same way twice, each time on its own fresh test event.</t>
+        </is>
+      </c>
+      <c r="L49" s="7" t="inlineStr">
+        <is>
+          <t>3 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="7" t="inlineStr">
+        <is>
+          <t>BUG-49</t>
+        </is>
+      </c>
+      <c r="B50" s="7" t="inlineStr">
+        <is>
+          <t>Adding a round</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="inlineStr">
+        <is>
+          <t>Adding an auction round with an invalid auction setting crashes</t>
+        </is>
+      </c>
+      <c r="D50" s="7" t="inlineStr">
+        <is>
+          <t>When an auction round is added with an auction setting outside the allowed choices or in the wrong form, the server crashes instead of refusing the setting. Seen with: an auction strategy that does not exist, the knockout step written as text instead of a number, the time-extension trigger written as text or as a fraction (e.g. 2.5 minutes), the 'basket auction' switch written as the word "false" instead of off, and a basket auction whose items carry no per-item terms.</t>
+        </is>
+      </c>
+      <c r="E50" s="7" t="inlineStr">
+        <is>
+          <t>Add an auction round to a draft event with the auction strategy set to a value that does not exist (or the extension trigger set to 2.5).</t>
+        </is>
+      </c>
+      <c r="F50" s="7" t="inlineStr">
+        <is>
+          <t>Refused with a message such as 'invalid auction strategy' or 'extension trigger must be a whole number of minutes'.</t>
+        </is>
+      </c>
+      <c r="G50" s="7" t="inlineStr">
+        <is>
+          <t>The server crashes.</t>
+        </is>
+      </c>
+      <c r="H50" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I50" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J50" s="7" t="inlineStr">
+        <is>
+          <t>Server crash</t>
+        </is>
+      </c>
+      <c r="K50" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on PROCOL DEMO on 3 Oct 2026: every variant listed failed the same way twice, each time on its own fresh test event.</t>
+        </is>
+      </c>
+      <c r="L50" s="7" t="inlineStr">
+        <is>
+          <t>3 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="7" t="inlineStr">
+        <is>
+          <t>BUG-50</t>
+        </is>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>Adding a round</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="inlineStr">
+        <is>
+          <t>Adding a round with its timings in the wrong form crashes</t>
+        </is>
+      </c>
+      <c r="D51" s="7" t="inlineStr">
+        <is>
+          <t>When a round is added with a closing time that is not a real date-time, or as a staggered round (where each item closes at its own time) without the per-item times, the server crashes instead of asking for valid times.</t>
+        </is>
+      </c>
+      <c r="E51" s="7" t="inlineStr">
+        <is>
+          <t>Add a staggered round to a draft event without giving each item its own closing time.</t>
+        </is>
+      </c>
+      <c r="F51" s="7" t="inlineStr">
+        <is>
+          <t>Refused with a message asking for the missing or invalid times.</t>
+        </is>
+      </c>
+      <c r="G51" s="7" t="inlineStr">
+        <is>
+          <t>The server crashes.</t>
+        </is>
+      </c>
+      <c r="H51" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I51" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J51" s="7" t="inlineStr">
+        <is>
+          <t>Server crash</t>
+        </is>
+      </c>
+      <c r="K51" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on PROCOL DEMO on 3 Oct 2026: every variant listed failed the same way twice, each time on its own fresh test event.</t>
+        </is>
+      </c>
+      <c r="L51" s="7" t="inlineStr">
+        <is>
+          <t>3 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="7" t="inlineStr">
+        <is>
+          <t>BUG-51</t>
+        </is>
+      </c>
+      <c r="B52" s="7" t="inlineStr">
+        <is>
+          <t>Adding a round</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>Adding a round with invalid currency settings crashes</t>
+        </is>
+      </c>
+      <c r="D52" s="7" t="inlineStr">
+        <is>
+          <t>When a round's currency settings list no allowed currencies, or name a base currency that is not among the allowed ones, the server crashes. The second case should be a simple refusal: the base currency must be one the vendors are allowed to quote in.</t>
+        </is>
+      </c>
+      <c r="E52" s="7" t="inlineStr">
+        <is>
+          <t>Add a round to a draft event whose base currency is not in its list of allowed currencies.</t>
+        </is>
+      </c>
+      <c r="F52" s="7" t="inlineStr">
+        <is>
+          <t>Refused with a message such as 'base currency must be one of the allowed currencies'.</t>
+        </is>
+      </c>
+      <c r="G52" s="7" t="inlineStr">
+        <is>
+          <t>The server crashes.</t>
+        </is>
+      </c>
+      <c r="H52" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I52" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J52" s="7" t="inlineStr">
+        <is>
+          <t>Server crash</t>
+        </is>
+      </c>
+      <c r="K52" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on PROCOL DEMO on 3 Oct 2026: every variant listed failed the same way twice, each time on its own fresh test event.</t>
+        </is>
+      </c>
+      <c r="L52" s="7" t="inlineStr">
+        <is>
+          <t>3 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="7" t="inlineStr">
+        <is>
+          <t>BUG-52</t>
+        </is>
+      </c>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>Adding a round</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="inlineStr">
+        <is>
+          <t>Adding a round with other settings in the wrong form crashes</t>
+        </is>
+      </c>
+      <c r="D53" s="7" t="inlineStr">
+        <is>
+          <t>Several round settings crash the server when they arrive in the wrong form instead of being refused: an unknown round status, the evaluators written as plain text instead of a list of people, the savings options sent as a list, the auto-award settings sent as text, and the invited-vendor list sent as an empty value.</t>
+        </is>
+      </c>
+      <c r="E53" s="7" t="inlineStr">
+        <is>
+          <t>Add a round to a draft event with the evaluators written as plain text (or any other variant listed).</t>
+        </is>
+      </c>
+      <c r="F53" s="7" t="inlineStr">
+        <is>
+          <t>Refused with a clear message naming the setting.</t>
+        </is>
+      </c>
+      <c r="G53" s="7" t="inlineStr">
+        <is>
+          <t>The server crashes.</t>
+        </is>
+      </c>
+      <c r="H53" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I53" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J53" s="7" t="inlineStr">
+        <is>
+          <t>Server crash</t>
+        </is>
+      </c>
+      <c r="K53" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on PROCOL DEMO on 3 Oct 2026: every variant listed failed the same way twice, each time on its own fresh test event.</t>
+        </is>
+      </c>
+      <c r="L53" s="7" t="inlineStr">
+        <is>
+          <t>3 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="7" t="inlineStr">
+        <is>
+          <t>BUG-53</t>
+        </is>
+      </c>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>Adding a round</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="inlineStr">
+        <is>
+          <t>Adding a technical or auction round with a template that does not exist crashes</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="inlineStr">
+        <is>
+          <t>A price round that names a template that does not exist is wrongly accepted (see the row 'A round can be created with a template that does not exist'). A technical round or an auction round naming a template that does not exist goes further and crashes the server.</t>
+        </is>
+      </c>
+      <c r="E54" s="7" t="inlineStr">
+        <is>
+          <t>Add a technical round (or an auction round) to a draft event, naming a template that does not exist.</t>
+        </is>
+      </c>
+      <c r="F54" s="7" t="inlineStr">
+        <is>
+          <t>Refused with 'template not found'.</t>
+        </is>
+      </c>
+      <c r="G54" s="7" t="inlineStr">
+        <is>
+          <t>The server crashes.</t>
+        </is>
+      </c>
+      <c r="H54" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I54" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J54" s="7" t="inlineStr">
+        <is>
+          <t>Server crash</t>
+        </is>
+      </c>
+      <c r="K54" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on PROCOL DEMO on 3 Oct 2026: every variant listed failed the same way twice, each time on its own fresh test event.</t>
+        </is>
+      </c>
+      <c r="L54" s="7" t="inlineStr">
+        <is>
+          <t>3 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="7" t="inlineStr">
+        <is>
+          <t>BUG-54</t>
+        </is>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>Event update</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="inlineStr">
+        <is>
+          <t>Changing a round's status to an unknown value crashes</t>
+        </is>
+      </c>
+      <c r="D55" s="7" t="inlineStr">
+        <is>
+          <t>Updating a single round of an event with a status word that does not exist (for example 'banana') crashes the server instead of refusing the status. This is about a round; the open question about the same mistake on the whole event is on the 'To confirm' tab.</t>
+        </is>
+      </c>
+      <c r="E55" s="7" t="inlineStr">
+        <is>
+          <t>Publish a test event, then update one of its rounds with the status set to a word that does not exist.</t>
+        </is>
+      </c>
+      <c r="F55" s="7" t="inlineStr">
+        <is>
+          <t>Refused with a message such as 'invalid status'. The round is unchanged.</t>
+        </is>
+      </c>
+      <c r="G55" s="7" t="inlineStr">
+        <is>
+          <t>The server crashes.</t>
+        </is>
+      </c>
+      <c r="H55" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I55" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J55" s="7" t="inlineStr">
+        <is>
+          <t>Server crash</t>
+        </is>
+      </c>
+      <c r="K55" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on PROCOL DEMO on 3 Oct 2026: every variant listed failed the same way twice, each time on its own fresh test event.</t>
+        </is>
+      </c>
+      <c r="L55" s="7" t="inlineStr">
+        <is>
+          <t>3 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="7" t="inlineStr">
+        <is>
+          <t>BUG-55</t>
+        </is>
+      </c>
+      <c r="B56" s="7" t="inlineStr">
+        <is>
+          <t>Bidding &amp; vendor permissions</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="inlineStr">
+        <is>
+          <t>A vendor's answer to 'will you participate?' crashes on an unknown choice</t>
+        </is>
+      </c>
+      <c r="D56" s="7" t="inlineStr">
+        <is>
+          <t>An invited vendor tells the buyer whether they will take part (participate or decline). When the answer sent is not one of those choices (for example 'maybe'), the server crashes instead of refusing it.</t>
+        </is>
+      </c>
+      <c r="E56" s="7" t="inlineStr">
+        <is>
+          <t>1. Invite a QA vendor to a live event.
+2. As the vendor, answer the participation question with a choice that does not exist.</t>
+        </is>
+      </c>
+      <c r="F56" s="7" t="inlineStr">
+        <is>
+          <t>Refused with a message such as 'choose participate or decline'.</t>
+        </is>
+      </c>
+      <c r="G56" s="7" t="inlineStr">
+        <is>
+          <t>The server crashes.</t>
+        </is>
+      </c>
+      <c r="H56" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I56" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J56" s="7" t="inlineStr">
+        <is>
+          <t>Server crash</t>
+        </is>
+      </c>
+      <c r="K56" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on PROCOL DEMO on 3 Oct 2026: every variant listed failed the same way twice, each time on its own fresh test event.</t>
+        </is>
+      </c>
+      <c r="L56" s="7" t="inlineStr">
+        <is>
+          <t>3 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="7" t="inlineStr">
+        <is>
+          <t>BUG-56</t>
+        </is>
+      </c>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>Bidding &amp; vendor permissions</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="inlineStr">
+        <is>
+          <t>A vendor reaching the buyer's 'bid on behalf of a vendor' route crashes it</t>
+        </is>
+      </c>
+      <c r="D57" s="7" t="inlineStr">
+        <is>
+          <t>Entering a bid on a vendor's behalf is a buyer action. A vendor's own login can still reach that route, and with an ordinary request it crashes the server instead of being told it is not allowed. The row 'A vendor that was never invited can still put a bid into an event' shows the same route also lets vendors in.</t>
+        </is>
+      </c>
+      <c r="E57" s="7" t="inlineStr">
+        <is>
+          <t>1. Invite a QA vendor to a live event.
+2. Signed in as that vendor, send a bid through the buyer's 'bid on behalf of a vendor' route.</t>
+        </is>
+      </c>
+      <c r="F57" s="7" t="inlineStr">
+        <is>
+          <t>Refused with 'you are not allowed to perform this action'.</t>
+        </is>
+      </c>
+      <c r="G57" s="7" t="inlineStr">
+        <is>
+          <t>The server crashes.</t>
+        </is>
+      </c>
+      <c r="H57" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I57" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J57" s="7" t="inlineStr">
+        <is>
+          <t>Server crash</t>
+        </is>
+      </c>
+      <c r="K57" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on PROCOL DEMO on 3 Oct 2026: every variant listed failed the same way twice, each time on its own fresh test event.</t>
+        </is>
+      </c>
+      <c r="L57" s="7" t="inlineStr">
         <is>
           <t>3 Oct 2026</t>
         </is>

</xml_diff>

<commit_message>
Known bugs recognised by exact test-case id, never by similarity
- Bug sheet gains a 'Test cases' column (15 rows filled where ids are known).
- Memory labels each known-bug chunk with those ids; the oracle marks a finding
  'already on the bug sheet as BUG-xx' only on an exact id match. The old
  similarity rule (score > 0.85) never fired and could have hidden a new bug.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
+++ b/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
@@ -221,9 +221,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:L57" headerRowCount="1">
-  <autoFilter ref="A1:L57"/>
-  <tableColumns count="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:M57" headerRowCount="1">
+  <autoFilter ref="A1:M57"/>
+  <tableColumns count="13">
     <tableColumn id="1" name="Bug #"/>
     <tableColumn id="2" name="Area"/>
     <tableColumn id="3" name="Bug"/>
@@ -236,6 +236,7 @@
     <tableColumn id="10" name="Kind"/>
     <tableColumn id="11" name="How it was verified"/>
     <tableColumn id="12" name="Last confirmed"/>
+    <tableColumn id="13" name="Test cases"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showRowStripes="0"/>
 </table>
@@ -837,7 +838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L57"/>
+  <dimension ref="A1:M57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -852,6 +853,7 @@
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="40" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="28" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -915,6 +917,11 @@
           <t>Last confirmed</t>
         </is>
       </c>
+      <c r="M1" s="6" t="inlineStr">
+        <is>
+          <t>Test cases</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
@@ -979,6 +986,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M2" s="7" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
@@ -1042,6 +1050,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M3" s="7" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
@@ -1106,6 +1115,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M4" s="7" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -1170,6 +1180,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M5" s="7" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -1234,6 +1245,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M6" s="7" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
@@ -1297,6 +1309,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M7" s="7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
@@ -1361,6 +1374,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M8" s="7" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
@@ -1424,6 +1438,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M9" s="7" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
@@ -1487,6 +1502,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M10" s="7" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -1552,6 +1568,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M11" s="7" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
@@ -1615,6 +1632,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M12" s="7" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
@@ -1677,6 +1695,11 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M13" s="7" t="inlineStr">
+        <is>
+          <t>EDGE-BID-018</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -1739,6 +1762,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M14" s="7" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -1801,6 +1825,11 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M15" s="7" t="inlineStr">
+        <is>
+          <t>API-VAL-003</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -1863,6 +1892,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M16" s="7" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -1926,6 +1956,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M17" s="7" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -1988,6 +2019,11 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M18" s="7" t="inlineStr">
+        <is>
+          <t>EDGE-STG-095</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -2050,6 +2086,11 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M19" s="7" t="inlineStr">
+        <is>
+          <t>EDGE-STG-074</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -2112,6 +2153,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M20" s="7" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -2174,6 +2216,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M21" s="7" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -2236,6 +2279,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M22" s="7" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -2298,6 +2342,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M23" s="7" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -2360,6 +2405,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M24" s="7" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -2422,6 +2468,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M25" s="7" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -2486,6 +2533,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M26" s="7" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -2549,6 +2597,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M27" s="7" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -2612,6 +2661,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M28" s="7" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -2675,6 +2725,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M29" s="7" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -2738,6 +2789,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M30" s="7" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -2801,6 +2853,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M31" s="7" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -2863,6 +2916,7 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M32" s="7" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -2925,6 +2979,7 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M33" s="7" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -2987,6 +3042,7 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M34" s="7" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -3049,6 +3105,7 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M35" s="7" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -3111,6 +3168,7 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M36" s="7" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -3175,6 +3233,7 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M37" s="7" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -3238,6 +3297,7 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M38" s="7" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -3300,6 +3360,7 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M39" s="7" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -3362,6 +3423,7 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M40" s="7" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -3424,6 +3486,7 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M41" s="7" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -3486,6 +3549,7 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M42" s="7" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -3548,6 +3612,7 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M43" s="7" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -3611,6 +3676,7 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M44" s="7" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -3673,6 +3739,7 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M45" s="7" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -3735,6 +3802,7 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M46" s="7" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -3797,6 +3865,11 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M47" s="7" t="inlineStr">
+        <is>
+          <t>EDGE-STG-006, EDGE-STG-072, EDGE-STG-073</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -3859,6 +3932,11 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M48" s="7" t="inlineStr">
+        <is>
+          <t>EDGE-STG-075, EDGE-STG-076, EDGE-STG-102</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -3921,6 +3999,11 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M49" s="7" t="inlineStr">
+        <is>
+          <t>EDGE-STG-096, EDGE-STG-098, EDGE-STG-099</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -3983,6 +4066,11 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M50" s="7" t="inlineStr">
+        <is>
+          <t>EDGE-STG-036, EDGE-STG-047, EDGE-STG-055, EDGE-STG-056, EDGE-STG-066, EDGE-STG-067</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -4045,6 +4133,11 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M51" s="7" t="inlineStr">
+        <is>
+          <t>EDGE-STG-033, EDGE-STG-035</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -4107,6 +4200,11 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M52" s="7" t="inlineStr">
+        <is>
+          <t>EDGE-STG-109, EDGE-STG-111</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -4169,6 +4267,11 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M53" s="7" t="inlineStr">
+        <is>
+          <t>EDGE-STG-015, EDGE-STG-085, EDGE-STG-105, EDGE-STG-112, EDGE-STG-116</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -4231,6 +4334,11 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M54" s="7" t="inlineStr">
+        <is>
+          <t>EDGE-STG-089, EDGE-STG-090</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -4293,6 +4401,11 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M55" s="7" t="inlineStr">
+        <is>
+          <t>EDGE-PUB-073</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -4356,6 +4469,11 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M56" s="7" t="inlineStr">
+        <is>
+          <t>EDGE-BID-005</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -4417,6 +4535,11 @@
       <c r="L57" s="7" t="inlineStr">
         <is>
           <t>3 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M57" s="7" t="inlineStr">
+        <is>
+          <t>BID-SURR-002</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Known bugs recognised by exact test-case id
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
+++ b/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
@@ -221,9 +221,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:L57" headerRowCount="1">
-  <autoFilter ref="A1:L57"/>
-  <tableColumns count="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:M57" headerRowCount="1">
+  <autoFilter ref="A1:M57"/>
+  <tableColumns count="13">
     <tableColumn id="1" name="Bug #"/>
     <tableColumn id="2" name="Area"/>
     <tableColumn id="3" name="Bug"/>
@@ -236,6 +236,7 @@
     <tableColumn id="10" name="Kind"/>
     <tableColumn id="11" name="How it was verified"/>
     <tableColumn id="12" name="Last confirmed"/>
+    <tableColumn id="13" name="Test cases"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showRowStripes="0"/>
 </table>
@@ -837,7 +838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L57"/>
+  <dimension ref="A1:M57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -852,6 +853,7 @@
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="40" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="28" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -915,6 +917,11 @@
           <t>Last confirmed</t>
         </is>
       </c>
+      <c r="M1" s="6" t="inlineStr">
+        <is>
+          <t>Test cases</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
@@ -979,6 +986,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M2" s="7" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
@@ -1042,6 +1050,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M3" s="7" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
@@ -1106,6 +1115,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M4" s="7" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -1170,6 +1180,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M5" s="7" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -1234,6 +1245,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M6" s="7" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
@@ -1297,6 +1309,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M7" s="7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
@@ -1361,6 +1374,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M8" s="7" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
@@ -1424,6 +1438,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M9" s="7" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
@@ -1487,6 +1502,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M10" s="7" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -1552,6 +1568,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M11" s="7" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
@@ -1615,6 +1632,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M12" s="7" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
@@ -1677,6 +1695,11 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M13" s="7" t="inlineStr">
+        <is>
+          <t>EDGE-BID-018</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -1739,6 +1762,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M14" s="7" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -1801,6 +1825,11 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M15" s="7" t="inlineStr">
+        <is>
+          <t>API-VAL-003</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -1863,6 +1892,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M16" s="7" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -1926,6 +1956,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M17" s="7" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -1988,6 +2019,11 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M18" s="7" t="inlineStr">
+        <is>
+          <t>EDGE-STG-095</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -2050,6 +2086,11 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M19" s="7" t="inlineStr">
+        <is>
+          <t>EDGE-STG-074</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -2112,6 +2153,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M20" s="7" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -2174,6 +2216,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M21" s="7" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -2236,6 +2279,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M22" s="7" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -2298,6 +2342,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M23" s="7" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -2360,6 +2405,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M24" s="7" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -2422,6 +2468,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M25" s="7" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -2486,6 +2533,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M26" s="7" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -2549,6 +2597,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M27" s="7" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -2612,6 +2661,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M28" s="7" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -2675,6 +2725,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M29" s="7" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -2738,6 +2789,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M30" s="7" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -2801,6 +2853,7 @@
           <t>1 Oct 2026</t>
         </is>
       </c>
+      <c r="M31" s="7" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -2863,6 +2916,7 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M32" s="7" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -2925,6 +2979,7 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M33" s="7" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -2987,6 +3042,7 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M34" s="7" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -3049,6 +3105,7 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M35" s="7" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -3111,6 +3168,7 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M36" s="7" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -3175,6 +3233,7 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M37" s="7" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -3238,6 +3297,7 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M38" s="7" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -3300,6 +3360,7 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M39" s="7" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -3362,6 +3423,7 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M40" s="7" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -3424,6 +3486,7 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M41" s="7" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -3486,6 +3549,7 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M42" s="7" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -3548,6 +3612,7 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M43" s="7" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -3611,6 +3676,7 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M44" s="7" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -3673,6 +3739,7 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M45" s="7" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -3735,6 +3802,7 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M46" s="7" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -3797,6 +3865,11 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M47" s="7" t="inlineStr">
+        <is>
+          <t>EDGE-STG-006, EDGE-STG-072, EDGE-STG-073</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -3859,6 +3932,11 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M48" s="7" t="inlineStr">
+        <is>
+          <t>EDGE-STG-075, EDGE-STG-076, EDGE-STG-102</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -3921,6 +3999,11 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M49" s="7" t="inlineStr">
+        <is>
+          <t>EDGE-STG-096, EDGE-STG-098, EDGE-STG-099</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -3983,6 +4066,11 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M50" s="7" t="inlineStr">
+        <is>
+          <t>EDGE-STG-036, EDGE-STG-047, EDGE-STG-055, EDGE-STG-056, EDGE-STG-066, EDGE-STG-067</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -4045,6 +4133,11 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M51" s="7" t="inlineStr">
+        <is>
+          <t>EDGE-STG-033, EDGE-STG-035</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -4107,6 +4200,11 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M52" s="7" t="inlineStr">
+        <is>
+          <t>EDGE-STG-109, EDGE-STG-111</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -4169,6 +4267,11 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M53" s="7" t="inlineStr">
+        <is>
+          <t>EDGE-STG-015, EDGE-STG-085, EDGE-STG-105, EDGE-STG-112, EDGE-STG-116</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -4231,6 +4334,11 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M54" s="7" t="inlineStr">
+        <is>
+          <t>EDGE-STG-089, EDGE-STG-090</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -4293,6 +4401,11 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M55" s="7" t="inlineStr">
+        <is>
+          <t>EDGE-PUB-073</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -4356,6 +4469,11 @@
           <t>3 Oct 2026</t>
         </is>
       </c>
+      <c r="M56" s="7" t="inlineStr">
+        <is>
+          <t>EDGE-BID-005</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -4417,6 +4535,11 @@
       <c r="L57" s="7" t="inlineStr">
         <is>
           <t>3 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M57" s="7" t="inlineStr">
+        <is>
+          <t>BID-SURR-002</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bug sheet: 59 verified defects (3 from the UI<->API cross-check), 9 to confirm; README numbers
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
+++ b/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
@@ -221,8 +221,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:M57" headerRowCount="1">
-  <autoFilter ref="A1:M57"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:M60" headerRowCount="1">
+  <autoFilter ref="A1:M60"/>
   <tableColumns count="13">
     <tableColumn id="1" name="Bug #"/>
     <tableColumn id="2" name="Area"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Confirm" displayName="Confirm" ref="A1:F8" headerRowCount="1">
-  <autoFilter ref="A1:F8"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Confirm" displayName="Confirm" ref="A1:F10" headerRowCount="1">
+  <autoFilter ref="A1:F10"/>
   <tableColumns count="6">
     <tableColumn id="1" name="#"/>
     <tableColumn id="2" name="Area"/>
@@ -590,7 +590,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>COUNTA(Bugs!A2:A57)</f>
+        <f>COUNTA(Bugs!A2:A60)</f>
         <v/>
       </c>
     </row>
@@ -609,7 +609,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF(Bugs!I2:I57,A7)</f>
+        <f>COUNTIF(Bugs!I2:I60,A7)</f>
         <v/>
       </c>
     </row>
@@ -620,7 +620,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF(Bugs!I2:I57,A8)</f>
+        <f>COUNTIF(Bugs!I2:I60,A8)</f>
         <v/>
       </c>
     </row>
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIF(Bugs!I2:I57,A9)</f>
+        <f>COUNTIF(Bugs!I2:I60,A9)</f>
         <v/>
       </c>
     </row>
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIF(Bugs!I2:I57,A10)</f>
+        <f>COUNTIF(Bugs!I2:I60,A10)</f>
         <v/>
       </c>
     </row>
@@ -661,7 +661,7 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF(Bugs!J2:J57,A13)</f>
+        <f>COUNTIF(Bugs!J2:J60,A13)</f>
         <v/>
       </c>
     </row>
@@ -672,7 +672,7 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF(Bugs!J2:J57,A14)</f>
+        <f>COUNTIF(Bugs!J2:J60,A14)</f>
         <v/>
       </c>
     </row>
@@ -683,7 +683,7 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF(Bugs!J2:J57,A15)</f>
+        <f>COUNTIF(Bugs!J2:J60,A15)</f>
         <v/>
       </c>
     </row>
@@ -694,7 +694,7 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF(Bugs!J2:J57,A16)</f>
+        <f>COUNTIF(Bugs!J2:J60,A16)</f>
         <v/>
       </c>
     </row>
@@ -705,7 +705,7 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF(Bugs!J2:J57,A17)</f>
+        <f>COUNTIF(Bugs!J2:J60,A17)</f>
         <v/>
       </c>
     </row>
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF(Bugs!J2:J57,A18)</f>
+        <f>COUNTIF(Bugs!J2:J60,A18)</f>
         <v/>
       </c>
     </row>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF(Bugs!J2:J57,A19)</f>
+        <f>COUNTIF(Bugs!J2:J60,A19)</f>
         <v/>
       </c>
     </row>
@@ -738,7 +738,7 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF(Bugs!J2:J57,A20)</f>
+        <f>COUNTIF(Bugs!J2:J60,A20)</f>
         <v/>
       </c>
     </row>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF(Bugs!J2:J57,A21)</f>
+        <f>COUNTIF(Bugs!J2:J60,A21)</f>
         <v/>
       </c>
     </row>
@@ -768,7 +768,7 @@
         </is>
       </c>
       <c r="B24" s="5">
-        <f>COUNTIF(Bugs!H2:H57,"*"&amp;A24&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H60,"*"&amp;A24&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B25" s="5">
-        <f>COUNTIF(Bugs!H2:H57,"*"&amp;A25&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H60,"*"&amp;A25&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF(Bugs!H2:H57,"*"&amp;A26&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H60,"*"&amp;A26&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -809,7 +809,7 @@
         </is>
       </c>
       <c r="B29" s="5">
-        <f>COUNTA('Needs confirmation'!A2:A8)</f>
+        <f>COUNTA('Needs confirmation'!A2:A10)</f>
         <v/>
       </c>
     </row>
@@ -838,7 +838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M57"/>
+  <dimension ref="A1:M60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4543,6 +4543,212 @@
         </is>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" s="7" t="inlineStr">
+        <is>
+          <t>BUG-57</t>
+        </is>
+      </c>
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>Event screens</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="inlineStr">
+        <is>
+          <t>The Overview tab shows the wrong number of seconds for a stage's duration and evaluation time</t>
+        </is>
+      </c>
+      <c r="D58" s="7" t="inlineStr">
+        <is>
+          <t>On a stage's Overview tab, Order Configurations shows how long bidding lasts and how long evaluation lasts. The seconds part is wrong: the screen prints the minutes figure in place of the seconds. A window of 2 minutes 50 seconds reads '2 mins 2 seconds', and a 10-second evaluation time reads '0 second'. The backend sends the right times; only the screen's wording is wrong.</t>
+        </is>
+      </c>
+      <c r="E58" s="7" t="inlineStr">
+        <is>
+          <t>1. Open a published event and click one of its stages.
+2. Open the Overview tab and read Order Duration and Evaluation Time.
+3. Compare them with the stage's start, end and extra closing time.</t>
+        </is>
+      </c>
+      <c r="F58" s="7" t="inlineStr">
+        <is>
+          <t>The durations read correctly, e.g. '2 mins 50 seconds' and '10 seconds'.</t>
+        </is>
+      </c>
+      <c r="G58" s="7" t="inlineStr">
+        <is>
+          <t>The seconds are wrong: '2 mins 2 seconds' and '0 second'.</t>
+        </is>
+      </c>
+      <c r="H58" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO; Demo Account 2</t>
+        </is>
+      </c>
+      <c r="I58" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J58" s="7" t="inlineStr">
+        <is>
+          <t>Screen shows wrong data</t>
+        </is>
+      </c>
+      <c r="K58" s="7" t="inlineStr">
+        <is>
+          <t>Seen on 8 fresh test events (4 per client), comparing what the backend sent with what the screen shows. The console's duration formatter prints the minutes value as the seconds (utils/index.js:567-568).</t>
+        </is>
+      </c>
+      <c r="L58" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M58" s="7" t="inlineStr">
+        <is>
+          <t>UI-XCHK-033</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="7" t="inlineStr">
+        <is>
+          <t>BUG-58</t>
+        </is>
+      </c>
+      <c r="B59" s="7" t="inlineStr">
+        <is>
+          <t>Awarding</t>
+        </is>
+      </c>
+      <c r="C59" s="7" t="inlineStr">
+        <is>
+          <t>On the award proposal page, the Participants list is numbered 'NaN' instead of 1, 2, 3</t>
+        </is>
+      </c>
+      <c r="D59" s="7" t="inlineStr">
+        <is>
+          <t>The award proposal page has a Participants panel listing the invited vendors. Its 'S No.' column shows 'NaN' (not a number) on every row instead of 1, 2, 3, because the page uses the participants table without telling it which page of the list it is on.</t>
+        </is>
+      </c>
+      <c r="E59" s="7" t="inlineStr">
+        <is>
+          <t>1. Open an event that has an award proposal.
+2. Open Master QCS and click 'Bid Selection Proposal'.
+3. Open the Participants panel and read the S No. column.</t>
+        </is>
+      </c>
+      <c r="F59" s="7" t="inlineStr">
+        <is>
+          <t>The rows are numbered 1, 2, 3 …</t>
+        </is>
+      </c>
+      <c r="G59" s="7" t="inlineStr">
+        <is>
+          <t>Every row shows 'NaN'.</t>
+        </is>
+      </c>
+      <c r="H59" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO; Demo Account 2</t>
+        </is>
+      </c>
+      <c r="I59" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J59" s="7" t="inlineStr">
+        <is>
+          <t>Screen shows wrong data</t>
+        </is>
+      </c>
+      <c r="K59" s="7" t="inlineStr">
+        <is>
+          <t>Seen on 7 fresh test events (4 on Demo Account 2, 3 on PROCOL DEMO). Cause in the console code: projectProposal.jsx:1175 renders the table without a page number, which participantsTable.jsx:153-155 needs for the numbering.</t>
+        </is>
+      </c>
+      <c r="L59" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M59" s="7" t="inlineStr">
+        <is>
+          <t>UI-XCHK-PROP-005</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="7" t="inlineStr">
+        <is>
+          <t>BUG-59</t>
+        </is>
+      </c>
+      <c r="B60" s="7" t="inlineStr">
+        <is>
+          <t>Event screens</t>
+        </is>
+      </c>
+      <c r="C60" s="7" t="inlineStr">
+        <is>
+          <t>The Price Trends tab fails with a server crash on Demo Account 2</t>
+        </is>
+      </c>
+      <c r="D60" s="7" t="inlineStr">
+        <is>
+          <t>A pricing or auction stage has a Price Trends tab that shows past deals for the same products. On Demo Account 2 the request behind this tab crashes on the server for every stage, so no past prices can ever be shown there. The same tab works on PROCOL DEMO.</t>
+        </is>
+      </c>
+      <c r="E60" s="7" t="inlineStr">
+        <is>
+          <t>1. On Demo Account 2, open any pricing or auction stage.
+2. Click the Price Trends tab.</t>
+        </is>
+      </c>
+      <c r="F60" s="7" t="inlineStr">
+        <is>
+          <t>Past deals for the stage's products are listed (or 'no past deals').</t>
+        </is>
+      </c>
+      <c r="G60" s="7" t="inlineStr">
+        <is>
+          <t>The server crashes and no price history is shown.</t>
+        </is>
+      </c>
+      <c r="H60" s="7" t="inlineStr">
+        <is>
+          <t>Demo Account 2</t>
+        </is>
+      </c>
+      <c r="I60" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J60" s="7" t="inlineStr">
+        <is>
+          <t>Server crash</t>
+        </is>
+      </c>
+      <c r="K60" s="7" t="inlineStr">
+        <is>
+          <t>The price-trends request answered with a server error on 4 of 4 fresh test events on Demo Account 2; PROCOL DEMO answered normally for the same kind of stage.</t>
+        </is>
+      </c>
+      <c r="L60" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M60" s="7" t="inlineStr">
+        <is>
+          <t>UI-XCHK-TRND-001</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
@@ -4557,7 +4763,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -4821,6 +5027,70 @@
       <c r="F8" s="7" t="inlineStr">
         <is>
           <t>Confirm whether attachments must always come from Procol's own storage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Q-08</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Event screens</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Two tabs of the same stage show different savings</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>When savings are compared on the whole lot, a stage's Responses tab shows savings of ₹30 while its Overview tab shows '–' for the same stage. The Overview reads the first bidder's own savings record, which the backend leaves empty in this mode.</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Demo Account 2</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>Decide which is right: should the backend fill the bidder's savings in lot mode, or should the Overview read the stage's total savings? Seen on 2 of 2 auction test events.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Q-09</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Events list</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Searching the events list straight after opening it can show the wrong events</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Typing an event's title into the search box as soon as the events list opens sometimes leaves the newest ten events on screen instead of the one event the search returned, while the search box still shows the title. It happened in about 1 run in 3, on both clients.</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO; Demo Account 2</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>Confirm in the screen's code whether an older list response can overwrite the search result (a race between the first load and the search). It is intermittent, so it is not yet counted as a verified bug.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
UI<->API cross-check on 12 screens; bug sheet 59 verified defects
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
+++ b/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
@@ -221,8 +221,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:M57" headerRowCount="1">
-  <autoFilter ref="A1:M57"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:M60" headerRowCount="1">
+  <autoFilter ref="A1:M60"/>
   <tableColumns count="13">
     <tableColumn id="1" name="Bug #"/>
     <tableColumn id="2" name="Area"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Confirm" displayName="Confirm" ref="A1:F8" headerRowCount="1">
-  <autoFilter ref="A1:F8"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Confirm" displayName="Confirm" ref="A1:F10" headerRowCount="1">
+  <autoFilter ref="A1:F10"/>
   <tableColumns count="6">
     <tableColumn id="1" name="#"/>
     <tableColumn id="2" name="Area"/>
@@ -590,7 +590,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>COUNTA(Bugs!A2:A57)</f>
+        <f>COUNTA(Bugs!A2:A60)</f>
         <v/>
       </c>
     </row>
@@ -609,7 +609,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF(Bugs!I2:I57,A7)</f>
+        <f>COUNTIF(Bugs!I2:I60,A7)</f>
         <v/>
       </c>
     </row>
@@ -620,7 +620,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF(Bugs!I2:I57,A8)</f>
+        <f>COUNTIF(Bugs!I2:I60,A8)</f>
         <v/>
       </c>
     </row>
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIF(Bugs!I2:I57,A9)</f>
+        <f>COUNTIF(Bugs!I2:I60,A9)</f>
         <v/>
       </c>
     </row>
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIF(Bugs!I2:I57,A10)</f>
+        <f>COUNTIF(Bugs!I2:I60,A10)</f>
         <v/>
       </c>
     </row>
@@ -661,7 +661,7 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF(Bugs!J2:J57,A13)</f>
+        <f>COUNTIF(Bugs!J2:J60,A13)</f>
         <v/>
       </c>
     </row>
@@ -672,7 +672,7 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF(Bugs!J2:J57,A14)</f>
+        <f>COUNTIF(Bugs!J2:J60,A14)</f>
         <v/>
       </c>
     </row>
@@ -683,7 +683,7 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF(Bugs!J2:J57,A15)</f>
+        <f>COUNTIF(Bugs!J2:J60,A15)</f>
         <v/>
       </c>
     </row>
@@ -694,7 +694,7 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF(Bugs!J2:J57,A16)</f>
+        <f>COUNTIF(Bugs!J2:J60,A16)</f>
         <v/>
       </c>
     </row>
@@ -705,7 +705,7 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF(Bugs!J2:J57,A17)</f>
+        <f>COUNTIF(Bugs!J2:J60,A17)</f>
         <v/>
       </c>
     </row>
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF(Bugs!J2:J57,A18)</f>
+        <f>COUNTIF(Bugs!J2:J60,A18)</f>
         <v/>
       </c>
     </row>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF(Bugs!J2:J57,A19)</f>
+        <f>COUNTIF(Bugs!J2:J60,A19)</f>
         <v/>
       </c>
     </row>
@@ -738,7 +738,7 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF(Bugs!J2:J57,A20)</f>
+        <f>COUNTIF(Bugs!J2:J60,A20)</f>
         <v/>
       </c>
     </row>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF(Bugs!J2:J57,A21)</f>
+        <f>COUNTIF(Bugs!J2:J60,A21)</f>
         <v/>
       </c>
     </row>
@@ -768,7 +768,7 @@
         </is>
       </c>
       <c r="B24" s="5">
-        <f>COUNTIF(Bugs!H2:H57,"*"&amp;A24&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H60,"*"&amp;A24&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B25" s="5">
-        <f>COUNTIF(Bugs!H2:H57,"*"&amp;A25&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H60,"*"&amp;A25&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF(Bugs!H2:H57,"*"&amp;A26&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H60,"*"&amp;A26&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -809,7 +809,7 @@
         </is>
       </c>
       <c r="B29" s="5">
-        <f>COUNTA('Needs confirmation'!A2:A8)</f>
+        <f>COUNTA('Needs confirmation'!A2:A10)</f>
         <v/>
       </c>
     </row>
@@ -838,7 +838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M57"/>
+  <dimension ref="A1:M60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4543,6 +4543,212 @@
         </is>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" s="7" t="inlineStr">
+        <is>
+          <t>BUG-57</t>
+        </is>
+      </c>
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>Event screens</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="inlineStr">
+        <is>
+          <t>The Overview tab shows the wrong number of seconds for a stage's duration and evaluation time</t>
+        </is>
+      </c>
+      <c r="D58" s="7" t="inlineStr">
+        <is>
+          <t>On a stage's Overview tab, Order Configurations shows how long bidding lasts and how long evaluation lasts. The seconds part is wrong: the screen prints the minutes figure in place of the seconds. A window of 2 minutes 50 seconds reads '2 mins 2 seconds', and a 10-second evaluation time reads '0 second'. The backend sends the right times; only the screen's wording is wrong.</t>
+        </is>
+      </c>
+      <c r="E58" s="7" t="inlineStr">
+        <is>
+          <t>1. Open a published event and click one of its stages.
+2. Open the Overview tab and read Order Duration and Evaluation Time.
+3. Compare them with the stage's start, end and extra closing time.</t>
+        </is>
+      </c>
+      <c r="F58" s="7" t="inlineStr">
+        <is>
+          <t>The durations read correctly, e.g. '2 mins 50 seconds' and '10 seconds'.</t>
+        </is>
+      </c>
+      <c r="G58" s="7" t="inlineStr">
+        <is>
+          <t>The seconds are wrong: '2 mins 2 seconds' and '0 second'.</t>
+        </is>
+      </c>
+      <c r="H58" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO; Demo Account 2</t>
+        </is>
+      </c>
+      <c r="I58" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J58" s="7" t="inlineStr">
+        <is>
+          <t>Screen shows wrong data</t>
+        </is>
+      </c>
+      <c r="K58" s="7" t="inlineStr">
+        <is>
+          <t>Seen on 8 fresh test events (4 per client), comparing what the backend sent with what the screen shows. The console's duration formatter prints the minutes value as the seconds (utils/index.js:567-568).</t>
+        </is>
+      </c>
+      <c r="L58" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M58" s="7" t="inlineStr">
+        <is>
+          <t>UI-XCHK-033</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="7" t="inlineStr">
+        <is>
+          <t>BUG-58</t>
+        </is>
+      </c>
+      <c r="B59" s="7" t="inlineStr">
+        <is>
+          <t>Awarding</t>
+        </is>
+      </c>
+      <c r="C59" s="7" t="inlineStr">
+        <is>
+          <t>On the award proposal page, the Participants list is numbered 'NaN' instead of 1, 2, 3</t>
+        </is>
+      </c>
+      <c r="D59" s="7" t="inlineStr">
+        <is>
+          <t>The award proposal page has a Participants panel listing the invited vendors. Its 'S No.' column shows 'NaN' (not a number) on every row instead of 1, 2, 3, because the page uses the participants table without telling it which page of the list it is on.</t>
+        </is>
+      </c>
+      <c r="E59" s="7" t="inlineStr">
+        <is>
+          <t>1. Open an event that has an award proposal.
+2. Open Master QCS and click 'Bid Selection Proposal'.
+3. Open the Participants panel and read the S No. column.</t>
+        </is>
+      </c>
+      <c r="F59" s="7" t="inlineStr">
+        <is>
+          <t>The rows are numbered 1, 2, 3 …</t>
+        </is>
+      </c>
+      <c r="G59" s="7" t="inlineStr">
+        <is>
+          <t>Every row shows 'NaN'.</t>
+        </is>
+      </c>
+      <c r="H59" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO; Demo Account 2</t>
+        </is>
+      </c>
+      <c r="I59" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J59" s="7" t="inlineStr">
+        <is>
+          <t>Screen shows wrong data</t>
+        </is>
+      </c>
+      <c r="K59" s="7" t="inlineStr">
+        <is>
+          <t>Seen on 7 fresh test events (4 on Demo Account 2, 3 on PROCOL DEMO). Cause in the console code: projectProposal.jsx:1175 renders the table without a page number, which participantsTable.jsx:153-155 needs for the numbering.</t>
+        </is>
+      </c>
+      <c r="L59" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M59" s="7" t="inlineStr">
+        <is>
+          <t>UI-XCHK-PROP-005</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="7" t="inlineStr">
+        <is>
+          <t>BUG-59</t>
+        </is>
+      </c>
+      <c r="B60" s="7" t="inlineStr">
+        <is>
+          <t>Event screens</t>
+        </is>
+      </c>
+      <c r="C60" s="7" t="inlineStr">
+        <is>
+          <t>The Price Trends tab fails with a server crash on Demo Account 2</t>
+        </is>
+      </c>
+      <c r="D60" s="7" t="inlineStr">
+        <is>
+          <t>A pricing or auction stage has a Price Trends tab that shows past deals for the same products. On Demo Account 2 the request behind this tab crashes on the server for every stage, so no past prices can ever be shown there. The same tab works on PROCOL DEMO.</t>
+        </is>
+      </c>
+      <c r="E60" s="7" t="inlineStr">
+        <is>
+          <t>1. On Demo Account 2, open any pricing or auction stage.
+2. Click the Price Trends tab.</t>
+        </is>
+      </c>
+      <c r="F60" s="7" t="inlineStr">
+        <is>
+          <t>Past deals for the stage's products are listed (or 'no past deals').</t>
+        </is>
+      </c>
+      <c r="G60" s="7" t="inlineStr">
+        <is>
+          <t>The server crashes and no price history is shown.</t>
+        </is>
+      </c>
+      <c r="H60" s="7" t="inlineStr">
+        <is>
+          <t>Demo Account 2</t>
+        </is>
+      </c>
+      <c r="I60" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J60" s="7" t="inlineStr">
+        <is>
+          <t>Server crash</t>
+        </is>
+      </c>
+      <c r="K60" s="7" t="inlineStr">
+        <is>
+          <t>The price-trends request answered with a server error on 4 of 4 fresh test events on Demo Account 2; PROCOL DEMO answered normally for the same kind of stage.</t>
+        </is>
+      </c>
+      <c r="L60" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M60" s="7" t="inlineStr">
+        <is>
+          <t>UI-XCHK-TRND-001</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
@@ -4557,7 +4763,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -4821,6 +5027,70 @@
       <c r="F8" s="7" t="inlineStr">
         <is>
           <t>Confirm whether attachments must always come from Procol's own storage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Q-08</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Event screens</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Two tabs of the same stage show different savings</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>When savings are compared on the whole lot, a stage's Responses tab shows savings of ₹30 while its Overview tab shows '–' for the same stage. The Overview reads the first bidder's own savings record, which the backend leaves empty in this mode.</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Demo Account 2</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>Decide which is right: should the backend fill the bidder's savings in lot mode, or should the Overview read the stage's total savings? Seen on 2 of 2 auction test events.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Q-09</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Events list</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Searching the events list straight after opening it can show the wrong events</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Typing an event's title into the search box as soon as the events list opens sometimes leaves the newest ten events on screen instead of the one event the search returned, while the search box still shows the title. It happened in about 1 run in 3, on both clients.</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO; Demo Account 2</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>Confirm in the screen's code whether an older list response can overwrite the search result (a race between the first load and the search). It is intermittent, so it is not yet counted as a verified bug.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bug sheet: 62 verified defects — competitor prices readable by every vendor (Critical), discount above 100% becomes the best bid (High), unknown report type crash (Low)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
+++ b/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
@@ -221,8 +221,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:M60" headerRowCount="1">
-  <autoFilter ref="A1:M60"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:M63" headerRowCount="1">
+  <autoFilter ref="A1:M63"/>
   <tableColumns count="13">
     <tableColumn id="1" name="Bug #"/>
     <tableColumn id="2" name="Area"/>
@@ -560,7 +560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -590,7 +590,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>COUNTA(Bugs!A2:A60)</f>
+        <f>COUNTA(Bugs!A2:A63)</f>
         <v/>
       </c>
     </row>
@@ -609,7 +609,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF(Bugs!I2:I60,A7)</f>
+        <f>COUNTIF(Bugs!I2:I63,A7)</f>
         <v/>
       </c>
     </row>
@@ -620,7 +620,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF(Bugs!I2:I60,A8)</f>
+        <f>COUNTIF(Bugs!I2:I63,A8)</f>
         <v/>
       </c>
     </row>
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIF(Bugs!I2:I60,A9)</f>
+        <f>COUNTIF(Bugs!I2:I63,A9)</f>
         <v/>
       </c>
     </row>
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIF(Bugs!I2:I60,A10)</f>
+        <f>COUNTIF(Bugs!I2:I63,A10)</f>
         <v/>
       </c>
     </row>
@@ -661,7 +661,7 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF(Bugs!J2:J60,A13)</f>
+        <f>COUNTIF(Bugs!J2:J63,A13)</f>
         <v/>
       </c>
     </row>
@@ -672,154 +672,165 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF(Bugs!J2:J60,A14)</f>
+        <f>COUNTIF(Bugs!J2:J63,A14)</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Data validation</t>
+          <t>Data leak</t>
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF(Bugs!J2:J60,A15)</f>
+        <f>COUNTIF(Bugs!J2:J63,A15)</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Permission / business rule</t>
+          <t>Data validation</t>
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF(Bugs!J2:J60,A16)</f>
+        <f>COUNTIF(Bugs!J2:J63,A16)</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Screen shows wrong data</t>
+          <t>Permission / business rule</t>
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF(Bugs!J2:J60,A17)</f>
+        <f>COUNTIF(Bugs!J2:J63,A17)</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Server crash</t>
+          <t>Screen shows wrong data</t>
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF(Bugs!J2:J60,A18)</f>
+        <f>COUNTIF(Bugs!J2:J63,A18)</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Server crash / wrong result</t>
+          <t>Server crash</t>
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF(Bugs!J2:J60,A19)</f>
+        <f>COUNTIF(Bugs!J2:J63,A19)</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Wrong message</t>
+          <t>Server crash / wrong result</t>
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF(Bugs!J2:J60,A20)</f>
+        <f>COUNTIF(Bugs!J2:J63,A20)</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
+          <t>Wrong message</t>
+        </is>
+      </c>
+      <c r="B21" s="5">
+        <f>COUNTIF(Bugs!J2:J63,A21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
           <t>Wrong result</t>
         </is>
       </c>
-      <c r="B21" s="5">
-        <f>COUNTIF(Bugs!J2:J60,A21)</f>
+      <c r="B22" s="5">
+        <f>COUNTIF(Bugs!J2:J63,A22)</f>
         <v/>
       </c>
     </row>
-    <row r="22"/>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+    <row r="23"/>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>By client (a bug can appear on more than one)</t>
         </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>PROCOL DEMO</t>
-        </is>
-      </c>
-      <c r="B24" s="5">
-        <f>COUNTIF(Bugs!H2:H60,"*"&amp;A24&amp;"*")</f>
-        <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>Demo Account 2</t>
+          <t>PROCOL DEMO</t>
         </is>
       </c>
       <c r="B25" s="5">
-        <f>COUNTIF(Bugs!H2:H60,"*"&amp;A25&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H63,"*"&amp;A25&amp;"*")</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
+          <t>Demo Account 2</t>
+        </is>
+      </c>
+      <c r="B26" s="5">
+        <f>COUNTIF(Bugs!H2:H63,"*"&amp;A26&amp;"*")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
           <t>Procol Sandbox Demo (PO)</t>
         </is>
       </c>
-      <c r="B26" s="5">
-        <f>COUNTIF(Bugs!H2:H60,"*"&amp;A26&amp;"*")</f>
+      <c r="B27" s="5">
+        <f>COUNTIF(Bugs!H2:H63,"*"&amp;A27&amp;"*")</f>
         <v/>
       </c>
     </row>
-    <row r="27"/>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
+    <row r="28"/>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
         <is>
           <t>Also in this file</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="5" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
         <is>
           <t>Needs product confirmation</t>
         </is>
       </c>
-      <c r="B29" s="5">
+      <c r="B30" s="5">
         <f>COUNTA('Needs confirmation'!A2:A10)</f>
         <v/>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="5" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
         <is>
           <t>Client data problems (not code bugs)</t>
         </is>
       </c>
-      <c r="B30" s="5">
+      <c r="B31" s="5">
         <f>COUNTA('Data problems'!A2:A4)</f>
         <v/>
       </c>
@@ -838,7 +849,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M60"/>
+  <dimension ref="A1:M63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4746,6 +4757,214 @@
       <c r="M60" s="7" t="inlineStr">
         <is>
           <t>UI-XCHK-TRND-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="7" t="inlineStr">
+        <is>
+          <t>BUG-60</t>
+        </is>
+      </c>
+      <c r="B61" s="7" t="inlineStr">
+        <is>
+          <t>Bidding &amp; vendor permissions</t>
+        </is>
+      </c>
+      <c r="C61" s="7" t="inlineStr">
+        <is>
+          <t>Every vendor can read every competitor's prices on a sealed RFQ</t>
+        </is>
+      </c>
+      <c r="D61" s="7" t="inlineStr">
+        <is>
+          <t>In a sealed RFQ a vendor must never see what other vendors quoted. Procol stores each vendor's unit price for every line in a shared record, labelled with that vendor's company id, and sends this record to every vendor when they open the event. The screen does not show it, but it is in the data the app sends to each vendor's browser, so any vendor can read all its competitors' prices line by line — including prices the buyer entered on a vendor's behalf.</t>
+        </is>
+      </c>
+      <c r="E61" s="7" t="inlineStr">
+        <is>
+          <t>1. Create an RFQ with two or more line items and invite three or more vendors.
+2. Let the vendors bid (or enter a bid on one vendor's behalf as the buyer).
+3. Sign in as any one vendor and open the RFQ.
+4. Look at the data the app sent for each line item.</t>
+        </is>
+      </c>
+      <c r="F61" s="7" t="inlineStr">
+        <is>
+          <t>Each vendor receives only its own prices — nothing about other vendors' prices, totals or company ids.</t>
+        </is>
+      </c>
+      <c r="G61" s="7" t="inlineStr">
+        <is>
+          <t>Each vendor receives every other vendor's unit price for every line, labelled by the competitor's company id.</t>
+        </is>
+      </c>
+      <c r="H61" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO; Demo Account 2</t>
+        </is>
+      </c>
+      <c r="I61" s="8" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="J61" s="7" t="inlineStr">
+        <is>
+          <t>Data leak</t>
+        </is>
+      </c>
+      <c r="K61" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on 12 fresh test events (RFQs and rank auctions) on both clients, and re-checked independently by signing in as two different QA vendors: each saw the prices of the 3 other vendors. Cause: bid_trade_product.rb:121-131 writes every vendor's price into the line item's shared record, which is sent to every caller.</t>
+        </is>
+      </c>
+      <c r="L61" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M61" s="7" t="inlineStr">
+        <is>
+          <t>EVI-ISO-001, EVI-ISO-002, EVI-ISO-003</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="7" t="inlineStr">
+        <is>
+          <t>BUG-61</t>
+        </is>
+      </c>
+      <c r="B62" s="7" t="inlineStr">
+        <is>
+          <t>Bidding &amp; vendor permissions</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="inlineStr">
+        <is>
+          <t>A vendor can give a discount above 100%, which makes its bid total negative and the best bid</t>
+        </is>
+      </c>
+      <c r="D62" s="7" t="inlineStr">
+        <is>
+          <t>On a bid sheet where the vendor enters a discount %, Procol accepts any number — 150% included. The bid total then becomes negative (here −₹6,503), and that negative total is shown to the buyer as the event's best bid. A discount must be between 0 and 100%; that check exists only on Procol's older bid screens, not on the bid sheet.</t>
+        </is>
+      </c>
+      <c r="E62" s="7" t="inlineStr">
+        <is>
+          <t>1. Create an RFQ whose bid sheet has a vendor-entered 'Discount %' field.
+2. Invite several vendors; let some bid normally.
+3. As one vendor, quote normal prices with a discount of 150%.
+4. Open the comparison as the buyer.</t>
+        </is>
+      </c>
+      <c r="F62" s="7" t="inlineStr">
+        <is>
+          <t>A discount above 100% is refused, so no bid total can be negative or rank first.</t>
+        </is>
+      </c>
+      <c r="G62" s="7" t="inlineStr">
+        <is>
+          <t>The 150% discount is accepted, the bid total is −₹6,503.28, and it is shown as the event's best bid.</t>
+        </is>
+      </c>
+      <c r="H62" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO; Demo Account 2</t>
+        </is>
+      </c>
+      <c r="I62" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J62" s="7" t="inlineStr">
+        <is>
+          <t>Data validation</t>
+        </is>
+      </c>
+      <c r="K62" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on 4 fresh test events across both clients; the negative total matches an independent recalculation exactly. The 0–100% check runs only on the older bid paths (bids_controller.rb:555-560). Entered through the vendor's API; whether the vendor screen also blocks it was not checked.</t>
+        </is>
+      </c>
+      <c r="L62" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M62" s="7" t="inlineStr">
+        <is>
+          <t>EVI-CHG-008, EVI-CHG-007</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="7" t="inlineStr">
+        <is>
+          <t>BUG-62</t>
+        </is>
+      </c>
+      <c r="B63" s="7" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>Asking for a report with an unknown report type crashes the server</t>
+        </is>
+      </c>
+      <c r="D63" s="7" t="inlineStr">
+        <is>
+          <t>When the comparison report is requested with a report type that does not exist (for example 'excel_report'), the server crashes instead of refusing the request. The same request without the report type returns the report normally.</t>
+        </is>
+      </c>
+      <c r="E63" s="7" t="inlineStr">
+        <is>
+          <t>1. Open an RFQ that has bids.
+2. Request its comparison report with the report type set to a value that does not exist.</t>
+        </is>
+      </c>
+      <c r="F63" s="7" t="inlineStr">
+        <is>
+          <t>Refused with a clear message, or the report is returned.</t>
+        </is>
+      </c>
+      <c r="G63" s="7" t="inlineStr">
+        <is>
+          <t>The server crashes.</t>
+        </is>
+      </c>
+      <c r="H63" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I63" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J63" s="7" t="inlineStr">
+        <is>
+          <t>Server crash</t>
+        </is>
+      </c>
+      <c r="K63" s="7" t="inlineStr">
+        <is>
+          <t>Seen on 2 fresh test events on PROCOL DEMO (3 requests). Likely cause: an unknown value for the report type (report.rb:24) — read from the code, not traced in the server logs.</t>
+        </is>
+      </c>
+      <c r="L63" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M63" s="7" t="inlineStr">
+        <is>
+          <t>EVI-REP-005</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bid-number integrity checks; bug sheet 62 verified defects
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
+++ b/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
@@ -221,8 +221,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:M60" headerRowCount="1">
-  <autoFilter ref="A1:M60"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:M63" headerRowCount="1">
+  <autoFilter ref="A1:M63"/>
   <tableColumns count="13">
     <tableColumn id="1" name="Bug #"/>
     <tableColumn id="2" name="Area"/>
@@ -560,7 +560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -590,7 +590,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>COUNTA(Bugs!A2:A60)</f>
+        <f>COUNTA(Bugs!A2:A63)</f>
         <v/>
       </c>
     </row>
@@ -609,7 +609,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF(Bugs!I2:I60,A7)</f>
+        <f>COUNTIF(Bugs!I2:I63,A7)</f>
         <v/>
       </c>
     </row>
@@ -620,7 +620,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF(Bugs!I2:I60,A8)</f>
+        <f>COUNTIF(Bugs!I2:I63,A8)</f>
         <v/>
       </c>
     </row>
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIF(Bugs!I2:I60,A9)</f>
+        <f>COUNTIF(Bugs!I2:I63,A9)</f>
         <v/>
       </c>
     </row>
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIF(Bugs!I2:I60,A10)</f>
+        <f>COUNTIF(Bugs!I2:I63,A10)</f>
         <v/>
       </c>
     </row>
@@ -661,7 +661,7 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF(Bugs!J2:J60,A13)</f>
+        <f>COUNTIF(Bugs!J2:J63,A13)</f>
         <v/>
       </c>
     </row>
@@ -672,154 +672,165 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF(Bugs!J2:J60,A14)</f>
+        <f>COUNTIF(Bugs!J2:J63,A14)</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Data validation</t>
+          <t>Data leak</t>
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF(Bugs!J2:J60,A15)</f>
+        <f>COUNTIF(Bugs!J2:J63,A15)</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Permission / business rule</t>
+          <t>Data validation</t>
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF(Bugs!J2:J60,A16)</f>
+        <f>COUNTIF(Bugs!J2:J63,A16)</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Screen shows wrong data</t>
+          <t>Permission / business rule</t>
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF(Bugs!J2:J60,A17)</f>
+        <f>COUNTIF(Bugs!J2:J63,A17)</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Server crash</t>
+          <t>Screen shows wrong data</t>
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF(Bugs!J2:J60,A18)</f>
+        <f>COUNTIF(Bugs!J2:J63,A18)</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Server crash / wrong result</t>
+          <t>Server crash</t>
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF(Bugs!J2:J60,A19)</f>
+        <f>COUNTIF(Bugs!J2:J63,A19)</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Wrong message</t>
+          <t>Server crash / wrong result</t>
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF(Bugs!J2:J60,A20)</f>
+        <f>COUNTIF(Bugs!J2:J63,A20)</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
+          <t>Wrong message</t>
+        </is>
+      </c>
+      <c r="B21" s="5">
+        <f>COUNTIF(Bugs!J2:J63,A21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
           <t>Wrong result</t>
         </is>
       </c>
-      <c r="B21" s="5">
-        <f>COUNTIF(Bugs!J2:J60,A21)</f>
+      <c r="B22" s="5">
+        <f>COUNTIF(Bugs!J2:J63,A22)</f>
         <v/>
       </c>
     </row>
-    <row r="22"/>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+    <row r="23"/>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>By client (a bug can appear on more than one)</t>
         </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>PROCOL DEMO</t>
-        </is>
-      </c>
-      <c r="B24" s="5">
-        <f>COUNTIF(Bugs!H2:H60,"*"&amp;A24&amp;"*")</f>
-        <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>Demo Account 2</t>
+          <t>PROCOL DEMO</t>
         </is>
       </c>
       <c r="B25" s="5">
-        <f>COUNTIF(Bugs!H2:H60,"*"&amp;A25&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H63,"*"&amp;A25&amp;"*")</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
+          <t>Demo Account 2</t>
+        </is>
+      </c>
+      <c r="B26" s="5">
+        <f>COUNTIF(Bugs!H2:H63,"*"&amp;A26&amp;"*")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
           <t>Procol Sandbox Demo (PO)</t>
         </is>
       </c>
-      <c r="B26" s="5">
-        <f>COUNTIF(Bugs!H2:H60,"*"&amp;A26&amp;"*")</f>
+      <c r="B27" s="5">
+        <f>COUNTIF(Bugs!H2:H63,"*"&amp;A27&amp;"*")</f>
         <v/>
       </c>
     </row>
-    <row r="27"/>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
+    <row r="28"/>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
         <is>
           <t>Also in this file</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="5" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
         <is>
           <t>Needs product confirmation</t>
         </is>
       </c>
-      <c r="B29" s="5">
+      <c r="B30" s="5">
         <f>COUNTA('Needs confirmation'!A2:A10)</f>
         <v/>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="5" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
         <is>
           <t>Client data problems (not code bugs)</t>
         </is>
       </c>
-      <c r="B30" s="5">
+      <c r="B31" s="5">
         <f>COUNTA('Data problems'!A2:A4)</f>
         <v/>
       </c>
@@ -838,7 +849,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M60"/>
+  <dimension ref="A1:M63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4746,6 +4757,214 @@
       <c r="M60" s="7" t="inlineStr">
         <is>
           <t>UI-XCHK-TRND-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="7" t="inlineStr">
+        <is>
+          <t>BUG-60</t>
+        </is>
+      </c>
+      <c r="B61" s="7" t="inlineStr">
+        <is>
+          <t>Bidding &amp; vendor permissions</t>
+        </is>
+      </c>
+      <c r="C61" s="7" t="inlineStr">
+        <is>
+          <t>Every vendor can read every competitor's prices on a sealed RFQ</t>
+        </is>
+      </c>
+      <c r="D61" s="7" t="inlineStr">
+        <is>
+          <t>In a sealed RFQ a vendor must never see what other vendors quoted. Procol stores each vendor's unit price for every line in a shared record, labelled with that vendor's company id, and sends this record to every vendor when they open the event. The screen does not show it, but it is in the data the app sends to each vendor's browser, so any vendor can read all its competitors' prices line by line — including prices the buyer entered on a vendor's behalf.</t>
+        </is>
+      </c>
+      <c r="E61" s="7" t="inlineStr">
+        <is>
+          <t>1. Create an RFQ with two or more line items and invite three or more vendors.
+2. Let the vendors bid (or enter a bid on one vendor's behalf as the buyer).
+3. Sign in as any one vendor and open the RFQ.
+4. Look at the data the app sent for each line item.</t>
+        </is>
+      </c>
+      <c r="F61" s="7" t="inlineStr">
+        <is>
+          <t>Each vendor receives only its own prices — nothing about other vendors' prices, totals or company ids.</t>
+        </is>
+      </c>
+      <c r="G61" s="7" t="inlineStr">
+        <is>
+          <t>Each vendor receives every other vendor's unit price for every line, labelled by the competitor's company id.</t>
+        </is>
+      </c>
+      <c r="H61" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO; Demo Account 2</t>
+        </is>
+      </c>
+      <c r="I61" s="8" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="J61" s="7" t="inlineStr">
+        <is>
+          <t>Data leak</t>
+        </is>
+      </c>
+      <c r="K61" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on 12 fresh test events (RFQs and rank auctions) on both clients, and re-checked independently by signing in as two different QA vendors: each saw the prices of the 3 other vendors. Cause: bid_trade_product.rb:121-131 writes every vendor's price into the line item's shared record, which is sent to every caller.</t>
+        </is>
+      </c>
+      <c r="L61" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M61" s="7" t="inlineStr">
+        <is>
+          <t>EVI-ISO-001, EVI-ISO-002, EVI-ISO-003</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="7" t="inlineStr">
+        <is>
+          <t>BUG-61</t>
+        </is>
+      </c>
+      <c r="B62" s="7" t="inlineStr">
+        <is>
+          <t>Bidding &amp; vendor permissions</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="inlineStr">
+        <is>
+          <t>A vendor can give a discount above 100%, which makes its bid total negative and the best bid</t>
+        </is>
+      </c>
+      <c r="D62" s="7" t="inlineStr">
+        <is>
+          <t>On a bid sheet where the vendor enters a discount %, Procol accepts any number — 150% included. The bid total then becomes negative (here −₹6,503), and that negative total is shown to the buyer as the event's best bid. A discount must be between 0 and 100%; that check exists only on Procol's older bid screens, not on the bid sheet.</t>
+        </is>
+      </c>
+      <c r="E62" s="7" t="inlineStr">
+        <is>
+          <t>1. Create an RFQ whose bid sheet has a vendor-entered 'Discount %' field.
+2. Invite several vendors; let some bid normally.
+3. As one vendor, quote normal prices with a discount of 150%.
+4. Open the comparison as the buyer.</t>
+        </is>
+      </c>
+      <c r="F62" s="7" t="inlineStr">
+        <is>
+          <t>A discount above 100% is refused, so no bid total can be negative or rank first.</t>
+        </is>
+      </c>
+      <c r="G62" s="7" t="inlineStr">
+        <is>
+          <t>The 150% discount is accepted, the bid total is −₹6,503.28, and it is shown as the event's best bid.</t>
+        </is>
+      </c>
+      <c r="H62" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO; Demo Account 2</t>
+        </is>
+      </c>
+      <c r="I62" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J62" s="7" t="inlineStr">
+        <is>
+          <t>Data validation</t>
+        </is>
+      </c>
+      <c r="K62" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on 4 fresh test events across both clients; the negative total matches an independent recalculation exactly. The 0–100% check runs only on the older bid paths (bids_controller.rb:555-560). Entered through the vendor's API; whether the vendor screen also blocks it was not checked.</t>
+        </is>
+      </c>
+      <c r="L62" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M62" s="7" t="inlineStr">
+        <is>
+          <t>EVI-CHG-008, EVI-CHG-007</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="7" t="inlineStr">
+        <is>
+          <t>BUG-62</t>
+        </is>
+      </c>
+      <c r="B63" s="7" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>Asking for a report with an unknown report type crashes the server</t>
+        </is>
+      </c>
+      <c r="D63" s="7" t="inlineStr">
+        <is>
+          <t>When the comparison report is requested with a report type that does not exist (for example 'excel_report'), the server crashes instead of refusing the request. The same request without the report type returns the report normally.</t>
+        </is>
+      </c>
+      <c r="E63" s="7" t="inlineStr">
+        <is>
+          <t>1. Open an RFQ that has bids.
+2. Request its comparison report with the report type set to a value that does not exist.</t>
+        </is>
+      </c>
+      <c r="F63" s="7" t="inlineStr">
+        <is>
+          <t>Refused with a clear message, or the report is returned.</t>
+        </is>
+      </c>
+      <c r="G63" s="7" t="inlineStr">
+        <is>
+          <t>The server crashes.</t>
+        </is>
+      </c>
+      <c r="H63" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I63" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J63" s="7" t="inlineStr">
+        <is>
+          <t>Server crash</t>
+        </is>
+      </c>
+      <c r="K63" s="7" t="inlineStr">
+        <is>
+          <t>Seen on 2 fresh test events on PROCOL DEMO (3 requests). Likely cause: an unknown value for the report type (report.rb:24) — read from the code, not traced in the server logs.</t>
+        </is>
+      </c>
+      <c r="L63" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M63" s="7" t="inlineStr">
+        <is>
+          <t>EVI-REP-005</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deep-dig round 3: award outcomes, award->PO and live multi-vendor competition (66 cases); bug sheet 68
- run-deep3.ts: scenarios with 3-4 QA vendors per event, exact award/PO/rank numbers computed from
  what the run submitted; every failure re-run on a second fresh event. 198678: 31 passed / 13 failed;
  32461: 25 / 8 (7 not run: approver differs from the buyer).
- 6 new verified defects: competitors named with bid status to every vendor (High), split award
  orders each vendor's full quantity (High), removing a vendor from a split award breaks the total
  (High), tied L1 counted as non-L1, awarded quantity cannot be lowered, extension leaves bids'
  old end time. BUG-60 widened (schema read, non-bidders, after award, rank-only auctions).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
+++ b/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
@@ -221,8 +221,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:M63" headerRowCount="1">
-  <autoFilter ref="A1:M63"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:M69" headerRowCount="1">
+  <autoFilter ref="A1:M69"/>
   <tableColumns count="13">
     <tableColumn id="1" name="Bug #"/>
     <tableColumn id="2" name="Area"/>
@@ -590,7 +590,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>COUNTA(Bugs!A2:A63)</f>
+        <f>COUNTA(Bugs!A2:A69)</f>
         <v/>
       </c>
     </row>
@@ -609,7 +609,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF(Bugs!I2:I63,A7)</f>
+        <f>COUNTIF(Bugs!I2:I69,A7)</f>
         <v/>
       </c>
     </row>
@@ -620,7 +620,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF(Bugs!I2:I63,A8)</f>
+        <f>COUNTIF(Bugs!I2:I69,A8)</f>
         <v/>
       </c>
     </row>
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIF(Bugs!I2:I63,A9)</f>
+        <f>COUNTIF(Bugs!I2:I69,A9)</f>
         <v/>
       </c>
     </row>
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIF(Bugs!I2:I63,A10)</f>
+        <f>COUNTIF(Bugs!I2:I69,A10)</f>
         <v/>
       </c>
     </row>
@@ -661,7 +661,7 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF(Bugs!J2:J63,A13)</f>
+        <f>COUNTIF(Bugs!J2:J69,A13)</f>
         <v/>
       </c>
     </row>
@@ -672,7 +672,7 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF(Bugs!J2:J63,A14)</f>
+        <f>COUNTIF(Bugs!J2:J69,A14)</f>
         <v/>
       </c>
     </row>
@@ -683,7 +683,7 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF(Bugs!J2:J63,A15)</f>
+        <f>COUNTIF(Bugs!J2:J69,A15)</f>
         <v/>
       </c>
     </row>
@@ -694,7 +694,7 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF(Bugs!J2:J63,A16)</f>
+        <f>COUNTIF(Bugs!J2:J69,A16)</f>
         <v/>
       </c>
     </row>
@@ -705,7 +705,7 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF(Bugs!J2:J63,A17)</f>
+        <f>COUNTIF(Bugs!J2:J69,A17)</f>
         <v/>
       </c>
     </row>
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF(Bugs!J2:J63,A18)</f>
+        <f>COUNTIF(Bugs!J2:J69,A18)</f>
         <v/>
       </c>
     </row>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF(Bugs!J2:J63,A19)</f>
+        <f>COUNTIF(Bugs!J2:J69,A19)</f>
         <v/>
       </c>
     </row>
@@ -738,7 +738,7 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF(Bugs!J2:J63,A20)</f>
+        <f>COUNTIF(Bugs!J2:J69,A20)</f>
         <v/>
       </c>
     </row>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF(Bugs!J2:J63,A21)</f>
+        <f>COUNTIF(Bugs!J2:J69,A21)</f>
         <v/>
       </c>
     </row>
@@ -760,7 +760,7 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF(Bugs!J2:J63,A22)</f>
+        <f>COUNTIF(Bugs!J2:J69,A22)</f>
         <v/>
       </c>
     </row>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B25" s="5">
-        <f>COUNTIF(Bugs!H2:H63,"*"&amp;A25&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H69,"*"&amp;A25&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF(Bugs!H2:H63,"*"&amp;A26&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H69,"*"&amp;A26&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -801,7 +801,7 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF(Bugs!H2:H63,"*"&amp;A27&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H69,"*"&amp;A27&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -849,7 +849,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M63"/>
+  <dimension ref="A1:M69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4778,7 +4778,7 @@
       </c>
       <c r="D61" s="7" t="inlineStr">
         <is>
-          <t>In a sealed RFQ a vendor must never see what other vendors quoted. Procol stores each vendor's unit price for every line in a shared record, labelled with that vendor's company id, and sends this record to every vendor when they open the event. The screen does not show it, but it is in the data the app sends to each vendor's browser, so any vendor can read all its competitors' prices line by line — including prices the buyer entered on a vendor's behalf.</t>
+          <t>In a sealed RFQ a vendor must never see what other vendors quoted. Procol stores each vendor's unit price for every line in a shared record, labelled with that vendor's company id, and sends this record to every vendor when they open the event. The screen does not show it, but it is in the data the app sends to each vendor's browser, so any vendor can read all its competitors' prices line by line — including prices the buyer entered on a vendor's behalf. The same prices are also in the round's page data, reach vendors that never bid, stay visible after the award, and defeat a rank-only auction (where vendors should see only their rank).</t>
         </is>
       </c>
       <c r="E61" s="7" t="inlineStr">
@@ -4826,7 +4826,7 @@
       </c>
       <c r="M61" s="7" t="inlineStr">
         <is>
-          <t>EVI-ISO-001, EVI-ISO-002, EVI-ISO-003</t>
+          <t>EVI-ISO-001, EVI-ISO-002, EVI-ISO-003, API-EVDLEK-002</t>
         </is>
       </c>
     </row>
@@ -4965,6 +4965,418 @@
       <c r="M63" s="7" t="inlineStr">
         <is>
           <t>EVI-REP-005</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="7" t="inlineStr">
+        <is>
+          <t>BUG-63</t>
+        </is>
+      </c>
+      <c r="B64" s="7" t="inlineStr">
+        <is>
+          <t>Bidding &amp; vendor permissions</t>
+        </is>
+      </c>
+      <c r="C64" s="7" t="inlineStr">
+        <is>
+          <t>Every invited vendor can see who else bid, their bid status and who won</t>
+        </is>
+      </c>
+      <c r="D64" s="7" t="inlineStr">
+        <is>
+          <t>In a sealed event a vendor must not learn who its competitors are. The data Procol sends each invited vendor for a round lists every bidder: the competitor's company name, its company id, its bid id, its bid status (for example 'selected' — i.e. who won) and how many times it revised its bid. Even a vendor that never bid receives it, and it stays visible after the award. Together with the price leak (the row 'Every vendor can read every competitor's prices on a sealed RFQ') a vendor can put a name to every competitor's price.</t>
+        </is>
+      </c>
+      <c r="E64" s="7" t="inlineStr">
+        <is>
+          <t>1. Publish an RFQ or auction and invite several vendors; let some of them bid.
+2. Sign in as any invited vendor (even one that has not bid) and open the round.
+3. Look at the data the app sent for the round's page.</t>
+        </is>
+      </c>
+      <c r="F64" s="7" t="inlineStr">
+        <is>
+          <t>A vendor receives only its own bid's details; competitors are never named or described.</t>
+        </is>
+      </c>
+      <c r="G64" s="7" t="inlineStr">
+        <is>
+          <t>Every other bidder is listed by company name with its bid id, bid status (including who was selected) and revision count.</t>
+        </is>
+      </c>
+      <c r="H64" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO; Demo Account 2</t>
+        </is>
+      </c>
+      <c r="I64" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J64" s="7" t="inlineStr">
+        <is>
+          <t>Data leak</t>
+        </is>
+      </c>
+      <c r="K64" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on 10 fresh test events on both clients (RFQs and auctions), and re-checked independently by signing in as a QA vendor who never bid: it saw the three other vendors by name, with bid ids and 'selected' status. Served by api/v1/trade_controller.rb:371 via trade_template_helper.rb:5856-5900.</t>
+        </is>
+      </c>
+      <c r="L64" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M64" s="7" t="inlineStr">
+        <is>
+          <t>API-EVDLEK-001, API-EVDLEK-003, API-EVDLEK-004, API-EVDLEK-005, API-EVDLEK-006, API-EVDLEK-007</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="7" t="inlineStr">
+        <is>
+          <t>BUG-64</t>
+        </is>
+      </c>
+      <c r="B65" s="7" t="inlineStr">
+        <is>
+          <t>Awarding</t>
+        </is>
+      </c>
+      <c r="C65" s="7" t="inlineStr">
+        <is>
+          <t>Splitting a line's award between vendors creates purchase orders for each vendor's full quantity</t>
+        </is>
+      </c>
+      <c r="D65" s="7" t="inlineStr">
+        <is>
+          <t>When a 30 KG line is awarded across three vendors (15, 10 and 5 KG), Procol creates three purchase orders of 30 KG each — 90 KG ordered for a 30 KG need. The prices on the orders are right; the quantities are each vendor's whole quote instead of the part awarded to it. This happens when the comparison template does not mark the awarded quantity as a field the buyer edits, although the company has partial awarding switched on.</t>
+        </is>
+      </c>
+      <c r="E65" s="7" t="inlineStr">
+        <is>
+          <t>1. Create an RFQ for one line of 30 KG and invite three vendors; let each quote for 30 KG.
+2. Award the line split 15 / 10 / 5 KG across the three vendors and get it approved.
+3. Create the purchase orders from the award and read their quantities.</t>
+        </is>
+      </c>
+      <c r="F65" s="7" t="inlineStr">
+        <is>
+          <t>The orders carry 15, 10 and 5 KG — 30 KG in total, as awarded.</t>
+        </is>
+      </c>
+      <c r="G65" s="7" t="inlineStr">
+        <is>
+          <t>Each order carries 30 KG — 90 KG in total.</t>
+        </is>
+      </c>
+      <c r="H65" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I65" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J65" s="7" t="inlineStr">
+        <is>
+          <t>Wrong result</t>
+        </is>
+      </c>
+      <c r="K65" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on 4 fresh test events on PROCOL DEMO. The order quantity comes from the vendor's quoted quantity when awarded quantity is not a buyer-editable field (proposal_helper.rb:1177-1190, bid_concern.rb:7-9, order.rb:300-306).</t>
+        </is>
+      </c>
+      <c r="L65" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M65" s="7" t="inlineStr">
+        <is>
+          <t>API-EVDAPO-002, API-EVDAPO-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="7" t="inlineStr">
+        <is>
+          <t>BUG-65</t>
+        </is>
+      </c>
+      <c r="B66" s="7" t="inlineStr">
+        <is>
+          <t>Awarding</t>
+        </is>
+      </c>
+      <c r="C66" s="7" t="inlineStr">
+        <is>
+          <t>Taking a vendor off a split award subtracts its whole quote, so the award total is wrong</t>
+        </is>
+      </c>
+      <c r="D66" s="7" t="inlineStr">
+        <is>
+          <t>When a buyer removes one vendor from a line that is split between several vendors (the way the award screen does it), Procol subtracts that vendor's whole quote from the award total instead of only the part awarded to it. In the test the total went to −₹1,550, and to ₹22,705 after the vendor was added back, instead of ₹1,43,980. The award was then approved with that wrong total — and the total decides which approval flow applies.</t>
+        </is>
+      </c>
+      <c r="E66" s="7" t="inlineStr">
+        <is>
+          <t>1. Award one line split across three vendors.
+2. Remove one of the vendors from the award, then add it back.
+3. Read the award total.</t>
+        </is>
+      </c>
+      <c r="F66" s="7" t="inlineStr">
+        <is>
+          <t>The total changes by the removed vendor's awarded amount only, and returns to ₹1,43,980 when it is added back.</t>
+        </is>
+      </c>
+      <c r="G66" s="7" t="inlineStr">
+        <is>
+          <t>The total becomes −₹1,550, then ₹22,705, and the award can be approved with it.</t>
+        </is>
+      </c>
+      <c r="H66" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I66" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J66" s="7" t="inlineStr">
+        <is>
+          <t>Wrong result</t>
+        </is>
+      </c>
+      <c r="K66" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on 2 fresh test events on PROCOL DEMO. The award value removed is the vendor's whole bid total (proposal_helper.rb, get_po_value_to_be_added falls back to the bid's gross total).</t>
+        </is>
+      </c>
+      <c r="L66" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M66" s="7" t="inlineStr">
+        <is>
+          <t>API-EVDAWD-003, API-EVDAWD-005</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="7" t="inlineStr">
+        <is>
+          <t>BUG-66</t>
+        </is>
+      </c>
+      <c r="B67" s="7" t="inlineStr">
+        <is>
+          <t>Awarding</t>
+        </is>
+      </c>
+      <c r="C67" s="7" t="inlineStr">
+        <is>
+          <t>Vendors tied at the lowest price are counted as 'not L1' in the award</t>
+        </is>
+      </c>
+      <c r="D67" s="7" t="inlineStr">
+        <is>
+          <t>When two vendors quote the same lowest price, the award summary counts neither of them as L1: the L1 value shows ₹0 and the tied vendors' amounts are counted under 'non-L1'.</t>
+        </is>
+      </c>
+      <c r="E67" s="7" t="inlineStr">
+        <is>
+          <t>1. Create an RFQ and let two vendors quote the same lowest price.
+2. Award the line to one of them and read the award's L1 / non-L1 values.</t>
+        </is>
+      </c>
+      <c r="F67" s="7" t="inlineStr">
+        <is>
+          <t>The tied vendors are L1, so the L1 value is the awarded amount.</t>
+        </is>
+      </c>
+      <c r="G67" s="7" t="inlineStr">
+        <is>
+          <t>L1 shows ₹0 and the award is counted as non-L1.</t>
+        </is>
+      </c>
+      <c r="H67" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO; Demo Account 2</t>
+        </is>
+      </c>
+      <c r="I67" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J67" s="7" t="inlineStr">
+        <is>
+          <t>Wrong result</t>
+        </is>
+      </c>
+      <c r="K67" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on 6 fresh test events across both clients (proposal_helper.rb:994-1001, bid_rank_helper.rb:215-218).</t>
+        </is>
+      </c>
+      <c r="L67" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M67" s="7" t="inlineStr">
+        <is>
+          <t>API-EVDAWD-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="7" t="inlineStr">
+        <is>
+          <t>BUG-67</t>
+        </is>
+      </c>
+      <c r="B68" s="7" t="inlineStr">
+        <is>
+          <t>Awarding</t>
+        </is>
+      </c>
+      <c r="C68" s="7" t="inlineStr">
+        <is>
+          <t>A vendor's awarded quantity cannot be lowered once a line is fully awarded</t>
+        </is>
+      </c>
+      <c r="D68" s="7" t="inlineStr">
+        <is>
+          <t>When a line is fully awarded across vendors and the buyer lowers one vendor's quantity, Procol refuses with 'You cannot select bid with more than requested quantity', because it counts that vendor's current award as well as the new, lower quantity. The only way round it is to remove the vendor and add it again, which triggers the wrong-total problem in the row above.</t>
+        </is>
+      </c>
+      <c r="E68" s="7" t="inlineStr">
+        <is>
+          <t>1. Award a 30 KG line as 15 / 10 / 5 KG.
+2. Change the 5 KG vendor's quantity to 3 KG.</t>
+        </is>
+      </c>
+      <c r="F68" s="7" t="inlineStr">
+        <is>
+          <t>The change is accepted (3 KG is within the requested 30 KG).</t>
+        </is>
+      </c>
+      <c r="G68" s="7" t="inlineStr">
+        <is>
+          <t>Refused: 'You cannot select bid with more than requested quantity'.</t>
+        </is>
+      </c>
+      <c r="H68" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I68" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J68" s="7" t="inlineStr">
+        <is>
+          <t>Business rule</t>
+        </is>
+      </c>
+      <c r="K68" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on 4 fresh test events on PROCOL DEMO (proposal_helper.rb:1295-1305).</t>
+        </is>
+      </c>
+      <c r="L68" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M68" s="7" t="inlineStr">
+        <is>
+          <t>API-EVDAWD-006</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="7" t="inlineStr">
+        <is>
+          <t>BUG-68</t>
+        </is>
+      </c>
+      <c r="B69" s="7" t="inlineStr">
+        <is>
+          <t>Auctions</t>
+        </is>
+      </c>
+      <c r="C69" s="7" t="inlineStr">
+        <is>
+          <t>After an auction's automatic extension, existing bids still show the old end time</t>
+        </is>
+      </c>
+      <c r="D69" s="7" t="inlineStr">
+        <is>
+          <t>When a late bid makes an auction extend automatically, the auction's end time moves, but the bids already placed keep the old end time as their 'valid till' time.</t>
+        </is>
+      </c>
+      <c r="E69" s="7" t="inlineStr">
+        <is>
+          <t>1. Run an auction with automatic extension and several vendors bidding.
+2. Place a winning bid in the last minutes so the auction extends.
+3. Read the earlier bids' end ('valid till') time.</t>
+        </is>
+      </c>
+      <c r="F69" s="7" t="inlineStr">
+        <is>
+          <t>Every bid shows the auction's new end time.</t>
+        </is>
+      </c>
+      <c r="G69" s="7" t="inlineStr">
+        <is>
+          <t>The earlier bids keep the old end time.</t>
+        </is>
+      </c>
+      <c r="H69" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO; Demo Account 2</t>
+        </is>
+      </c>
+      <c r="I69" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J69" s="7" t="inlineStr">
+        <is>
+          <t>Wrong result</t>
+        </is>
+      </c>
+      <c r="K69" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on 4 fresh test events across both clients (bid.rb:2264-2286 keeps the cached schedule).</t>
+        </is>
+      </c>
+      <c r="L69" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M69" s="7" t="inlineStr">
+        <is>
+          <t>API-EVDAUX-004</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deep-dig round 3 (award, PO, competition); bug sheet 68
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
+++ b/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
@@ -221,8 +221,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:M63" headerRowCount="1">
-  <autoFilter ref="A1:M63"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:M69" headerRowCount="1">
+  <autoFilter ref="A1:M69"/>
   <tableColumns count="13">
     <tableColumn id="1" name="Bug #"/>
     <tableColumn id="2" name="Area"/>
@@ -590,7 +590,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>COUNTA(Bugs!A2:A63)</f>
+        <f>COUNTA(Bugs!A2:A69)</f>
         <v/>
       </c>
     </row>
@@ -609,7 +609,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF(Bugs!I2:I63,A7)</f>
+        <f>COUNTIF(Bugs!I2:I69,A7)</f>
         <v/>
       </c>
     </row>
@@ -620,7 +620,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF(Bugs!I2:I63,A8)</f>
+        <f>COUNTIF(Bugs!I2:I69,A8)</f>
         <v/>
       </c>
     </row>
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIF(Bugs!I2:I63,A9)</f>
+        <f>COUNTIF(Bugs!I2:I69,A9)</f>
         <v/>
       </c>
     </row>
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIF(Bugs!I2:I63,A10)</f>
+        <f>COUNTIF(Bugs!I2:I69,A10)</f>
         <v/>
       </c>
     </row>
@@ -661,7 +661,7 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF(Bugs!J2:J63,A13)</f>
+        <f>COUNTIF(Bugs!J2:J69,A13)</f>
         <v/>
       </c>
     </row>
@@ -672,7 +672,7 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF(Bugs!J2:J63,A14)</f>
+        <f>COUNTIF(Bugs!J2:J69,A14)</f>
         <v/>
       </c>
     </row>
@@ -683,7 +683,7 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF(Bugs!J2:J63,A15)</f>
+        <f>COUNTIF(Bugs!J2:J69,A15)</f>
         <v/>
       </c>
     </row>
@@ -694,7 +694,7 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF(Bugs!J2:J63,A16)</f>
+        <f>COUNTIF(Bugs!J2:J69,A16)</f>
         <v/>
       </c>
     </row>
@@ -705,7 +705,7 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF(Bugs!J2:J63,A17)</f>
+        <f>COUNTIF(Bugs!J2:J69,A17)</f>
         <v/>
       </c>
     </row>
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF(Bugs!J2:J63,A18)</f>
+        <f>COUNTIF(Bugs!J2:J69,A18)</f>
         <v/>
       </c>
     </row>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF(Bugs!J2:J63,A19)</f>
+        <f>COUNTIF(Bugs!J2:J69,A19)</f>
         <v/>
       </c>
     </row>
@@ -738,7 +738,7 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF(Bugs!J2:J63,A20)</f>
+        <f>COUNTIF(Bugs!J2:J69,A20)</f>
         <v/>
       </c>
     </row>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF(Bugs!J2:J63,A21)</f>
+        <f>COUNTIF(Bugs!J2:J69,A21)</f>
         <v/>
       </c>
     </row>
@@ -760,7 +760,7 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF(Bugs!J2:J63,A22)</f>
+        <f>COUNTIF(Bugs!J2:J69,A22)</f>
         <v/>
       </c>
     </row>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B25" s="5">
-        <f>COUNTIF(Bugs!H2:H63,"*"&amp;A25&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H69,"*"&amp;A25&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF(Bugs!H2:H63,"*"&amp;A26&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H69,"*"&amp;A26&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -801,7 +801,7 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF(Bugs!H2:H63,"*"&amp;A27&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H69,"*"&amp;A27&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -849,7 +849,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M63"/>
+  <dimension ref="A1:M69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4778,7 +4778,7 @@
       </c>
       <c r="D61" s="7" t="inlineStr">
         <is>
-          <t>In a sealed RFQ a vendor must never see what other vendors quoted. Procol stores each vendor's unit price for every line in a shared record, labelled with that vendor's company id, and sends this record to every vendor when they open the event. The screen does not show it, but it is in the data the app sends to each vendor's browser, so any vendor can read all its competitors' prices line by line — including prices the buyer entered on a vendor's behalf.</t>
+          <t>In a sealed RFQ a vendor must never see what other vendors quoted. Procol stores each vendor's unit price for every line in a shared record, labelled with that vendor's company id, and sends this record to every vendor when they open the event. The screen does not show it, but it is in the data the app sends to each vendor's browser, so any vendor can read all its competitors' prices line by line — including prices the buyer entered on a vendor's behalf. The same prices are also in the round's page data, reach vendors that never bid, stay visible after the award, and defeat a rank-only auction (where vendors should see only their rank).</t>
         </is>
       </c>
       <c r="E61" s="7" t="inlineStr">
@@ -4826,7 +4826,7 @@
       </c>
       <c r="M61" s="7" t="inlineStr">
         <is>
-          <t>EVI-ISO-001, EVI-ISO-002, EVI-ISO-003</t>
+          <t>EVI-ISO-001, EVI-ISO-002, EVI-ISO-003, API-EVDLEK-002</t>
         </is>
       </c>
     </row>
@@ -4965,6 +4965,418 @@
       <c r="M63" s="7" t="inlineStr">
         <is>
           <t>EVI-REP-005</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="7" t="inlineStr">
+        <is>
+          <t>BUG-63</t>
+        </is>
+      </c>
+      <c r="B64" s="7" t="inlineStr">
+        <is>
+          <t>Bidding &amp; vendor permissions</t>
+        </is>
+      </c>
+      <c r="C64" s="7" t="inlineStr">
+        <is>
+          <t>Every invited vendor can see who else bid, their bid status and who won</t>
+        </is>
+      </c>
+      <c r="D64" s="7" t="inlineStr">
+        <is>
+          <t>In a sealed event a vendor must not learn who its competitors are. The data Procol sends each invited vendor for a round lists every bidder: the competitor's company name, its company id, its bid id, its bid status (for example 'selected' — i.e. who won) and how many times it revised its bid. Even a vendor that never bid receives it, and it stays visible after the award. Together with the price leak (the row 'Every vendor can read every competitor's prices on a sealed RFQ') a vendor can put a name to every competitor's price.</t>
+        </is>
+      </c>
+      <c r="E64" s="7" t="inlineStr">
+        <is>
+          <t>1. Publish an RFQ or auction and invite several vendors; let some of them bid.
+2. Sign in as any invited vendor (even one that has not bid) and open the round.
+3. Look at the data the app sent for the round's page.</t>
+        </is>
+      </c>
+      <c r="F64" s="7" t="inlineStr">
+        <is>
+          <t>A vendor receives only its own bid's details; competitors are never named or described.</t>
+        </is>
+      </c>
+      <c r="G64" s="7" t="inlineStr">
+        <is>
+          <t>Every other bidder is listed by company name with its bid id, bid status (including who was selected) and revision count.</t>
+        </is>
+      </c>
+      <c r="H64" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO; Demo Account 2</t>
+        </is>
+      </c>
+      <c r="I64" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J64" s="7" t="inlineStr">
+        <is>
+          <t>Data leak</t>
+        </is>
+      </c>
+      <c r="K64" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on 10 fresh test events on both clients (RFQs and auctions), and re-checked independently by signing in as a QA vendor who never bid: it saw the three other vendors by name, with bid ids and 'selected' status. Served by api/v1/trade_controller.rb:371 via trade_template_helper.rb:5856-5900.</t>
+        </is>
+      </c>
+      <c r="L64" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M64" s="7" t="inlineStr">
+        <is>
+          <t>API-EVDLEK-001, API-EVDLEK-003, API-EVDLEK-004, API-EVDLEK-005, API-EVDLEK-006, API-EVDLEK-007</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="7" t="inlineStr">
+        <is>
+          <t>BUG-64</t>
+        </is>
+      </c>
+      <c r="B65" s="7" t="inlineStr">
+        <is>
+          <t>Awarding</t>
+        </is>
+      </c>
+      <c r="C65" s="7" t="inlineStr">
+        <is>
+          <t>Splitting a line's award between vendors creates purchase orders for each vendor's full quantity</t>
+        </is>
+      </c>
+      <c r="D65" s="7" t="inlineStr">
+        <is>
+          <t>When a 30 KG line is awarded across three vendors (15, 10 and 5 KG), Procol creates three purchase orders of 30 KG each — 90 KG ordered for a 30 KG need. The prices on the orders are right; the quantities are each vendor's whole quote instead of the part awarded to it. This happens when the comparison template does not mark the awarded quantity as a field the buyer edits, although the company has partial awarding switched on.</t>
+        </is>
+      </c>
+      <c r="E65" s="7" t="inlineStr">
+        <is>
+          <t>1. Create an RFQ for one line of 30 KG and invite three vendors; let each quote for 30 KG.
+2. Award the line split 15 / 10 / 5 KG across the three vendors and get it approved.
+3. Create the purchase orders from the award and read their quantities.</t>
+        </is>
+      </c>
+      <c r="F65" s="7" t="inlineStr">
+        <is>
+          <t>The orders carry 15, 10 and 5 KG — 30 KG in total, as awarded.</t>
+        </is>
+      </c>
+      <c r="G65" s="7" t="inlineStr">
+        <is>
+          <t>Each order carries 30 KG — 90 KG in total.</t>
+        </is>
+      </c>
+      <c r="H65" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I65" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J65" s="7" t="inlineStr">
+        <is>
+          <t>Wrong result</t>
+        </is>
+      </c>
+      <c r="K65" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on 4 fresh test events on PROCOL DEMO. The order quantity comes from the vendor's quoted quantity when awarded quantity is not a buyer-editable field (proposal_helper.rb:1177-1190, bid_concern.rb:7-9, order.rb:300-306).</t>
+        </is>
+      </c>
+      <c r="L65" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M65" s="7" t="inlineStr">
+        <is>
+          <t>API-EVDAPO-002, API-EVDAPO-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="7" t="inlineStr">
+        <is>
+          <t>BUG-65</t>
+        </is>
+      </c>
+      <c r="B66" s="7" t="inlineStr">
+        <is>
+          <t>Awarding</t>
+        </is>
+      </c>
+      <c r="C66" s="7" t="inlineStr">
+        <is>
+          <t>Taking a vendor off a split award subtracts its whole quote, so the award total is wrong</t>
+        </is>
+      </c>
+      <c r="D66" s="7" t="inlineStr">
+        <is>
+          <t>When a buyer removes one vendor from a line that is split between several vendors (the way the award screen does it), Procol subtracts that vendor's whole quote from the award total instead of only the part awarded to it. In the test the total went to −₹1,550, and to ₹22,705 after the vendor was added back, instead of ₹1,43,980. The award was then approved with that wrong total — and the total decides which approval flow applies.</t>
+        </is>
+      </c>
+      <c r="E66" s="7" t="inlineStr">
+        <is>
+          <t>1. Award one line split across three vendors.
+2. Remove one of the vendors from the award, then add it back.
+3. Read the award total.</t>
+        </is>
+      </c>
+      <c r="F66" s="7" t="inlineStr">
+        <is>
+          <t>The total changes by the removed vendor's awarded amount only, and returns to ₹1,43,980 when it is added back.</t>
+        </is>
+      </c>
+      <c r="G66" s="7" t="inlineStr">
+        <is>
+          <t>The total becomes −₹1,550, then ₹22,705, and the award can be approved with it.</t>
+        </is>
+      </c>
+      <c r="H66" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I66" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J66" s="7" t="inlineStr">
+        <is>
+          <t>Wrong result</t>
+        </is>
+      </c>
+      <c r="K66" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on 2 fresh test events on PROCOL DEMO. The award value removed is the vendor's whole bid total (proposal_helper.rb, get_po_value_to_be_added falls back to the bid's gross total).</t>
+        </is>
+      </c>
+      <c r="L66" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M66" s="7" t="inlineStr">
+        <is>
+          <t>API-EVDAWD-003, API-EVDAWD-005</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="7" t="inlineStr">
+        <is>
+          <t>BUG-66</t>
+        </is>
+      </c>
+      <c r="B67" s="7" t="inlineStr">
+        <is>
+          <t>Awarding</t>
+        </is>
+      </c>
+      <c r="C67" s="7" t="inlineStr">
+        <is>
+          <t>Vendors tied at the lowest price are counted as 'not L1' in the award</t>
+        </is>
+      </c>
+      <c r="D67" s="7" t="inlineStr">
+        <is>
+          <t>When two vendors quote the same lowest price, the award summary counts neither of them as L1: the L1 value shows ₹0 and the tied vendors' amounts are counted under 'non-L1'.</t>
+        </is>
+      </c>
+      <c r="E67" s="7" t="inlineStr">
+        <is>
+          <t>1. Create an RFQ and let two vendors quote the same lowest price.
+2. Award the line to one of them and read the award's L1 / non-L1 values.</t>
+        </is>
+      </c>
+      <c r="F67" s="7" t="inlineStr">
+        <is>
+          <t>The tied vendors are L1, so the L1 value is the awarded amount.</t>
+        </is>
+      </c>
+      <c r="G67" s="7" t="inlineStr">
+        <is>
+          <t>L1 shows ₹0 and the award is counted as non-L1.</t>
+        </is>
+      </c>
+      <c r="H67" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO; Demo Account 2</t>
+        </is>
+      </c>
+      <c r="I67" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J67" s="7" t="inlineStr">
+        <is>
+          <t>Wrong result</t>
+        </is>
+      </c>
+      <c r="K67" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on 6 fresh test events across both clients (proposal_helper.rb:994-1001, bid_rank_helper.rb:215-218).</t>
+        </is>
+      </c>
+      <c r="L67" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M67" s="7" t="inlineStr">
+        <is>
+          <t>API-EVDAWD-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="7" t="inlineStr">
+        <is>
+          <t>BUG-67</t>
+        </is>
+      </c>
+      <c r="B68" s="7" t="inlineStr">
+        <is>
+          <t>Awarding</t>
+        </is>
+      </c>
+      <c r="C68" s="7" t="inlineStr">
+        <is>
+          <t>A vendor's awarded quantity cannot be lowered once a line is fully awarded</t>
+        </is>
+      </c>
+      <c r="D68" s="7" t="inlineStr">
+        <is>
+          <t>When a line is fully awarded across vendors and the buyer lowers one vendor's quantity, Procol refuses with 'You cannot select bid with more than requested quantity', because it counts that vendor's current award as well as the new, lower quantity. The only way round it is to remove the vendor and add it again, which triggers the wrong-total problem in the row above.</t>
+        </is>
+      </c>
+      <c r="E68" s="7" t="inlineStr">
+        <is>
+          <t>1. Award a 30 KG line as 15 / 10 / 5 KG.
+2. Change the 5 KG vendor's quantity to 3 KG.</t>
+        </is>
+      </c>
+      <c r="F68" s="7" t="inlineStr">
+        <is>
+          <t>The change is accepted (3 KG is within the requested 30 KG).</t>
+        </is>
+      </c>
+      <c r="G68" s="7" t="inlineStr">
+        <is>
+          <t>Refused: 'You cannot select bid with more than requested quantity'.</t>
+        </is>
+      </c>
+      <c r="H68" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I68" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J68" s="7" t="inlineStr">
+        <is>
+          <t>Business rule</t>
+        </is>
+      </c>
+      <c r="K68" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on 4 fresh test events on PROCOL DEMO (proposal_helper.rb:1295-1305).</t>
+        </is>
+      </c>
+      <c r="L68" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M68" s="7" t="inlineStr">
+        <is>
+          <t>API-EVDAWD-006</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="7" t="inlineStr">
+        <is>
+          <t>BUG-68</t>
+        </is>
+      </c>
+      <c r="B69" s="7" t="inlineStr">
+        <is>
+          <t>Auctions</t>
+        </is>
+      </c>
+      <c r="C69" s="7" t="inlineStr">
+        <is>
+          <t>After an auction's automatic extension, existing bids still show the old end time</t>
+        </is>
+      </c>
+      <c r="D69" s="7" t="inlineStr">
+        <is>
+          <t>When a late bid makes an auction extend automatically, the auction's end time moves, but the bids already placed keep the old end time as their 'valid till' time.</t>
+        </is>
+      </c>
+      <c r="E69" s="7" t="inlineStr">
+        <is>
+          <t>1. Run an auction with automatic extension and several vendors bidding.
+2. Place a winning bid in the last minutes so the auction extends.
+3. Read the earlier bids' end ('valid till') time.</t>
+        </is>
+      </c>
+      <c r="F69" s="7" t="inlineStr">
+        <is>
+          <t>Every bid shows the auction's new end time.</t>
+        </is>
+      </c>
+      <c r="G69" s="7" t="inlineStr">
+        <is>
+          <t>The earlier bids keep the old end time.</t>
+        </is>
+      </c>
+      <c r="H69" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO; Demo Account 2</t>
+        </is>
+      </c>
+      <c r="I69" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J69" s="7" t="inlineStr">
+        <is>
+          <t>Wrong result</t>
+        </is>
+      </c>
+      <c r="K69" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on 4 fresh test events across both clients (bid.rb:2264-2286 keeps the cached schedule).</t>
+        </is>
+      </c>
+      <c r="L69" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M69" s="7" t="inlineStr">
+        <is>
+          <t>API-EVDAUX-004</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deep-dig round 2 (543 cases, 314 runnable twins), deeper code knowledge, rule coverage; bug sheet 79
- Round 2: clarifications, documents, reminders, vendor declines, bid rejection, weighted bidding,
  reschedule/per-line timing, drafts. 198678: 300 run, 231 passed, 62 failed; 32461 part-run.
  11 grouped new verified defects (competitor weights visible to vendors, a malformed attachment
  makes a round unreadable, file-ownership check bypassable, T&C clauses deleted, ...).
- Knowledge: backend digests for models, services, jobs, policies/serializers, settings; console
  screen digests; doc-vs-code contradictions.
- rule-coverage.ts: 3,227 cited rules, 41% covered by a case, 1,567 not covered (docs/rule-coverage.md).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
+++ b/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
@@ -221,8 +221,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:M69" headerRowCount="1">
-  <autoFilter ref="A1:M69"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:M80" headerRowCount="1">
+  <autoFilter ref="A1:M80"/>
   <tableColumns count="13">
     <tableColumn id="1" name="Bug #"/>
     <tableColumn id="2" name="Area"/>
@@ -590,7 +590,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>COUNTA(Bugs!A2:A69)</f>
+        <f>COUNTA(Bugs!A2:A80)</f>
         <v/>
       </c>
     </row>
@@ -609,7 +609,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF(Bugs!I2:I69,A7)</f>
+        <f>COUNTIF(Bugs!I2:I80,A7)</f>
         <v/>
       </c>
     </row>
@@ -620,7 +620,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF(Bugs!I2:I69,A8)</f>
+        <f>COUNTIF(Bugs!I2:I80,A8)</f>
         <v/>
       </c>
     </row>
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIF(Bugs!I2:I69,A9)</f>
+        <f>COUNTIF(Bugs!I2:I80,A9)</f>
         <v/>
       </c>
     </row>
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIF(Bugs!I2:I69,A10)</f>
+        <f>COUNTIF(Bugs!I2:I80,A10)</f>
         <v/>
       </c>
     </row>
@@ -661,7 +661,7 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF(Bugs!J2:J69,A13)</f>
+        <f>COUNTIF(Bugs!J2:J80,A13)</f>
         <v/>
       </c>
     </row>
@@ -672,7 +672,7 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF(Bugs!J2:J69,A14)</f>
+        <f>COUNTIF(Bugs!J2:J80,A14)</f>
         <v/>
       </c>
     </row>
@@ -683,7 +683,7 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF(Bugs!J2:J69,A15)</f>
+        <f>COUNTIF(Bugs!J2:J80,A15)</f>
         <v/>
       </c>
     </row>
@@ -694,7 +694,7 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF(Bugs!J2:J69,A16)</f>
+        <f>COUNTIF(Bugs!J2:J80,A16)</f>
         <v/>
       </c>
     </row>
@@ -705,7 +705,7 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF(Bugs!J2:J69,A17)</f>
+        <f>COUNTIF(Bugs!J2:J80,A17)</f>
         <v/>
       </c>
     </row>
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF(Bugs!J2:J69,A18)</f>
+        <f>COUNTIF(Bugs!J2:J80,A18)</f>
         <v/>
       </c>
     </row>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF(Bugs!J2:J69,A19)</f>
+        <f>COUNTIF(Bugs!J2:J80,A19)</f>
         <v/>
       </c>
     </row>
@@ -738,7 +738,7 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF(Bugs!J2:J69,A20)</f>
+        <f>COUNTIF(Bugs!J2:J80,A20)</f>
         <v/>
       </c>
     </row>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF(Bugs!J2:J69,A21)</f>
+        <f>COUNTIF(Bugs!J2:J80,A21)</f>
         <v/>
       </c>
     </row>
@@ -760,7 +760,7 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF(Bugs!J2:J69,A22)</f>
+        <f>COUNTIF(Bugs!J2:J80,A22)</f>
         <v/>
       </c>
     </row>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B25" s="5">
-        <f>COUNTIF(Bugs!H2:H69,"*"&amp;A25&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H80,"*"&amp;A25&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF(Bugs!H2:H69,"*"&amp;A26&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H80,"*"&amp;A26&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -801,7 +801,7 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF(Bugs!H2:H69,"*"&amp;A27&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H80,"*"&amp;A27&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -849,7 +849,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M69"/>
+  <dimension ref="A1:M80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -5377,6 +5377,754 @@
       <c r="M69" s="7" t="inlineStr">
         <is>
           <t>API-EVDAUX-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="7" t="inlineStr">
+        <is>
+          <t>BUG-69</t>
+        </is>
+      </c>
+      <c r="B70" s="7" t="inlineStr">
+        <is>
+          <t>Bidding &amp; vendor permissions</t>
+        </is>
+      </c>
+      <c r="C70" s="7" t="inlineStr">
+        <is>
+          <t>A vendor can read the weight the buyer gave a competing vendor</t>
+        </is>
+      </c>
+      <c r="D70" s="7" t="inlineStr">
+        <is>
+          <t>In weighted bidding the buyer gives each vendor a weight that changes how its price is ranked. These weights are the buyer's private assessment. When a vendor opens the round, the data Procol sends it includes the weight the buyer set for every other vendor, not just its own.</t>
+        </is>
+      </c>
+      <c r="E70" s="7" t="inlineStr">
+        <is>
+          <t>1. On a live RFQ with weighted bidding, give QA vendor 1 a weight of 100 and QA vendor 2 a weight of 300.
+2. Sign in as vendor 1 and open the round.
+3. Look at the data the app sent.</t>
+        </is>
+      </c>
+      <c r="F70" s="7" t="inlineStr">
+        <is>
+          <t>Vendor 1 receives only its own weight (or none).</t>
+        </is>
+      </c>
+      <c r="G70" s="7" t="inlineStr">
+        <is>
+          <t>Vendor 1 receives vendor 2's weight (300).</t>
+        </is>
+      </c>
+      <c r="H70" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I70" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J70" s="7" t="inlineStr">
+        <is>
+          <t>Data leak</t>
+        </is>
+      </c>
+      <c r="K70" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on PROCOL DEMO on 3–4 Oct 2026: each variant failed the same way on two fresh test events. Cause: trade_template_serializer.rb:877-879 sends every vendor's weights.</t>
+        </is>
+      </c>
+      <c r="L70" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M70" s="7" t="inlineStr">
+        <is>
+          <t>API-EVDWGT-071</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="7" t="inlineStr">
+        <is>
+          <t>BUG-70</t>
+        </is>
+      </c>
+      <c r="B71" s="7" t="inlineStr">
+        <is>
+          <t>Documents</t>
+        </is>
+      </c>
+      <c r="C71" s="7" t="inlineStr">
+        <is>
+          <t>One badly formed attachment makes the event or round unreadable for everyone</t>
+        </is>
+      </c>
+      <c r="D71" s="7" t="inlineStr">
+        <is>
+          <t>When an attachment is saved in the wrong shape (for example as plain text instead of a file entry), Procol accepts and stores it. From then on every attempt to open that round crashes, for the buyer and for the vendors — the event is effectively broken.</t>
+        </is>
+      </c>
+      <c r="E71" s="7" t="inlineStr">
+        <is>
+          <t>1. Publish an event.
+2. Save the round's terms-and-conditions attachments with a value that is plain text instead of a file entry.
+3. Open the round again (as buyer or vendor).</t>
+        </is>
+      </c>
+      <c r="F71" s="7" t="inlineStr">
+        <is>
+          <t>The bad attachment is refused when it is saved; the round keeps working.</t>
+        </is>
+      </c>
+      <c r="G71" s="7" t="inlineStr">
+        <is>
+          <t>The save is accepted, and every later opening of the round crashes.</t>
+        </is>
+      </c>
+      <c r="H71" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I71" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J71" s="7" t="inlineStr">
+        <is>
+          <t>Data integrity</t>
+        </is>
+      </c>
+      <c r="K71" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on PROCOL DEMO on 3–4 Oct 2026: each variant failed the same way on two fresh test events. (event_group.rb:329-338; trade_controller.rb).</t>
+        </is>
+      </c>
+      <c r="L71" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M71" s="7" t="inlineStr">
+        <is>
+          <t>API-EVDDOC-046, API-EVDDOC-051, API-EVDDOC-052</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="7" t="inlineStr">
+        <is>
+          <t>BUG-71</t>
+        </is>
+      </c>
+      <c r="B72" s="7" t="inlineStr">
+        <is>
+          <t>Documents</t>
+        </is>
+      </c>
+      <c r="C72" s="7" t="inlineStr">
+        <is>
+          <t>The check that an attached file belongs to the buyer's own company can be bypassed</t>
+        </is>
+      </c>
+      <c r="D72" s="7" t="inlineStr">
+        <is>
+          <t>Procol checks that a file linked to an event comes from the company's own storage. That check can be passed with an encoded link or a link to another host, so a file that is not the company's own is accepted. We proved only that the check lets such links through; we did not read another company's file.</t>
+        </is>
+      </c>
+      <c r="E72" s="7" t="inlineStr">
+        <is>
+          <t>1. Attach a file to an event using a link whose address is encoded, or points to another storage host.
+2. Save the event.</t>
+        </is>
+      </c>
+      <c r="F72" s="7" t="inlineStr">
+        <is>
+          <t>The link is refused because the file is not in the company's own storage.</t>
+        </is>
+      </c>
+      <c r="G72" s="7" t="inlineStr">
+        <is>
+          <t>The link is accepted.</t>
+        </is>
+      </c>
+      <c r="H72" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I72" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J72" s="7" t="inlineStr">
+        <is>
+          <t>Permission / business rule</t>
+        </is>
+      </c>
+      <c r="K72" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on PROCOL DEMO on 3–4 Oct 2026: each variant failed the same way on two fresh test events. (s3_url_validator.rb:25-33).</t>
+        </is>
+      </c>
+      <c r="L72" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M72" s="7" t="inlineStr">
+        <is>
+          <t>API-EVDDOC-043, API-EVDDOC-044, API-EVDDOC-045, API-EVDDOC-049</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="7" t="inlineStr">
+        <is>
+          <t>BUG-72</t>
+        </is>
+      </c>
+      <c r="B73" s="7" t="inlineStr">
+        <is>
+          <t>Documents</t>
+        </is>
+      </c>
+      <c r="C73" s="7" t="inlineStr">
+        <is>
+          <t>Changing only a round's terms-and-conditions files deletes its written clauses</t>
+        </is>
+      </c>
+      <c r="D73" s="7" t="inlineStr">
+        <is>
+          <t>A round's terms and conditions have written clauses and attached files. Updating only the files deletes every written clause, without any warning.</t>
+        </is>
+      </c>
+      <c r="E73" s="7" t="inlineStr">
+        <is>
+          <t>1. Give a round written T&amp;C clauses and a T&amp;C file.
+2. Update only the round's T&amp;C files.
+3. Read the round's T&amp;C.</t>
+        </is>
+      </c>
+      <c r="F73" s="7" t="inlineStr">
+        <is>
+          <t>The written clauses stay as they were.</t>
+        </is>
+      </c>
+      <c r="G73" s="7" t="inlineStr">
+        <is>
+          <t>All written clauses are gone.</t>
+        </is>
+      </c>
+      <c r="H73" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I73" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J73" s="7" t="inlineStr">
+        <is>
+          <t>Data integrity</t>
+        </is>
+      </c>
+      <c r="K73" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on PROCOL DEMO on 3–4 Oct 2026: each variant failed the same way on two fresh test events. (trade_controller.rb:714-720).</t>
+        </is>
+      </c>
+      <c r="L73" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M73" s="7" t="inlineStr">
+        <is>
+          <t>API-EVDDOC-053</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="7" t="inlineStr">
+        <is>
+          <t>BUG-73</t>
+        </is>
+      </c>
+      <c r="B74" s="7" t="inlineStr">
+        <is>
+          <t>Documents</t>
+        </is>
+      </c>
+      <c r="C74" s="7" t="inlineStr">
+        <is>
+          <t>An upload reports success for content it did not store</t>
+        </is>
+      </c>
+      <c r="D74" s="7" t="inlineStr">
+        <is>
+          <t>When a file upload sends content Procol does not store, the upload still answers 'Successfully uploaded File', so the user believes the file is attached when it is not.</t>
+        </is>
+      </c>
+      <c r="E74" s="7" t="inlineStr">
+        <is>
+          <t>1. Upload a file to a round with content that Procol does not keep (for example an empty or unsupported upload).
+2. Read the round's files.</t>
+        </is>
+      </c>
+      <c r="F74" s="7" t="inlineStr">
+        <is>
+          <t>The upload is refused, or reports that nothing was stored.</t>
+        </is>
+      </c>
+      <c r="G74" s="7" t="inlineStr">
+        <is>
+          <t>'Successfully uploaded File' — and nothing is attached.</t>
+        </is>
+      </c>
+      <c r="H74" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I74" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J74" s="7" t="inlineStr">
+        <is>
+          <t>Wrong result</t>
+        </is>
+      </c>
+      <c r="K74" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on PROCOL DEMO on 3–4 Oct 2026: each variant failed the same way on two fresh test events. (s3_upload.rb:83-101).</t>
+        </is>
+      </c>
+      <c r="L74" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M74" s="7" t="inlineStr">
+        <is>
+          <t>API-EVDDOC-015, API-EVDDOC-016, API-EVDDOC-017</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="7" t="inlineStr">
+        <is>
+          <t>BUG-74</t>
+        </is>
+      </c>
+      <c r="B75" s="7" t="inlineStr">
+        <is>
+          <t>Event update</t>
+        </is>
+      </c>
+      <c r="C75" s="7" t="inlineStr">
+        <is>
+          <t>Saving any partial change to a draft round crashes</t>
+        </is>
+      </c>
+      <c r="D75" s="7" t="inlineStr">
+        <is>
+          <t>Updating a draft round with only some of its fields — even with nothing in the update — crashes the server, so a draft round cannot be edited one field at a time.</t>
+        </is>
+      </c>
+      <c r="E75" s="7" t="inlineStr">
+        <is>
+          <t>1. Create a draft event with a round.
+2. Update the round with only one changed field (or with an empty update).</t>
+        </is>
+      </c>
+      <c r="F75" s="7" t="inlineStr">
+        <is>
+          <t>The change is saved (or an empty update does nothing).</t>
+        </is>
+      </c>
+      <c r="G75" s="7" t="inlineStr">
+        <is>
+          <t>The server crashes.</t>
+        </is>
+      </c>
+      <c r="H75" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I75" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J75" s="7" t="inlineStr">
+        <is>
+          <t>Server crash</t>
+        </is>
+      </c>
+      <c r="K75" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on PROCOL DEMO on 3–4 Oct 2026: each variant failed the same way on two fresh test events. (trade_controller.rb:603 sends drafts to edit_draft).</t>
+        </is>
+      </c>
+      <c r="L75" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M75" s="7" t="inlineStr">
+        <is>
+          <t>API-EVDDRF-001, API-EVDDRF-002, API-EVDDRF-003, API-EVDDRF-004, API-EVDDRF-005, API-EVDDRF-006, API-EVDDRF-007</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="7" t="inlineStr">
+        <is>
+          <t>BUG-75</t>
+        </is>
+      </c>
+      <c r="B76" s="7" t="inlineStr">
+        <is>
+          <t>Clarifications</t>
+        </is>
+      </c>
+      <c r="C76" s="7" t="inlineStr">
+        <is>
+          <t>Clarification questions crash for an unknown or draft event and on malformed filters</t>
+        </is>
+      </c>
+      <c r="D76" s="7" t="inlineStr">
+        <is>
+          <t>Vendors and the buyer exchange clarification questions inside an event. Asking for or creating clarifications on an event that does not exist or is still a draft, or sending malformed filters, context or attachments, crashes the server instead of answering 'not found' or refusing the request.</t>
+        </is>
+      </c>
+      <c r="E76" s="7" t="inlineStr">
+        <is>
+          <t>1. Open clarifications for an event id that does not exist (or a draft event).
+2. Or send a clarification with malformed filters or attachments.</t>
+        </is>
+      </c>
+      <c r="F76" s="7" t="inlineStr">
+        <is>
+          <t>'Not found', or a clear refusal.</t>
+        </is>
+      </c>
+      <c r="G76" s="7" t="inlineStr">
+        <is>
+          <t>The server crashes.</t>
+        </is>
+      </c>
+      <c r="H76" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO; Demo Account 2</t>
+        </is>
+      </c>
+      <c r="I76" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J76" s="7" t="inlineStr">
+        <is>
+          <t>Server crash</t>
+        </is>
+      </c>
+      <c r="K76" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on both clients (18 variants on PROCOL DEMO, 8 on Demo Account 2), each on two fresh test events (v1/chats_controller.rb).</t>
+        </is>
+      </c>
+      <c r="L76" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M76" s="7" t="inlineStr">
+        <is>
+          <t>API-EVDQRY-004, API-EVDQRY-008, API-EVDQRY-014, API-EVDQRY-018, API-EVDQRY-019, API-EVDQRY-020, API-EVDQRY-021, API-EVDQRY-023, API-EVDQRY-024, API-EVDQRY-025, API-EVDQRY-026, API-EVDQRY-041, API-EVDQRY-055, API-EVDQRY-056, API-EVDQRY-057, API-EVDQRY-061, API-EVDQRY-062, API-EVDQRY-068</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="7" t="inlineStr">
+        <is>
+          <t>BUG-76</t>
+        </is>
+      </c>
+      <c r="B77" s="7" t="inlineStr">
+        <is>
+          <t>Reminders</t>
+        </is>
+      </c>
+      <c r="C77" s="7" t="inlineStr">
+        <is>
+          <t>Sending or listing reminders crashes on malformed or unknown input</t>
+        </is>
+      </c>
+      <c r="D77" s="7" t="inlineStr">
+        <is>
+          <t>The buyer can send reminders to vendors who still have to act. Sending reminders without the list of recipients, with the recipients written as text, with an unknown reminder type, or for an event that does not exist crashes the server instead of refusing.</t>
+        </is>
+      </c>
+      <c r="E77" s="7" t="inlineStr">
+        <is>
+          <t>1. Send reminders for an event without saying who should get them (or with an unknown reminder type, or for an event that does not exist).</t>
+        </is>
+      </c>
+      <c r="F77" s="7" t="inlineStr">
+        <is>
+          <t>A clear refusal or 'not found'.</t>
+        </is>
+      </c>
+      <c r="G77" s="7" t="inlineStr">
+        <is>
+          <t>The server crashes.</t>
+        </is>
+      </c>
+      <c r="H77" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I77" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J77" s="7" t="inlineStr">
+        <is>
+          <t>Server crash</t>
+        </is>
+      </c>
+      <c r="K77" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on PROCOL DEMO on 3–4 Oct 2026: each variant failed the same way on two fresh test events. (reminders_controller.rb; reminders/base_service.rb:40).</t>
+        </is>
+      </c>
+      <c r="L77" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M77" s="7" t="inlineStr">
+        <is>
+          <t>API-EVDREM-019, API-EVDREM-020, API-EVDREM-024, API-EVDREM-048, API-EVDREM-049, API-EVDREM-050, API-EVDREM-051, API-EVDREM-052, API-EVDREM-057, API-EVDREM-058, API-EVDREM-059</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="7" t="inlineStr">
+        <is>
+          <t>BUG-77</t>
+        </is>
+      </c>
+      <c r="B78" s="7" t="inlineStr">
+        <is>
+          <t>Documents</t>
+        </is>
+      </c>
+      <c r="C78" s="7" t="inlineStr">
+        <is>
+          <t>Malformed attachments on a round or a surrogate bid crash, and the attachment link crashes without a token</t>
+        </is>
+      </c>
+      <c r="D78" s="7" t="inlineStr">
+        <is>
+          <t>Sending a round's attachments in the wrong shape, or a bid entered on a vendor's behalf with a reference note but no files, crashes the server. The attachment-link address also crashes when it is called without a token instead of refusing.</t>
+        </is>
+      </c>
+      <c r="E78" s="7" t="inlineStr">
+        <is>
+          <t>1. Update a round with attachments in the wrong shape (or enter a surrogate bid with a note and no files).
+2. Or open an attachment link without its token.</t>
+        </is>
+      </c>
+      <c r="F78" s="7" t="inlineStr">
+        <is>
+          <t>A clear refusal.</t>
+        </is>
+      </c>
+      <c r="G78" s="7" t="inlineStr">
+        <is>
+          <t>The server crashes.</t>
+        </is>
+      </c>
+      <c r="H78" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO; Demo Account 2</t>
+        </is>
+      </c>
+      <c r="I78" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J78" s="7" t="inlineStr">
+        <is>
+          <t>Server crash</t>
+        </is>
+      </c>
+      <c r="K78" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on two fresh test events per variant; the attachment-link variant on both clients (trade_controller.rb:459; v1/attachments_controller.rb:12-18).</t>
+        </is>
+      </c>
+      <c r="L78" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M78" s="7" t="inlineStr">
+        <is>
+          <t>API-EVDDOC-034, API-EVDDOC-039, API-EVDDOC-054, API-EVDDOC-055, API-EVDDOC-061, API-EVDDOC-062</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="7" t="inlineStr">
+        <is>
+          <t>BUG-78</t>
+        </is>
+      </c>
+      <c r="B79" s="7" t="inlineStr">
+        <is>
+          <t>Weighted bidding</t>
+        </is>
+      </c>
+      <c r="C79" s="7" t="inlineStr">
+        <is>
+          <t>Saving malformed weights crashes</t>
+        </is>
+      </c>
+      <c r="D79" s="7" t="inlineStr">
+        <is>
+          <t>Saving vendor weights in the wrong shape (for example text where a number belongs) crashes the server instead of refusing the weights.</t>
+        </is>
+      </c>
+      <c r="E79" s="7" t="inlineStr">
+        <is>
+          <t>1. On a round with weighted bidding, save the weights with a value in the wrong shape.</t>
+        </is>
+      </c>
+      <c r="F79" s="7" t="inlineStr">
+        <is>
+          <t>A clear refusal naming the bad weight.</t>
+        </is>
+      </c>
+      <c r="G79" s="7" t="inlineStr">
+        <is>
+          <t>The server crashes.</t>
+        </is>
+      </c>
+      <c r="H79" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I79" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J79" s="7" t="inlineStr">
+        <is>
+          <t>Server crash</t>
+        </is>
+      </c>
+      <c r="K79" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on PROCOL DEMO on 3–4 Oct 2026: each variant failed the same way on two fresh test events. (trade_controller.rb:1779,1804).</t>
+        </is>
+      </c>
+      <c r="L79" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M79" s="7" t="inlineStr">
+        <is>
+          <t>API-EVDWGT-047, API-EVDWGT-048, API-EVDWGT-050, API-EVDWGT-051, API-EVDWGT-052, API-EVDWGT-053</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="7" t="inlineStr">
+        <is>
+          <t>BUG-79</t>
+        </is>
+      </c>
+      <c r="B80" s="7" t="inlineStr">
+        <is>
+          <t>Event update</t>
+        </is>
+      </c>
+      <c r="C80" s="7" t="inlineStr">
+        <is>
+          <t>Sending an empty value for any list of ids crashes the server</t>
+        </is>
+      </c>
+      <c r="D80" s="7" t="inlineStr">
+        <is>
+          <t>Many requests carry lists of ids (for example the line items to reopen). Sending an empty value instead of a list for any such field crashes the server before the request is even looked at, because a shared check does not expect it.</t>
+        </is>
+      </c>
+      <c r="E80" s="7" t="inlineStr">
+        <is>
+          <t>1. Reopen line items on a round with the list of line items sent as an empty value.</t>
+        </is>
+      </c>
+      <c r="F80" s="7" t="inlineStr">
+        <is>
+          <t>A clear refusal, or the request treated as an empty list.</t>
+        </is>
+      </c>
+      <c r="G80" s="7" t="inlineStr">
+        <is>
+          <t>The server crashes.</t>
+        </is>
+      </c>
+      <c r="H80" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I80" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J80" s="7" t="inlineStr">
+        <is>
+          <t>Server crash</t>
+        </is>
+      </c>
+      <c r="K80" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on PROCOL DEMO on 3–4 Oct 2026: each variant failed the same way on two fresh test events. (params_auth.rb:70-73 — applies to every such field).</t>
+        </is>
+      </c>
+      <c r="L80" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M80" s="7" t="inlineStr">
+        <is>
+          <t>API-EVDTME-054</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deep-dig round 2, code knowledge, rule coverage; bug sheet 79
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
+++ b/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
@@ -221,8 +221,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:M69" headerRowCount="1">
-  <autoFilter ref="A1:M69"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:M80" headerRowCount="1">
+  <autoFilter ref="A1:M80"/>
   <tableColumns count="13">
     <tableColumn id="1" name="Bug #"/>
     <tableColumn id="2" name="Area"/>
@@ -590,7 +590,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>COUNTA(Bugs!A2:A69)</f>
+        <f>COUNTA(Bugs!A2:A80)</f>
         <v/>
       </c>
     </row>
@@ -609,7 +609,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF(Bugs!I2:I69,A7)</f>
+        <f>COUNTIF(Bugs!I2:I80,A7)</f>
         <v/>
       </c>
     </row>
@@ -620,7 +620,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF(Bugs!I2:I69,A8)</f>
+        <f>COUNTIF(Bugs!I2:I80,A8)</f>
         <v/>
       </c>
     </row>
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIF(Bugs!I2:I69,A9)</f>
+        <f>COUNTIF(Bugs!I2:I80,A9)</f>
         <v/>
       </c>
     </row>
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIF(Bugs!I2:I69,A10)</f>
+        <f>COUNTIF(Bugs!I2:I80,A10)</f>
         <v/>
       </c>
     </row>
@@ -661,7 +661,7 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF(Bugs!J2:J69,A13)</f>
+        <f>COUNTIF(Bugs!J2:J80,A13)</f>
         <v/>
       </c>
     </row>
@@ -672,7 +672,7 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF(Bugs!J2:J69,A14)</f>
+        <f>COUNTIF(Bugs!J2:J80,A14)</f>
         <v/>
       </c>
     </row>
@@ -683,7 +683,7 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF(Bugs!J2:J69,A15)</f>
+        <f>COUNTIF(Bugs!J2:J80,A15)</f>
         <v/>
       </c>
     </row>
@@ -694,7 +694,7 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF(Bugs!J2:J69,A16)</f>
+        <f>COUNTIF(Bugs!J2:J80,A16)</f>
         <v/>
       </c>
     </row>
@@ -705,7 +705,7 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF(Bugs!J2:J69,A17)</f>
+        <f>COUNTIF(Bugs!J2:J80,A17)</f>
         <v/>
       </c>
     </row>
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF(Bugs!J2:J69,A18)</f>
+        <f>COUNTIF(Bugs!J2:J80,A18)</f>
         <v/>
       </c>
     </row>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF(Bugs!J2:J69,A19)</f>
+        <f>COUNTIF(Bugs!J2:J80,A19)</f>
         <v/>
       </c>
     </row>
@@ -738,7 +738,7 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF(Bugs!J2:J69,A20)</f>
+        <f>COUNTIF(Bugs!J2:J80,A20)</f>
         <v/>
       </c>
     </row>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF(Bugs!J2:J69,A21)</f>
+        <f>COUNTIF(Bugs!J2:J80,A21)</f>
         <v/>
       </c>
     </row>
@@ -760,7 +760,7 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF(Bugs!J2:J69,A22)</f>
+        <f>COUNTIF(Bugs!J2:J80,A22)</f>
         <v/>
       </c>
     </row>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B25" s="5">
-        <f>COUNTIF(Bugs!H2:H69,"*"&amp;A25&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H80,"*"&amp;A25&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF(Bugs!H2:H69,"*"&amp;A26&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H80,"*"&amp;A26&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -801,7 +801,7 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF(Bugs!H2:H69,"*"&amp;A27&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H80,"*"&amp;A27&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -849,7 +849,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M69"/>
+  <dimension ref="A1:M80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -5377,6 +5377,754 @@
       <c r="M69" s="7" t="inlineStr">
         <is>
           <t>API-EVDAUX-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="7" t="inlineStr">
+        <is>
+          <t>BUG-69</t>
+        </is>
+      </c>
+      <c r="B70" s="7" t="inlineStr">
+        <is>
+          <t>Bidding &amp; vendor permissions</t>
+        </is>
+      </c>
+      <c r="C70" s="7" t="inlineStr">
+        <is>
+          <t>A vendor can read the weight the buyer gave a competing vendor</t>
+        </is>
+      </c>
+      <c r="D70" s="7" t="inlineStr">
+        <is>
+          <t>In weighted bidding the buyer gives each vendor a weight that changes how its price is ranked. These weights are the buyer's private assessment. When a vendor opens the round, the data Procol sends it includes the weight the buyer set for every other vendor, not just its own.</t>
+        </is>
+      </c>
+      <c r="E70" s="7" t="inlineStr">
+        <is>
+          <t>1. On a live RFQ with weighted bidding, give QA vendor 1 a weight of 100 and QA vendor 2 a weight of 300.
+2. Sign in as vendor 1 and open the round.
+3. Look at the data the app sent.</t>
+        </is>
+      </c>
+      <c r="F70" s="7" t="inlineStr">
+        <is>
+          <t>Vendor 1 receives only its own weight (or none).</t>
+        </is>
+      </c>
+      <c r="G70" s="7" t="inlineStr">
+        <is>
+          <t>Vendor 1 receives vendor 2's weight (300).</t>
+        </is>
+      </c>
+      <c r="H70" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I70" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J70" s="7" t="inlineStr">
+        <is>
+          <t>Data leak</t>
+        </is>
+      </c>
+      <c r="K70" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on PROCOL DEMO on 3–4 Oct 2026: each variant failed the same way on two fresh test events. Cause: trade_template_serializer.rb:877-879 sends every vendor's weights.</t>
+        </is>
+      </c>
+      <c r="L70" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M70" s="7" t="inlineStr">
+        <is>
+          <t>API-EVDWGT-071</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="7" t="inlineStr">
+        <is>
+          <t>BUG-70</t>
+        </is>
+      </c>
+      <c r="B71" s="7" t="inlineStr">
+        <is>
+          <t>Documents</t>
+        </is>
+      </c>
+      <c r="C71" s="7" t="inlineStr">
+        <is>
+          <t>One badly formed attachment makes the event or round unreadable for everyone</t>
+        </is>
+      </c>
+      <c r="D71" s="7" t="inlineStr">
+        <is>
+          <t>When an attachment is saved in the wrong shape (for example as plain text instead of a file entry), Procol accepts and stores it. From then on every attempt to open that round crashes, for the buyer and for the vendors — the event is effectively broken.</t>
+        </is>
+      </c>
+      <c r="E71" s="7" t="inlineStr">
+        <is>
+          <t>1. Publish an event.
+2. Save the round's terms-and-conditions attachments with a value that is plain text instead of a file entry.
+3. Open the round again (as buyer or vendor).</t>
+        </is>
+      </c>
+      <c r="F71" s="7" t="inlineStr">
+        <is>
+          <t>The bad attachment is refused when it is saved; the round keeps working.</t>
+        </is>
+      </c>
+      <c r="G71" s="7" t="inlineStr">
+        <is>
+          <t>The save is accepted, and every later opening of the round crashes.</t>
+        </is>
+      </c>
+      <c r="H71" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I71" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J71" s="7" t="inlineStr">
+        <is>
+          <t>Data integrity</t>
+        </is>
+      </c>
+      <c r="K71" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on PROCOL DEMO on 3–4 Oct 2026: each variant failed the same way on two fresh test events. (event_group.rb:329-338; trade_controller.rb).</t>
+        </is>
+      </c>
+      <c r="L71" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M71" s="7" t="inlineStr">
+        <is>
+          <t>API-EVDDOC-046, API-EVDDOC-051, API-EVDDOC-052</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="7" t="inlineStr">
+        <is>
+          <t>BUG-71</t>
+        </is>
+      </c>
+      <c r="B72" s="7" t="inlineStr">
+        <is>
+          <t>Documents</t>
+        </is>
+      </c>
+      <c r="C72" s="7" t="inlineStr">
+        <is>
+          <t>The check that an attached file belongs to the buyer's own company can be bypassed</t>
+        </is>
+      </c>
+      <c r="D72" s="7" t="inlineStr">
+        <is>
+          <t>Procol checks that a file linked to an event comes from the company's own storage. That check can be passed with an encoded link or a link to another host, so a file that is not the company's own is accepted. We proved only that the check lets such links through; we did not read another company's file.</t>
+        </is>
+      </c>
+      <c r="E72" s="7" t="inlineStr">
+        <is>
+          <t>1. Attach a file to an event using a link whose address is encoded, or points to another storage host.
+2. Save the event.</t>
+        </is>
+      </c>
+      <c r="F72" s="7" t="inlineStr">
+        <is>
+          <t>The link is refused because the file is not in the company's own storage.</t>
+        </is>
+      </c>
+      <c r="G72" s="7" t="inlineStr">
+        <is>
+          <t>The link is accepted.</t>
+        </is>
+      </c>
+      <c r="H72" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I72" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J72" s="7" t="inlineStr">
+        <is>
+          <t>Permission / business rule</t>
+        </is>
+      </c>
+      <c r="K72" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on PROCOL DEMO on 3–4 Oct 2026: each variant failed the same way on two fresh test events. (s3_url_validator.rb:25-33).</t>
+        </is>
+      </c>
+      <c r="L72" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M72" s="7" t="inlineStr">
+        <is>
+          <t>API-EVDDOC-043, API-EVDDOC-044, API-EVDDOC-045, API-EVDDOC-049</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="7" t="inlineStr">
+        <is>
+          <t>BUG-72</t>
+        </is>
+      </c>
+      <c r="B73" s="7" t="inlineStr">
+        <is>
+          <t>Documents</t>
+        </is>
+      </c>
+      <c r="C73" s="7" t="inlineStr">
+        <is>
+          <t>Changing only a round's terms-and-conditions files deletes its written clauses</t>
+        </is>
+      </c>
+      <c r="D73" s="7" t="inlineStr">
+        <is>
+          <t>A round's terms and conditions have written clauses and attached files. Updating only the files deletes every written clause, without any warning.</t>
+        </is>
+      </c>
+      <c r="E73" s="7" t="inlineStr">
+        <is>
+          <t>1. Give a round written T&amp;C clauses and a T&amp;C file.
+2. Update only the round's T&amp;C files.
+3. Read the round's T&amp;C.</t>
+        </is>
+      </c>
+      <c r="F73" s="7" t="inlineStr">
+        <is>
+          <t>The written clauses stay as they were.</t>
+        </is>
+      </c>
+      <c r="G73" s="7" t="inlineStr">
+        <is>
+          <t>All written clauses are gone.</t>
+        </is>
+      </c>
+      <c r="H73" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I73" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J73" s="7" t="inlineStr">
+        <is>
+          <t>Data integrity</t>
+        </is>
+      </c>
+      <c r="K73" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on PROCOL DEMO on 3–4 Oct 2026: each variant failed the same way on two fresh test events. (trade_controller.rb:714-720).</t>
+        </is>
+      </c>
+      <c r="L73" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M73" s="7" t="inlineStr">
+        <is>
+          <t>API-EVDDOC-053</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="7" t="inlineStr">
+        <is>
+          <t>BUG-73</t>
+        </is>
+      </c>
+      <c r="B74" s="7" t="inlineStr">
+        <is>
+          <t>Documents</t>
+        </is>
+      </c>
+      <c r="C74" s="7" t="inlineStr">
+        <is>
+          <t>An upload reports success for content it did not store</t>
+        </is>
+      </c>
+      <c r="D74" s="7" t="inlineStr">
+        <is>
+          <t>When a file upload sends content Procol does not store, the upload still answers 'Successfully uploaded File', so the user believes the file is attached when it is not.</t>
+        </is>
+      </c>
+      <c r="E74" s="7" t="inlineStr">
+        <is>
+          <t>1. Upload a file to a round with content that Procol does not keep (for example an empty or unsupported upload).
+2. Read the round's files.</t>
+        </is>
+      </c>
+      <c r="F74" s="7" t="inlineStr">
+        <is>
+          <t>The upload is refused, or reports that nothing was stored.</t>
+        </is>
+      </c>
+      <c r="G74" s="7" t="inlineStr">
+        <is>
+          <t>'Successfully uploaded File' — and nothing is attached.</t>
+        </is>
+      </c>
+      <c r="H74" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I74" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J74" s="7" t="inlineStr">
+        <is>
+          <t>Wrong result</t>
+        </is>
+      </c>
+      <c r="K74" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on PROCOL DEMO on 3–4 Oct 2026: each variant failed the same way on two fresh test events. (s3_upload.rb:83-101).</t>
+        </is>
+      </c>
+      <c r="L74" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M74" s="7" t="inlineStr">
+        <is>
+          <t>API-EVDDOC-015, API-EVDDOC-016, API-EVDDOC-017</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="7" t="inlineStr">
+        <is>
+          <t>BUG-74</t>
+        </is>
+      </c>
+      <c r="B75" s="7" t="inlineStr">
+        <is>
+          <t>Event update</t>
+        </is>
+      </c>
+      <c r="C75" s="7" t="inlineStr">
+        <is>
+          <t>Saving any partial change to a draft round crashes</t>
+        </is>
+      </c>
+      <c r="D75" s="7" t="inlineStr">
+        <is>
+          <t>Updating a draft round with only some of its fields — even with nothing in the update — crashes the server, so a draft round cannot be edited one field at a time.</t>
+        </is>
+      </c>
+      <c r="E75" s="7" t="inlineStr">
+        <is>
+          <t>1. Create a draft event with a round.
+2. Update the round with only one changed field (or with an empty update).</t>
+        </is>
+      </c>
+      <c r="F75" s="7" t="inlineStr">
+        <is>
+          <t>The change is saved (or an empty update does nothing).</t>
+        </is>
+      </c>
+      <c r="G75" s="7" t="inlineStr">
+        <is>
+          <t>The server crashes.</t>
+        </is>
+      </c>
+      <c r="H75" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I75" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J75" s="7" t="inlineStr">
+        <is>
+          <t>Server crash</t>
+        </is>
+      </c>
+      <c r="K75" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on PROCOL DEMO on 3–4 Oct 2026: each variant failed the same way on two fresh test events. (trade_controller.rb:603 sends drafts to edit_draft).</t>
+        </is>
+      </c>
+      <c r="L75" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M75" s="7" t="inlineStr">
+        <is>
+          <t>API-EVDDRF-001, API-EVDDRF-002, API-EVDDRF-003, API-EVDDRF-004, API-EVDDRF-005, API-EVDDRF-006, API-EVDDRF-007</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="7" t="inlineStr">
+        <is>
+          <t>BUG-75</t>
+        </is>
+      </c>
+      <c r="B76" s="7" t="inlineStr">
+        <is>
+          <t>Clarifications</t>
+        </is>
+      </c>
+      <c r="C76" s="7" t="inlineStr">
+        <is>
+          <t>Clarification questions crash for an unknown or draft event and on malformed filters</t>
+        </is>
+      </c>
+      <c r="D76" s="7" t="inlineStr">
+        <is>
+          <t>Vendors and the buyer exchange clarification questions inside an event. Asking for or creating clarifications on an event that does not exist or is still a draft, or sending malformed filters, context or attachments, crashes the server instead of answering 'not found' or refusing the request.</t>
+        </is>
+      </c>
+      <c r="E76" s="7" t="inlineStr">
+        <is>
+          <t>1. Open clarifications for an event id that does not exist (or a draft event).
+2. Or send a clarification with malformed filters or attachments.</t>
+        </is>
+      </c>
+      <c r="F76" s="7" t="inlineStr">
+        <is>
+          <t>'Not found', or a clear refusal.</t>
+        </is>
+      </c>
+      <c r="G76" s="7" t="inlineStr">
+        <is>
+          <t>The server crashes.</t>
+        </is>
+      </c>
+      <c r="H76" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO; Demo Account 2</t>
+        </is>
+      </c>
+      <c r="I76" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J76" s="7" t="inlineStr">
+        <is>
+          <t>Server crash</t>
+        </is>
+      </c>
+      <c r="K76" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on both clients (18 variants on PROCOL DEMO, 8 on Demo Account 2), each on two fresh test events (v1/chats_controller.rb).</t>
+        </is>
+      </c>
+      <c r="L76" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M76" s="7" t="inlineStr">
+        <is>
+          <t>API-EVDQRY-004, API-EVDQRY-008, API-EVDQRY-014, API-EVDQRY-018, API-EVDQRY-019, API-EVDQRY-020, API-EVDQRY-021, API-EVDQRY-023, API-EVDQRY-024, API-EVDQRY-025, API-EVDQRY-026, API-EVDQRY-041, API-EVDQRY-055, API-EVDQRY-056, API-EVDQRY-057, API-EVDQRY-061, API-EVDQRY-062, API-EVDQRY-068</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="7" t="inlineStr">
+        <is>
+          <t>BUG-76</t>
+        </is>
+      </c>
+      <c r="B77" s="7" t="inlineStr">
+        <is>
+          <t>Reminders</t>
+        </is>
+      </c>
+      <c r="C77" s="7" t="inlineStr">
+        <is>
+          <t>Sending or listing reminders crashes on malformed or unknown input</t>
+        </is>
+      </c>
+      <c r="D77" s="7" t="inlineStr">
+        <is>
+          <t>The buyer can send reminders to vendors who still have to act. Sending reminders without the list of recipients, with the recipients written as text, with an unknown reminder type, or for an event that does not exist crashes the server instead of refusing.</t>
+        </is>
+      </c>
+      <c r="E77" s="7" t="inlineStr">
+        <is>
+          <t>1. Send reminders for an event without saying who should get them (or with an unknown reminder type, or for an event that does not exist).</t>
+        </is>
+      </c>
+      <c r="F77" s="7" t="inlineStr">
+        <is>
+          <t>A clear refusal or 'not found'.</t>
+        </is>
+      </c>
+      <c r="G77" s="7" t="inlineStr">
+        <is>
+          <t>The server crashes.</t>
+        </is>
+      </c>
+      <c r="H77" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I77" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J77" s="7" t="inlineStr">
+        <is>
+          <t>Server crash</t>
+        </is>
+      </c>
+      <c r="K77" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on PROCOL DEMO on 3–4 Oct 2026: each variant failed the same way on two fresh test events. (reminders_controller.rb; reminders/base_service.rb:40).</t>
+        </is>
+      </c>
+      <c r="L77" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M77" s="7" t="inlineStr">
+        <is>
+          <t>API-EVDREM-019, API-EVDREM-020, API-EVDREM-024, API-EVDREM-048, API-EVDREM-049, API-EVDREM-050, API-EVDREM-051, API-EVDREM-052, API-EVDREM-057, API-EVDREM-058, API-EVDREM-059</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="7" t="inlineStr">
+        <is>
+          <t>BUG-77</t>
+        </is>
+      </c>
+      <c r="B78" s="7" t="inlineStr">
+        <is>
+          <t>Documents</t>
+        </is>
+      </c>
+      <c r="C78" s="7" t="inlineStr">
+        <is>
+          <t>Malformed attachments on a round or a surrogate bid crash, and the attachment link crashes without a token</t>
+        </is>
+      </c>
+      <c r="D78" s="7" t="inlineStr">
+        <is>
+          <t>Sending a round's attachments in the wrong shape, or a bid entered on a vendor's behalf with a reference note but no files, crashes the server. The attachment-link address also crashes when it is called without a token instead of refusing.</t>
+        </is>
+      </c>
+      <c r="E78" s="7" t="inlineStr">
+        <is>
+          <t>1. Update a round with attachments in the wrong shape (or enter a surrogate bid with a note and no files).
+2. Or open an attachment link without its token.</t>
+        </is>
+      </c>
+      <c r="F78" s="7" t="inlineStr">
+        <is>
+          <t>A clear refusal.</t>
+        </is>
+      </c>
+      <c r="G78" s="7" t="inlineStr">
+        <is>
+          <t>The server crashes.</t>
+        </is>
+      </c>
+      <c r="H78" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO; Demo Account 2</t>
+        </is>
+      </c>
+      <c r="I78" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J78" s="7" t="inlineStr">
+        <is>
+          <t>Server crash</t>
+        </is>
+      </c>
+      <c r="K78" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on two fresh test events per variant; the attachment-link variant on both clients (trade_controller.rb:459; v1/attachments_controller.rb:12-18).</t>
+        </is>
+      </c>
+      <c r="L78" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M78" s="7" t="inlineStr">
+        <is>
+          <t>API-EVDDOC-034, API-EVDDOC-039, API-EVDDOC-054, API-EVDDOC-055, API-EVDDOC-061, API-EVDDOC-062</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="7" t="inlineStr">
+        <is>
+          <t>BUG-78</t>
+        </is>
+      </c>
+      <c r="B79" s="7" t="inlineStr">
+        <is>
+          <t>Weighted bidding</t>
+        </is>
+      </c>
+      <c r="C79" s="7" t="inlineStr">
+        <is>
+          <t>Saving malformed weights crashes</t>
+        </is>
+      </c>
+      <c r="D79" s="7" t="inlineStr">
+        <is>
+          <t>Saving vendor weights in the wrong shape (for example text where a number belongs) crashes the server instead of refusing the weights.</t>
+        </is>
+      </c>
+      <c r="E79" s="7" t="inlineStr">
+        <is>
+          <t>1. On a round with weighted bidding, save the weights with a value in the wrong shape.</t>
+        </is>
+      </c>
+      <c r="F79" s="7" t="inlineStr">
+        <is>
+          <t>A clear refusal naming the bad weight.</t>
+        </is>
+      </c>
+      <c r="G79" s="7" t="inlineStr">
+        <is>
+          <t>The server crashes.</t>
+        </is>
+      </c>
+      <c r="H79" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I79" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J79" s="7" t="inlineStr">
+        <is>
+          <t>Server crash</t>
+        </is>
+      </c>
+      <c r="K79" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on PROCOL DEMO on 3–4 Oct 2026: each variant failed the same way on two fresh test events. (trade_controller.rb:1779,1804).</t>
+        </is>
+      </c>
+      <c r="L79" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M79" s="7" t="inlineStr">
+        <is>
+          <t>API-EVDWGT-047, API-EVDWGT-048, API-EVDWGT-050, API-EVDWGT-051, API-EVDWGT-052, API-EVDWGT-053</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="7" t="inlineStr">
+        <is>
+          <t>BUG-79</t>
+        </is>
+      </c>
+      <c r="B80" s="7" t="inlineStr">
+        <is>
+          <t>Event update</t>
+        </is>
+      </c>
+      <c r="C80" s="7" t="inlineStr">
+        <is>
+          <t>Sending an empty value for any list of ids crashes the server</t>
+        </is>
+      </c>
+      <c r="D80" s="7" t="inlineStr">
+        <is>
+          <t>Many requests carry lists of ids (for example the line items to reopen). Sending an empty value instead of a list for any such field crashes the server before the request is even looked at, because a shared check does not expect it.</t>
+        </is>
+      </c>
+      <c r="E80" s="7" t="inlineStr">
+        <is>
+          <t>1. Reopen line items on a round with the list of line items sent as an empty value.</t>
+        </is>
+      </c>
+      <c r="F80" s="7" t="inlineStr">
+        <is>
+          <t>A clear refusal, or the request treated as an empty list.</t>
+        </is>
+      </c>
+      <c r="G80" s="7" t="inlineStr">
+        <is>
+          <t>The server crashes.</t>
+        </is>
+      </c>
+      <c r="H80" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I80" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J80" s="7" t="inlineStr">
+        <is>
+          <t>Server crash</t>
+        </is>
+      </c>
+      <c r="K80" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on PROCOL DEMO on 3–4 Oct 2026: each variant failed the same way on two fresh test events. (params_auth.rb:70-73 — applies to every such field).</t>
+        </is>
+      </c>
+      <c r="L80" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M80" s="7" t="inlineStr">
+        <is>
+          <t>API-EVDTME-054</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rule coverage: 100 cases for untested calculation, visibility and bid/award rules; bug sheet 81
- events-rules-cal/vis/mbp.md (API-EVR*), each citing its rule's file:line; 11 runnable twins.
  Coverage of 3,713 cited rules: covered 1,523 -> 1,814; CAL 56 -> 152, VIS 92 -> 180, MBP 54 -> 145.
  43 rules recorded as not checkable through the API or screens, with the reason.
- Case runner may now read bid details and post a chat message on the sandbox round; a mention
  only ever names the signed-in buyer (a mention notifies a person).
- 2 new verified defects (bid details before a bid crash; a double mention refused). Memory eval
  grows to 115 questions (hit@1 76.5% with the 30 harder new ones).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
+++ b/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
@@ -221,8 +221,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:M80" headerRowCount="1">
-  <autoFilter ref="A1:M80"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:M82" headerRowCount="1">
+  <autoFilter ref="A1:M82"/>
   <tableColumns count="13">
     <tableColumn id="1" name="Bug #"/>
     <tableColumn id="2" name="Area"/>
@@ -590,7 +590,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>COUNTA(Bugs!A2:A80)</f>
+        <f>COUNTA(Bugs!A2:A82)</f>
         <v/>
       </c>
     </row>
@@ -609,7 +609,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF(Bugs!I2:I80,A7)</f>
+        <f>COUNTIF(Bugs!I2:I82,A7)</f>
         <v/>
       </c>
     </row>
@@ -620,7 +620,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF(Bugs!I2:I80,A8)</f>
+        <f>COUNTIF(Bugs!I2:I82,A8)</f>
         <v/>
       </c>
     </row>
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIF(Bugs!I2:I80,A9)</f>
+        <f>COUNTIF(Bugs!I2:I82,A9)</f>
         <v/>
       </c>
     </row>
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIF(Bugs!I2:I80,A10)</f>
+        <f>COUNTIF(Bugs!I2:I82,A10)</f>
         <v/>
       </c>
     </row>
@@ -661,7 +661,7 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF(Bugs!J2:J80,A13)</f>
+        <f>COUNTIF(Bugs!J2:J82,A13)</f>
         <v/>
       </c>
     </row>
@@ -672,7 +672,7 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF(Bugs!J2:J80,A14)</f>
+        <f>COUNTIF(Bugs!J2:J82,A14)</f>
         <v/>
       </c>
     </row>
@@ -683,7 +683,7 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF(Bugs!J2:J80,A15)</f>
+        <f>COUNTIF(Bugs!J2:J82,A15)</f>
         <v/>
       </c>
     </row>
@@ -694,7 +694,7 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF(Bugs!J2:J80,A16)</f>
+        <f>COUNTIF(Bugs!J2:J82,A16)</f>
         <v/>
       </c>
     </row>
@@ -705,7 +705,7 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF(Bugs!J2:J80,A17)</f>
+        <f>COUNTIF(Bugs!J2:J82,A17)</f>
         <v/>
       </c>
     </row>
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF(Bugs!J2:J80,A18)</f>
+        <f>COUNTIF(Bugs!J2:J82,A18)</f>
         <v/>
       </c>
     </row>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF(Bugs!J2:J80,A19)</f>
+        <f>COUNTIF(Bugs!J2:J82,A19)</f>
         <v/>
       </c>
     </row>
@@ -738,7 +738,7 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF(Bugs!J2:J80,A20)</f>
+        <f>COUNTIF(Bugs!J2:J82,A20)</f>
         <v/>
       </c>
     </row>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF(Bugs!J2:J80,A21)</f>
+        <f>COUNTIF(Bugs!J2:J82,A21)</f>
         <v/>
       </c>
     </row>
@@ -760,7 +760,7 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF(Bugs!J2:J80,A22)</f>
+        <f>COUNTIF(Bugs!J2:J82,A22)</f>
         <v/>
       </c>
     </row>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B25" s="5">
-        <f>COUNTIF(Bugs!H2:H80,"*"&amp;A25&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H82,"*"&amp;A25&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF(Bugs!H2:H80,"*"&amp;A26&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H82,"*"&amp;A26&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -801,7 +801,7 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF(Bugs!H2:H80,"*"&amp;A27&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H82,"*"&amp;A27&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -849,7 +849,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M80"/>
+  <dimension ref="A1:M82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -6125,6 +6125,141 @@
       <c r="M80" s="7" t="inlineStr">
         <is>
           <t>API-EVDTME-054</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="7" t="inlineStr">
+        <is>
+          <t>BUG-80</t>
+        </is>
+      </c>
+      <c r="B81" s="7" t="inlineStr">
+        <is>
+          <t>Bidding &amp; vendor permissions</t>
+        </is>
+      </c>
+      <c r="C81" s="7" t="inlineStr">
+        <is>
+          <t>Opening a vendor's bid details before that vendor has bid crashes the server</t>
+        </is>
+      </c>
+      <c r="D81" s="7" t="inlineStr">
+        <is>
+          <t>The buyer can open the details of a vendor's bid on a round. If that vendor has not bid yet, the server crashes instead of answering that there is no bid, because it tries to read a bid that does not exist.</t>
+        </is>
+      </c>
+      <c r="E81" s="7" t="inlineStr">
+        <is>
+          <t>1. Publish a round and invite a QA vendor.
+2. Before the vendor bids, open that vendor's bid details as the buyer.</t>
+        </is>
+      </c>
+      <c r="F81" s="7" t="inlineStr">
+        <is>
+          <t>A clear 'Bid not found' answer.</t>
+        </is>
+      </c>
+      <c r="G81" s="7" t="inlineStr">
+        <is>
+          <t>The server crashes.</t>
+        </is>
+      </c>
+      <c r="H81" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I81" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J81" s="7" t="inlineStr">
+        <is>
+          <t>Server crash</t>
+        </is>
+      </c>
+      <c r="K81" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on two fresh test events on PROCOL DEMO (bids_controller.rb:370-386).</t>
+        </is>
+      </c>
+      <c r="L81" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M81" s="7" t="inlineStr">
+        <is>
+          <t>API-EVRVIS-025</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="7" t="inlineStr">
+        <is>
+          <t>BUG-81</t>
+        </is>
+      </c>
+      <c r="B82" s="7" t="inlineStr">
+        <is>
+          <t>Clarifications</t>
+        </is>
+      </c>
+      <c r="C82" s="7" t="inlineStr">
+        <is>
+          <t>A chat message that mentions the same colleague twice is refused as 'not allowed'</t>
+        </is>
+      </c>
+      <c r="D82" s="7" t="inlineStr">
+        <is>
+          <t>In a round's chat a buyer can mention colleagues. Mentioning the same person twice in one message is refused with 'You are not allowed to perform this action', although mentioning them once, or sending a plain message, works. The check compares the list of mentioned people with a copy that has the duplicates removed.</t>
+        </is>
+      </c>
+      <c r="E82" s="7" t="inlineStr">
+        <is>
+          <t>1. On a live round, post a chat message that mentions the same colleague twice.</t>
+        </is>
+      </c>
+      <c r="F82" s="7" t="inlineStr">
+        <is>
+          <t>The message is posted (the person is notified once).</t>
+        </is>
+      </c>
+      <c r="G82" s="7" t="inlineStr">
+        <is>
+          <t>Refused: 'You are not allowed to perform this action'.</t>
+        </is>
+      </c>
+      <c r="H82" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I82" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J82" s="7" t="inlineStr">
+        <is>
+          <t>Wrong message</t>
+        </is>
+      </c>
+      <c r="K82" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on two fresh test events on PROCOL DEMO (expression_evaluator_service.rb:30-33).</t>
+        </is>
+      </c>
+      <c r="L82" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M82" s="7" t="inlineStr">
+        <is>
+          <t>API-EVRCAL-035</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rule coverage cases; bug sheet 81
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
+++ b/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
@@ -221,8 +221,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:M80" headerRowCount="1">
-  <autoFilter ref="A1:M80"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:M82" headerRowCount="1">
+  <autoFilter ref="A1:M82"/>
   <tableColumns count="13">
     <tableColumn id="1" name="Bug #"/>
     <tableColumn id="2" name="Area"/>
@@ -590,7 +590,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>COUNTA(Bugs!A2:A80)</f>
+        <f>COUNTA(Bugs!A2:A82)</f>
         <v/>
       </c>
     </row>
@@ -609,7 +609,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF(Bugs!I2:I80,A7)</f>
+        <f>COUNTIF(Bugs!I2:I82,A7)</f>
         <v/>
       </c>
     </row>
@@ -620,7 +620,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF(Bugs!I2:I80,A8)</f>
+        <f>COUNTIF(Bugs!I2:I82,A8)</f>
         <v/>
       </c>
     </row>
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIF(Bugs!I2:I80,A9)</f>
+        <f>COUNTIF(Bugs!I2:I82,A9)</f>
         <v/>
       </c>
     </row>
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIF(Bugs!I2:I80,A10)</f>
+        <f>COUNTIF(Bugs!I2:I82,A10)</f>
         <v/>
       </c>
     </row>
@@ -661,7 +661,7 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF(Bugs!J2:J80,A13)</f>
+        <f>COUNTIF(Bugs!J2:J82,A13)</f>
         <v/>
       </c>
     </row>
@@ -672,7 +672,7 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF(Bugs!J2:J80,A14)</f>
+        <f>COUNTIF(Bugs!J2:J82,A14)</f>
         <v/>
       </c>
     </row>
@@ -683,7 +683,7 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF(Bugs!J2:J80,A15)</f>
+        <f>COUNTIF(Bugs!J2:J82,A15)</f>
         <v/>
       </c>
     </row>
@@ -694,7 +694,7 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF(Bugs!J2:J80,A16)</f>
+        <f>COUNTIF(Bugs!J2:J82,A16)</f>
         <v/>
       </c>
     </row>
@@ -705,7 +705,7 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF(Bugs!J2:J80,A17)</f>
+        <f>COUNTIF(Bugs!J2:J82,A17)</f>
         <v/>
       </c>
     </row>
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF(Bugs!J2:J80,A18)</f>
+        <f>COUNTIF(Bugs!J2:J82,A18)</f>
         <v/>
       </c>
     </row>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF(Bugs!J2:J80,A19)</f>
+        <f>COUNTIF(Bugs!J2:J82,A19)</f>
         <v/>
       </c>
     </row>
@@ -738,7 +738,7 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF(Bugs!J2:J80,A20)</f>
+        <f>COUNTIF(Bugs!J2:J82,A20)</f>
         <v/>
       </c>
     </row>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF(Bugs!J2:J80,A21)</f>
+        <f>COUNTIF(Bugs!J2:J82,A21)</f>
         <v/>
       </c>
     </row>
@@ -760,7 +760,7 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF(Bugs!J2:J80,A22)</f>
+        <f>COUNTIF(Bugs!J2:J82,A22)</f>
         <v/>
       </c>
     </row>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B25" s="5">
-        <f>COUNTIF(Bugs!H2:H80,"*"&amp;A25&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H82,"*"&amp;A25&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF(Bugs!H2:H80,"*"&amp;A26&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H82,"*"&amp;A26&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -801,7 +801,7 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF(Bugs!H2:H80,"*"&amp;A27&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H82,"*"&amp;A27&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -849,7 +849,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M80"/>
+  <dimension ref="A1:M82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -6125,6 +6125,141 @@
       <c r="M80" s="7" t="inlineStr">
         <is>
           <t>API-EVDTME-054</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="7" t="inlineStr">
+        <is>
+          <t>BUG-80</t>
+        </is>
+      </c>
+      <c r="B81" s="7" t="inlineStr">
+        <is>
+          <t>Bidding &amp; vendor permissions</t>
+        </is>
+      </c>
+      <c r="C81" s="7" t="inlineStr">
+        <is>
+          <t>Opening a vendor's bid details before that vendor has bid crashes the server</t>
+        </is>
+      </c>
+      <c r="D81" s="7" t="inlineStr">
+        <is>
+          <t>The buyer can open the details of a vendor's bid on a round. If that vendor has not bid yet, the server crashes instead of answering that there is no bid, because it tries to read a bid that does not exist.</t>
+        </is>
+      </c>
+      <c r="E81" s="7" t="inlineStr">
+        <is>
+          <t>1. Publish a round and invite a QA vendor.
+2. Before the vendor bids, open that vendor's bid details as the buyer.</t>
+        </is>
+      </c>
+      <c r="F81" s="7" t="inlineStr">
+        <is>
+          <t>A clear 'Bid not found' answer.</t>
+        </is>
+      </c>
+      <c r="G81" s="7" t="inlineStr">
+        <is>
+          <t>The server crashes.</t>
+        </is>
+      </c>
+      <c r="H81" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I81" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J81" s="7" t="inlineStr">
+        <is>
+          <t>Server crash</t>
+        </is>
+      </c>
+      <c r="K81" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on two fresh test events on PROCOL DEMO (bids_controller.rb:370-386).</t>
+        </is>
+      </c>
+      <c r="L81" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M81" s="7" t="inlineStr">
+        <is>
+          <t>API-EVRVIS-025</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="7" t="inlineStr">
+        <is>
+          <t>BUG-81</t>
+        </is>
+      </c>
+      <c r="B82" s="7" t="inlineStr">
+        <is>
+          <t>Clarifications</t>
+        </is>
+      </c>
+      <c r="C82" s="7" t="inlineStr">
+        <is>
+          <t>A chat message that mentions the same colleague twice is refused as 'not allowed'</t>
+        </is>
+      </c>
+      <c r="D82" s="7" t="inlineStr">
+        <is>
+          <t>In a round's chat a buyer can mention colleagues. Mentioning the same person twice in one message is refused with 'You are not allowed to perform this action', although mentioning them once, or sending a plain message, works. The check compares the list of mentioned people with a copy that has the duplicates removed.</t>
+        </is>
+      </c>
+      <c r="E82" s="7" t="inlineStr">
+        <is>
+          <t>1. On a live round, post a chat message that mentions the same colleague twice.</t>
+        </is>
+      </c>
+      <c r="F82" s="7" t="inlineStr">
+        <is>
+          <t>The message is posted (the person is notified once).</t>
+        </is>
+      </c>
+      <c r="G82" s="7" t="inlineStr">
+        <is>
+          <t>Refused: 'You are not allowed to perform this action'.</t>
+        </is>
+      </c>
+      <c r="H82" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I82" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J82" s="7" t="inlineStr">
+        <is>
+          <t>Wrong message</t>
+        </is>
+      </c>
+      <c r="K82" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on two fresh test events on PROCOL DEMO (expression_evaluator_service.rb:30-33).</t>
+        </is>
+      </c>
+      <c r="L82" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M82" s="7" t="inlineStr">
+        <is>
+          <t>API-EVRCAL-035</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bug sheet: three round-2 bugs reproduced on Demo Account 2 too (competitor weights visible, malformed weights crash, empty id list crash)
Round 2 on Demo Account 2 finished: 122 passed, 9 failed (all known bugs, now on both clients),
5 couldn't tell. A script-like weight name answered 403 on both clients: a security filter, not a bug.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
+++ b/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
@@ -5420,7 +5420,7 @@
       </c>
       <c r="H70" s="7" t="inlineStr">
         <is>
-          <t>PROCOL DEMO</t>
+          <t>PROCOL DEMO; Demo Account 2</t>
         </is>
       </c>
       <c r="I70" s="9" t="inlineStr">
@@ -5435,7 +5435,7 @@
       </c>
       <c r="K70" s="7" t="inlineStr">
         <is>
-          <t>Reproduced on PROCOL DEMO on 3–4 Oct 2026: each variant failed the same way on two fresh test events. Cause: trade_template_serializer.rb:877-879 sends every vendor's weights.</t>
+          <t>Reproduced on PROCOL DEMO on 3–4 Oct 2026: each variant failed the same way on two fresh test events. Cause: trade_template_serializer.rb:877-879 sends every vendor's weights. Also reproduced on Demo Account 2 (4 Oct 2026, two fresh test events).</t>
         </is>
       </c>
       <c r="L70" s="7" t="inlineStr">
@@ -6032,7 +6032,7 @@
       </c>
       <c r="H79" s="7" t="inlineStr">
         <is>
-          <t>PROCOL DEMO</t>
+          <t>PROCOL DEMO; Demo Account 2</t>
         </is>
       </c>
       <c r="I79" s="11" t="inlineStr">
@@ -6047,7 +6047,7 @@
       </c>
       <c r="K79" s="7" t="inlineStr">
         <is>
-          <t>Reproduced on PROCOL DEMO on 3–4 Oct 2026: each variant failed the same way on two fresh test events. (trade_controller.rb:1779,1804).</t>
+          <t>Reproduced on PROCOL DEMO on 3–4 Oct 2026: each variant failed the same way on two fresh test events. (trade_controller.rb:1779,1804). Also reproduced on Demo Account 2 (6 variants, two fresh test events each).</t>
         </is>
       </c>
       <c r="L79" s="7" t="inlineStr">
@@ -6099,7 +6099,7 @@
       </c>
       <c r="H80" s="7" t="inlineStr">
         <is>
-          <t>PROCOL DEMO</t>
+          <t>PROCOL DEMO; Demo Account 2</t>
         </is>
       </c>
       <c r="I80" s="10" t="inlineStr">
@@ -6114,7 +6114,7 @@
       </c>
       <c r="K80" s="7" t="inlineStr">
         <is>
-          <t>Reproduced on PROCOL DEMO on 3–4 Oct 2026: each variant failed the same way on two fresh test events. (params_auth.rb:70-73 — applies to every such field).</t>
+          <t>Reproduced on PROCOL DEMO on 3–4 Oct 2026: each variant failed the same way on two fresh test events. (params_auth.rb:70-73 — applies to every such field). Also reproduced on Demo Account 2 (two fresh test events).</t>
         </is>
       </c>
       <c r="L80" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Bug sheet: three bugs confirmed on both clients; UI automation design
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
+++ b/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
@@ -5420,7 +5420,7 @@
       </c>
       <c r="H70" s="7" t="inlineStr">
         <is>
-          <t>PROCOL DEMO</t>
+          <t>PROCOL DEMO; Demo Account 2</t>
         </is>
       </c>
       <c r="I70" s="9" t="inlineStr">
@@ -5435,7 +5435,7 @@
       </c>
       <c r="K70" s="7" t="inlineStr">
         <is>
-          <t>Reproduced on PROCOL DEMO on 3–4 Oct 2026: each variant failed the same way on two fresh test events. Cause: trade_template_serializer.rb:877-879 sends every vendor's weights.</t>
+          <t>Reproduced on PROCOL DEMO on 3–4 Oct 2026: each variant failed the same way on two fresh test events. Cause: trade_template_serializer.rb:877-879 sends every vendor's weights. Also reproduced on Demo Account 2 (4 Oct 2026, two fresh test events).</t>
         </is>
       </c>
       <c r="L70" s="7" t="inlineStr">
@@ -6032,7 +6032,7 @@
       </c>
       <c r="H79" s="7" t="inlineStr">
         <is>
-          <t>PROCOL DEMO</t>
+          <t>PROCOL DEMO; Demo Account 2</t>
         </is>
       </c>
       <c r="I79" s="11" t="inlineStr">
@@ -6047,7 +6047,7 @@
       </c>
       <c r="K79" s="7" t="inlineStr">
         <is>
-          <t>Reproduced on PROCOL DEMO on 3–4 Oct 2026: each variant failed the same way on two fresh test events. (trade_controller.rb:1779,1804).</t>
+          <t>Reproduced on PROCOL DEMO on 3–4 Oct 2026: each variant failed the same way on two fresh test events. (trade_controller.rb:1779,1804). Also reproduced on Demo Account 2 (6 variants, two fresh test events each).</t>
         </is>
       </c>
       <c r="L79" s="7" t="inlineStr">
@@ -6099,7 +6099,7 @@
       </c>
       <c r="H80" s="7" t="inlineStr">
         <is>
-          <t>PROCOL DEMO</t>
+          <t>PROCOL DEMO; Demo Account 2</t>
         </is>
       </c>
       <c r="I80" s="10" t="inlineStr">
@@ -6114,7 +6114,7 @@
       </c>
       <c r="K80" s="7" t="inlineStr">
         <is>
-          <t>Reproduced on PROCOL DEMO on 3–4 Oct 2026: each variant failed the same way on two fresh test events. (params_auth.rb:70-73 — applies to every such field).</t>
+          <t>Reproduced on PROCOL DEMO on 3–4 Oct 2026: each variant failed the same way on two fresh test events. (params_auth.rb:70-73 — applies to every such field). Also reproduced on Demo Account 2 (two fresh test events).</t>
         </is>
       </c>
       <c r="L80" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Bug sheet 82: an amendment starts every copied window now, so evaluation ends before bidding closes (reproduced twice); repro script
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
+++ b/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
@@ -221,8 +221,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:M82" headerRowCount="1">
-  <autoFilter ref="A1:M82"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:M83" headerRowCount="1">
+  <autoFilter ref="A1:M83"/>
   <tableColumns count="13">
     <tableColumn id="1" name="Bug #"/>
     <tableColumn id="2" name="Area"/>
@@ -590,7 +590,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>COUNTA(Bugs!A2:A82)</f>
+        <f>COUNTA(Bugs!A2:A83)</f>
         <v/>
       </c>
     </row>
@@ -609,7 +609,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF(Bugs!I2:I82,A7)</f>
+        <f>COUNTIF(Bugs!I2:I83,A7)</f>
         <v/>
       </c>
     </row>
@@ -620,7 +620,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF(Bugs!I2:I82,A8)</f>
+        <f>COUNTIF(Bugs!I2:I83,A8)</f>
         <v/>
       </c>
     </row>
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIF(Bugs!I2:I82,A9)</f>
+        <f>COUNTIF(Bugs!I2:I83,A9)</f>
         <v/>
       </c>
     </row>
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIF(Bugs!I2:I82,A10)</f>
+        <f>COUNTIF(Bugs!I2:I83,A10)</f>
         <v/>
       </c>
     </row>
@@ -661,7 +661,7 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF(Bugs!J2:J82,A13)</f>
+        <f>COUNTIF(Bugs!J2:J83,A13)</f>
         <v/>
       </c>
     </row>
@@ -672,7 +672,7 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF(Bugs!J2:J82,A14)</f>
+        <f>COUNTIF(Bugs!J2:J83,A14)</f>
         <v/>
       </c>
     </row>
@@ -683,7 +683,7 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF(Bugs!J2:J82,A15)</f>
+        <f>COUNTIF(Bugs!J2:J83,A15)</f>
         <v/>
       </c>
     </row>
@@ -694,7 +694,7 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF(Bugs!J2:J82,A16)</f>
+        <f>COUNTIF(Bugs!J2:J83,A16)</f>
         <v/>
       </c>
     </row>
@@ -705,7 +705,7 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF(Bugs!J2:J82,A17)</f>
+        <f>COUNTIF(Bugs!J2:J83,A17)</f>
         <v/>
       </c>
     </row>
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF(Bugs!J2:J82,A18)</f>
+        <f>COUNTIF(Bugs!J2:J83,A18)</f>
         <v/>
       </c>
     </row>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF(Bugs!J2:J82,A19)</f>
+        <f>COUNTIF(Bugs!J2:J83,A19)</f>
         <v/>
       </c>
     </row>
@@ -738,7 +738,7 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF(Bugs!J2:J82,A20)</f>
+        <f>COUNTIF(Bugs!J2:J83,A20)</f>
         <v/>
       </c>
     </row>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF(Bugs!J2:J82,A21)</f>
+        <f>COUNTIF(Bugs!J2:J83,A21)</f>
         <v/>
       </c>
     </row>
@@ -760,7 +760,7 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF(Bugs!J2:J82,A22)</f>
+        <f>COUNTIF(Bugs!J2:J83,A22)</f>
         <v/>
       </c>
     </row>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B25" s="5">
-        <f>COUNTIF(Bugs!H2:H82,"*"&amp;A25&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H83,"*"&amp;A25&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF(Bugs!H2:H82,"*"&amp;A26&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H83,"*"&amp;A26&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -801,7 +801,7 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF(Bugs!H2:H82,"*"&amp;A27&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H83,"*"&amp;A27&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -849,7 +849,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M82"/>
+  <dimension ref="A1:M83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -6260,6 +6260,75 @@
       <c r="M82" s="7" t="inlineStr">
         <is>
           <t>API-EVRCAL-035</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="7" t="inlineStr">
+        <is>
+          <t>BUG-82</t>
+        </is>
+      </c>
+      <c r="B83" s="7" t="inlineStr">
+        <is>
+          <t>Amending a live event</t>
+        </is>
+      </c>
+      <c r="C83" s="7" t="inlineStr">
+        <is>
+          <t>After an amendment, the evaluation window starts and ends before bidding has even closed</t>
+        </is>
+      </c>
+      <c r="D83" s="7" t="inlineStr">
+        <is>
+          <t>A technical round has a bidding window and then an evaluation window that starts when bidding ends. When the buyer issues an amendment (a new version of the event), Procol copies every window of the round but starts all of them at the moment of the amendment. The evaluation window therefore opens together with bidding and, being short, is already over long before bidding closes — so evaluators have no window left once the bids are in.</t>
+        </is>
+      </c>
+      <c r="E83" s="7" t="inlineStr">
+        <is>
+          <t>1. Publish an event with a technical round (bidding 10 minutes, then a short evaluation window).
+2. Issue an amendment (a new version of the event).
+3. Read the amended round's bidding and evaluation windows.</t>
+        </is>
+      </c>
+      <c r="F83" s="7" t="inlineStr">
+        <is>
+          <t>Bidding runs from the amendment for its configured length, and evaluation starts when bidding ends — as on the original event.</t>
+        </is>
+      </c>
+      <c r="G83" s="7" t="inlineStr">
+        <is>
+          <t>Both windows start at the moment of the amendment: bidding 06:32:27 → 06:42:27, evaluation 06:32:27 → 06:32:32 (over ten minutes before bidding closes).</t>
+        </is>
+      </c>
+      <c r="H83" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I83" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J83" s="7" t="inlineStr">
+        <is>
+          <t>Business rule</t>
+        </is>
+      </c>
+      <c r="K83" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on two fresh test events on PROCOL DEMO (4 Oct 2026), read from the amended round's stored windows; on each original event evaluation correctly started when bidding ended. Cause: versions/trade_request.rb replicate_trade_schedules sets every copied window to start now. Whether publishing the amendment re-times the windows was not checked.</t>
+        </is>
+      </c>
+      <c r="L83" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M83" s="7" t="inlineStr">
+        <is>
+          <t>API-EVRMEG-024, API-EVRLIF-014</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Needs confirmation: an RFI round may close on its first evaluation (code-confirmed, not yet reproduced live)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
+++ b/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Confirm" displayName="Confirm" ref="A1:F10" headerRowCount="1">
-  <autoFilter ref="A1:F10"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Confirm" displayName="Confirm" ref="A1:F11" headerRowCount="1">
+  <autoFilter ref="A1:F11"/>
   <tableColumns count="6">
     <tableColumn id="1" name="#"/>
     <tableColumn id="2" name="Area"/>
@@ -820,7 +820,7 @@
         </is>
       </c>
       <c r="B30" s="5">
-        <f>COUNTA('Needs confirmation'!A2:A10)</f>
+        <f>COUNTA('Needs confirmation'!A2:A11)</f>
         <v/>
       </c>
     </row>
@@ -6346,7 +6346,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -6674,6 +6674,38 @@
       <c r="F10" s="7" t="inlineStr">
         <is>
           <t>Confirm in the screen's code whether an older list response can overwrite the search result (a race between the first load and the search). It is intermittent, so it is not yet counted as a verified bug.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Q-10</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Technical evaluation</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>An information-request (RFI) round may close as soon as the first vendor is evaluated</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>In Procol's code, saving any evaluation on an RFI round closes the whole round, because the round counts as 'evaluated' as soon as one evaluation exists (models/evaluation.rb close_trade_request; trade_request_model_helper.rb is_evaluated? for RFI). Vendors not yet evaluated would then meet a closed round. Read in the code only: our runner does not yet build RFI rounds, so it has not been reproduced live.</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>Reproduce on an RFI round with two or more responding vendors, or confirm with the product team whether one evaluation is meant to close an RFI.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bug sheet 83: a rescheduled start comes back shifted by the browser↔server clock gap (dialog saves the browser time unshifted; the screen shows server time + timeDiff) — reproduced on 4 fresh events, Low
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
+++ b/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
@@ -583,6 +583,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -590,7 +591,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>COUNTA(Bugs!A2:A83)</f>
+        <f>COUNTA(Bugs!A2:A84)</f>
         <v/>
       </c>
     </row>
@@ -609,7 +610,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF(Bugs!I2:I83,A7)</f>
+        <f>COUNTIF(Bugs!I2:I84,A7)</f>
         <v/>
       </c>
     </row>
@@ -620,7 +621,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF(Bugs!I2:I83,A8)</f>
+        <f>COUNTIF(Bugs!I2:I84,A8)</f>
         <v/>
       </c>
     </row>
@@ -631,7 +632,7 @@
         </is>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIF(Bugs!I2:I83,A9)</f>
+        <f>COUNTIF(Bugs!I2:I84,A9)</f>
         <v/>
       </c>
     </row>
@@ -642,7 +643,7 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIF(Bugs!I2:I83,A10)</f>
+        <f>COUNTIF(Bugs!I2:I84,A10)</f>
         <v/>
       </c>
     </row>
@@ -661,7 +662,7 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF(Bugs!J2:J83,A13)</f>
+        <f>COUNTIF(Bugs!J2:J84,A13)</f>
         <v/>
       </c>
     </row>
@@ -672,7 +673,7 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF(Bugs!J2:J83,A14)</f>
+        <f>COUNTIF(Bugs!J2:J84,A14)</f>
         <v/>
       </c>
     </row>
@@ -683,7 +684,7 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF(Bugs!J2:J83,A15)</f>
+        <f>COUNTIF(Bugs!J2:J84,A15)</f>
         <v/>
       </c>
     </row>
@@ -694,7 +695,7 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF(Bugs!J2:J83,A16)</f>
+        <f>COUNTIF(Bugs!J2:J84,A16)</f>
         <v/>
       </c>
     </row>
@@ -705,7 +706,7 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF(Bugs!J2:J83,A17)</f>
+        <f>COUNTIF(Bugs!J2:J84,A17)</f>
         <v/>
       </c>
     </row>
@@ -716,7 +717,7 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF(Bugs!J2:J83,A18)</f>
+        <f>COUNTIF(Bugs!J2:J84,A18)</f>
         <v/>
       </c>
     </row>
@@ -727,7 +728,7 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF(Bugs!J2:J83,A19)</f>
+        <f>COUNTIF(Bugs!J2:J84,A19)</f>
         <v/>
       </c>
     </row>
@@ -738,7 +739,7 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF(Bugs!J2:J83,A20)</f>
+        <f>COUNTIF(Bugs!J2:J84,A20)</f>
         <v/>
       </c>
     </row>
@@ -749,7 +750,7 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF(Bugs!J2:J83,A21)</f>
+        <f>COUNTIF(Bugs!J2:J84,A21)</f>
         <v/>
       </c>
     </row>
@@ -760,7 +761,7 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF(Bugs!J2:J83,A22)</f>
+        <f>COUNTIF(Bugs!J2:J84,A22)</f>
         <v/>
       </c>
     </row>
@@ -779,7 +780,7 @@
         </is>
       </c>
       <c r="B25" s="5">
-        <f>COUNTIF(Bugs!H2:H83,"*"&amp;A25&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H84,"*"&amp;A25&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -790,7 +791,7 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF(Bugs!H2:H83,"*"&amp;A26&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H84,"*"&amp;A26&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -801,7 +802,7 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF(Bugs!H2:H83,"*"&amp;A27&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H84,"*"&amp;A27&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -849,7 +850,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M83"/>
+  <dimension ref="A1:M84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -6329,6 +6330,76 @@
       <c r="M83" s="7" t="inlineStr">
         <is>
           <t>API-EVRMEG-024, API-EVRLIF-014</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="7" t="inlineStr">
+        <is>
+          <t>BUG-83</t>
+        </is>
+      </c>
+      <c r="B84" s="7" t="inlineStr">
+        <is>
+          <t>Scheduling &amp; rescheduling</t>
+        </is>
+      </c>
+      <c r="C84" s="7" t="inlineStr">
+        <is>
+          <t>A rescheduled start comes back a minute earlier than the buyer picked</t>
+        </is>
+      </c>
+      <c r="D84" s="7" t="inlineStr">
+        <is>
+          <t>The event screen shows every time adjusted for the gap between the buyer's computer clock and Procol's server clock, but the Reschedule dialog saves the picked time without that adjustment. Whenever the two clocks differ, the saved start is off by that gap and the screen then shows a different time from the one the buyer chose. On UAT the browser was 1 second behind the server, so 2:30 pm came back as 2:29 pm.</t>
+        </is>
+      </c>
+      <c r="E84" s="7" t="inlineStr">
+        <is>
+          <t>1. Publish an event that starts later (upcoming).
+2. Event Settings → Reschedule Event.
+3. Pick a new start, e.g. 2:30 pm, and press Ok.
+4. Open Reschedule Event again (or look at the event's start time).</t>
+        </is>
+      </c>
+      <c r="F84" s="7" t="inlineStr">
+        <is>
+          <t>The event starts at the time the buyer picked and the screen shows that same time (2:30 pm).</t>
+        </is>
+      </c>
+      <c r="G84" s="7" t="inlineStr">
+        <is>
+          <t>The save sends 14:30:00 in the buyer's browser time; the screen then shows 2:29 pm, because it adds the clock gap (timeDiff = −1 s) when it shows the time. With a larger clock gap, the difference is larger.</t>
+        </is>
+      </c>
+      <c r="H84" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I84" s="10" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J84" s="7" t="inlineStr">
+        <is>
+          <t>Screen shows wrong data</t>
+        </is>
+      </c>
+      <c r="K84" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on four fresh test events on PROCOL DEMO with QA vendors only (5 Oct 2026); the save call and the clock gap were recorded each time. Cause in client-dashboard: rescheduleEventModal.jsx sends scheduledDateTime.unix() unshifted, while selectors.js shows start = adjustForClient(starting_from) (server time + timeDiff).</t>
+        </is>
+      </c>
+      <c r="L84" s="7" t="inlineStr">
+        <is>
+          <t>5 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M84" s="7" t="inlineStr">
+        <is>
+          <t>UI-EVDTME-001</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reschedule automation + BUG-83; planner fixes (save before reopen, deliberate skips kept); Settings-menu retry; every failed model provider logged; screen crawl + probe tools
Synced from procol-qa-platform 6293951.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
+++ b/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
@@ -221,8 +221,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:M82" headerRowCount="1">
-  <autoFilter ref="A1:M82"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:M83" headerRowCount="1">
+  <autoFilter ref="A1:M83"/>
   <tableColumns count="13">
     <tableColumn id="1" name="Bug #"/>
     <tableColumn id="2" name="Area"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Confirm" displayName="Confirm" ref="A1:F10" headerRowCount="1">
-  <autoFilter ref="A1:F10"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Confirm" displayName="Confirm" ref="A1:F11" headerRowCount="1">
+  <autoFilter ref="A1:F11"/>
   <tableColumns count="6">
     <tableColumn id="1" name="#"/>
     <tableColumn id="2" name="Area"/>
@@ -583,6 +583,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -590,7 +591,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>COUNTA(Bugs!A2:A82)</f>
+        <f>COUNTA(Bugs!A2:A84)</f>
         <v/>
       </c>
     </row>
@@ -609,7 +610,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF(Bugs!I2:I82,A7)</f>
+        <f>COUNTIF(Bugs!I2:I84,A7)</f>
         <v/>
       </c>
     </row>
@@ -620,7 +621,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF(Bugs!I2:I82,A8)</f>
+        <f>COUNTIF(Bugs!I2:I84,A8)</f>
         <v/>
       </c>
     </row>
@@ -631,7 +632,7 @@
         </is>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIF(Bugs!I2:I82,A9)</f>
+        <f>COUNTIF(Bugs!I2:I84,A9)</f>
         <v/>
       </c>
     </row>
@@ -642,7 +643,7 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIF(Bugs!I2:I82,A10)</f>
+        <f>COUNTIF(Bugs!I2:I84,A10)</f>
         <v/>
       </c>
     </row>
@@ -661,7 +662,7 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF(Bugs!J2:J82,A13)</f>
+        <f>COUNTIF(Bugs!J2:J84,A13)</f>
         <v/>
       </c>
     </row>
@@ -672,7 +673,7 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF(Bugs!J2:J82,A14)</f>
+        <f>COUNTIF(Bugs!J2:J84,A14)</f>
         <v/>
       </c>
     </row>
@@ -683,7 +684,7 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF(Bugs!J2:J82,A15)</f>
+        <f>COUNTIF(Bugs!J2:J84,A15)</f>
         <v/>
       </c>
     </row>
@@ -694,7 +695,7 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF(Bugs!J2:J82,A16)</f>
+        <f>COUNTIF(Bugs!J2:J84,A16)</f>
         <v/>
       </c>
     </row>
@@ -705,7 +706,7 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF(Bugs!J2:J82,A17)</f>
+        <f>COUNTIF(Bugs!J2:J84,A17)</f>
         <v/>
       </c>
     </row>
@@ -716,7 +717,7 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF(Bugs!J2:J82,A18)</f>
+        <f>COUNTIF(Bugs!J2:J84,A18)</f>
         <v/>
       </c>
     </row>
@@ -727,7 +728,7 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF(Bugs!J2:J82,A19)</f>
+        <f>COUNTIF(Bugs!J2:J84,A19)</f>
         <v/>
       </c>
     </row>
@@ -738,7 +739,7 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF(Bugs!J2:J82,A20)</f>
+        <f>COUNTIF(Bugs!J2:J84,A20)</f>
         <v/>
       </c>
     </row>
@@ -749,7 +750,7 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF(Bugs!J2:J82,A21)</f>
+        <f>COUNTIF(Bugs!J2:J84,A21)</f>
         <v/>
       </c>
     </row>
@@ -760,7 +761,7 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF(Bugs!J2:J82,A22)</f>
+        <f>COUNTIF(Bugs!J2:J84,A22)</f>
         <v/>
       </c>
     </row>
@@ -779,7 +780,7 @@
         </is>
       </c>
       <c r="B25" s="5">
-        <f>COUNTIF(Bugs!H2:H82,"*"&amp;A25&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H84,"*"&amp;A25&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -790,7 +791,7 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF(Bugs!H2:H82,"*"&amp;A26&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H84,"*"&amp;A26&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -801,7 +802,7 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF(Bugs!H2:H82,"*"&amp;A27&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H84,"*"&amp;A27&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -820,7 +821,7 @@
         </is>
       </c>
       <c r="B30" s="5">
-        <f>COUNTA('Needs confirmation'!A2:A10)</f>
+        <f>COUNTA('Needs confirmation'!A2:A11)</f>
         <v/>
       </c>
     </row>
@@ -849,7 +850,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M82"/>
+  <dimension ref="A1:M84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -6263,6 +6264,145 @@
         </is>
       </c>
     </row>
+    <row r="83">
+      <c r="A83" s="7" t="inlineStr">
+        <is>
+          <t>BUG-82</t>
+        </is>
+      </c>
+      <c r="B83" s="7" t="inlineStr">
+        <is>
+          <t>Amending a live event</t>
+        </is>
+      </c>
+      <c r="C83" s="7" t="inlineStr">
+        <is>
+          <t>After an amendment, the evaluation window starts and ends before bidding has even closed</t>
+        </is>
+      </c>
+      <c r="D83" s="7" t="inlineStr">
+        <is>
+          <t>A technical round has a bidding window and then an evaluation window that starts when bidding ends. When the buyer issues an amendment (a new version of the event), Procol copies every window of the round but starts all of them at the moment of the amendment. The evaluation window therefore opens together with bidding and, being short, is already over long before bidding closes — so evaluators have no window left once the bids are in.</t>
+        </is>
+      </c>
+      <c r="E83" s="7" t="inlineStr">
+        <is>
+          <t>1. Publish an event with a technical round (bidding 10 minutes, then a short evaluation window).
+2. Issue an amendment (a new version of the event).
+3. Read the amended round's bidding and evaluation windows.</t>
+        </is>
+      </c>
+      <c r="F83" s="7" t="inlineStr">
+        <is>
+          <t>Bidding runs from the amendment for its configured length, and evaluation starts when bidding ends — as on the original event.</t>
+        </is>
+      </c>
+      <c r="G83" s="7" t="inlineStr">
+        <is>
+          <t>Both windows start at the moment of the amendment: bidding 06:32:27 → 06:42:27, evaluation 06:32:27 → 06:32:32 (over ten minutes before bidding closes).</t>
+        </is>
+      </c>
+      <c r="H83" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I83" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J83" s="7" t="inlineStr">
+        <is>
+          <t>Business rule</t>
+        </is>
+      </c>
+      <c r="K83" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on two fresh test events on PROCOL DEMO (4 Oct 2026), read from the amended round's stored windows; on each original event evaluation correctly started when bidding ended. Cause: versions/trade_request.rb replicate_trade_schedules sets every copied window to start now. Whether publishing the amendment re-times the windows was not checked.</t>
+        </is>
+      </c>
+      <c r="L83" s="7" t="inlineStr">
+        <is>
+          <t>4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M83" s="7" t="inlineStr">
+        <is>
+          <t>API-EVRMEG-024, API-EVRLIF-014</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="7" t="inlineStr">
+        <is>
+          <t>BUG-83</t>
+        </is>
+      </c>
+      <c r="B84" s="7" t="inlineStr">
+        <is>
+          <t>Scheduling &amp; rescheduling</t>
+        </is>
+      </c>
+      <c r="C84" s="7" t="inlineStr">
+        <is>
+          <t>A rescheduled start comes back a minute earlier than the buyer picked</t>
+        </is>
+      </c>
+      <c r="D84" s="7" t="inlineStr">
+        <is>
+          <t>The event screen shows every time adjusted for the gap between the buyer's computer clock and Procol's server clock, but the Reschedule dialog saves the picked time without that adjustment. Whenever the two clocks differ, the saved start is off by that gap and the screen then shows a different time from the one the buyer chose. On UAT the browser was 1 second behind the server, so 2:30 pm came back as 2:29 pm.</t>
+        </is>
+      </c>
+      <c r="E84" s="7" t="inlineStr">
+        <is>
+          <t>1. Publish an event that starts later (upcoming).
+2. Event Settings → Reschedule Event.
+3. Pick a new start, e.g. 2:30 pm, and press Ok.
+4. Open Reschedule Event again (or look at the event's start time).</t>
+        </is>
+      </c>
+      <c r="F84" s="7" t="inlineStr">
+        <is>
+          <t>The event starts at the time the buyer picked and the screen shows that same time (2:30 pm).</t>
+        </is>
+      </c>
+      <c r="G84" s="7" t="inlineStr">
+        <is>
+          <t>The save sends 14:30:00 in the buyer's browser time; the screen then shows 2:29 pm, because it adds the clock gap (timeDiff = −1 s) when it shows the time. With a larger clock gap, the difference is larger.</t>
+        </is>
+      </c>
+      <c r="H84" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I84" s="10" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J84" s="7" t="inlineStr">
+        <is>
+          <t>Screen shows wrong data</t>
+        </is>
+      </c>
+      <c r="K84" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on four fresh test events on PROCOL DEMO with QA vendors only (5 Oct 2026); the save call and the clock gap were recorded each time. Cause in client-dashboard: rescheduleEventModal.jsx sends scheduledDateTime.unix() unshifted, while selectors.js shows start = adjustForClient(starting_from) (server time + timeDiff).</t>
+        </is>
+      </c>
+      <c r="L84" s="7" t="inlineStr">
+        <is>
+          <t>5 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M84" s="7" t="inlineStr">
+        <is>
+          <t>UI-EVDTME-001</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
@@ -6277,7 +6417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -6605,6 +6745,38 @@
       <c r="F10" s="7" t="inlineStr">
         <is>
           <t>Confirm in the screen's code whether an older list response can overwrite the search result (a race between the first load and the search). It is intermittent, so it is not yet counted as a verified bug.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Q-10</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Technical evaluation</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>An information-request (RFI) round may close as soon as the first vendor is evaluated</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>In Procol's code, saving any evaluation on an RFI round closes the whole round, because the round counts as 'evaluated' as soon as one evaluation exists (models/evaluation.rb close_trade_request; trade_request_model_helper.rb is_evaluated? for RFI). Vendors not yet evaluated would then meet a closed round. Read in the code only: our runner does not yet build RFI rounds, so it has not been reproduced live.</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>Reproduce on an RFI round with two or more responding vendors, or confirm with the product team whether one evaluation is meant to close an RFI.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Needs confirmation Q-11: the same product added twice becomes two identical rows with no message (UI-LI-016, 3 fresh create screens) — no product rule says otherwise, so asked rather than filed. expect_line_items now reports the count it saw and the products the sheet lists
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
+++ b/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
@@ -821,7 +821,7 @@
         </is>
       </c>
       <c r="B30" s="5">
-        <f>COUNTA('Needs confirmation'!A2:A11)</f>
+        <f>COUNTA('Needs confirmation'!A2:A12)</f>
         <v/>
       </c>
     </row>
@@ -6417,7 +6417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -6777,6 +6777,38 @@
       <c r="F11" s="7" t="inlineStr">
         <is>
           <t>Reproduce on an RFI round with two or more responding vendors, or confirm with the product team whether one evaluation is meant to close an RFI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Q-11</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Line items</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>The same product can be added twice as two separate rows, with no message</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>On the eRFX create screen, adding AAC BLOCKS (1100000401) and then adding it again gives two identical rows in the price sheet (Items shows 2). Nothing merges them, refuses the second one, or says anything. Seen on three fresh create screens on PROCOL DEMO (5 Oct 2026).</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>Confirm whether duplicate rows of one product are intended (e.g. for different delivery locations or specs). If not, should the second add merge the quantity or be refused with a message? Two identical rows make the award ambiguous (PRD §6 lists duplicate products as an edge case but states no rule). Test case UI-LI-016.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Case routing by the case's own setup; Q-11 duplicate products; line-item evidence
Synced from procol-qa-platform a3d0a4c.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
+++ b/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
@@ -821,7 +821,7 @@
         </is>
       </c>
       <c r="B30" s="5">
-        <f>COUNTA('Needs confirmation'!A2:A11)</f>
+        <f>COUNTA('Needs confirmation'!A2:A12)</f>
         <v/>
       </c>
     </row>
@@ -6417,7 +6417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -6777,6 +6777,38 @@
       <c r="F11" s="7" t="inlineStr">
         <is>
           <t>Reproduce on an RFI round with two or more responding vendors, or confirm with the product team whether one evaluation is meant to close an RFI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Q-11</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Line items</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>The same product can be added twice as two separate rows, with no message</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>On the eRFX create screen, adding AAC BLOCKS (1100000401) and then adding it again gives two identical rows in the price sheet (Items shows 2). Nothing merges them, refuses the second one, or says anything. Seen on three fresh create screens on PROCOL DEMO (5 Oct 2026).</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>Confirm whether duplicate rows of one product are intended (e.g. for different delivery locations or specs). If not, should the second add merge the quantity or be refused with a message? Two identical rows make the award ambiguous (PRD §6 lists duplicate products as an edge case but states no rule). Test case UI-LI-016.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
BUG-84: an inverted traffic-light range is refused with 'Traffic light type is required' (one flag for missing and inverted; reproduced live on two pairs). Single-stage configure now reports a refused Save with the app's own words instead of carrying on under an open drawer; an early app refusal is judged by the case's block assertion (skips the steps it made unreachable). SLINGRING_LOG_SIZE logs prompt sizes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
+++ b/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
@@ -591,7 +591,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>COUNTA(Bugs!A2:A84)</f>
+        <f>COUNTA(Bugs!A2:A85)</f>
         <v/>
       </c>
     </row>
@@ -610,7 +610,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF(Bugs!I2:I84,A7)</f>
+        <f>COUNTIF(Bugs!I2:I85,A7)</f>
         <v/>
       </c>
     </row>
@@ -621,7 +621,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF(Bugs!I2:I84,A8)</f>
+        <f>COUNTIF(Bugs!I2:I85,A8)</f>
         <v/>
       </c>
     </row>
@@ -632,7 +632,7 @@
         </is>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIF(Bugs!I2:I84,A9)</f>
+        <f>COUNTIF(Bugs!I2:I85,A9)</f>
         <v/>
       </c>
     </row>
@@ -643,7 +643,7 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIF(Bugs!I2:I84,A10)</f>
+        <f>COUNTIF(Bugs!I2:I85,A10)</f>
         <v/>
       </c>
     </row>
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF(Bugs!J2:J84,A13)</f>
+        <f>COUNTIF(Bugs!J2:J85,A13)</f>
         <v/>
       </c>
     </row>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF(Bugs!J2:J84,A14)</f>
+        <f>COUNTIF(Bugs!J2:J85,A14)</f>
         <v/>
       </c>
     </row>
@@ -684,7 +684,7 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF(Bugs!J2:J84,A15)</f>
+        <f>COUNTIF(Bugs!J2:J85,A15)</f>
         <v/>
       </c>
     </row>
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF(Bugs!J2:J84,A16)</f>
+        <f>COUNTIF(Bugs!J2:J85,A16)</f>
         <v/>
       </c>
     </row>
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF(Bugs!J2:J84,A17)</f>
+        <f>COUNTIF(Bugs!J2:J85,A17)</f>
         <v/>
       </c>
     </row>
@@ -717,7 +717,7 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF(Bugs!J2:J84,A18)</f>
+        <f>COUNTIF(Bugs!J2:J85,A18)</f>
         <v/>
       </c>
     </row>
@@ -728,7 +728,7 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF(Bugs!J2:J84,A19)</f>
+        <f>COUNTIF(Bugs!J2:J85,A19)</f>
         <v/>
       </c>
     </row>
@@ -739,7 +739,7 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF(Bugs!J2:J84,A20)</f>
+        <f>COUNTIF(Bugs!J2:J85,A20)</f>
         <v/>
       </c>
     </row>
@@ -750,7 +750,7 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF(Bugs!J2:J84,A21)</f>
+        <f>COUNTIF(Bugs!J2:J85,A21)</f>
         <v/>
       </c>
     </row>
@@ -761,7 +761,7 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF(Bugs!J2:J84,A22)</f>
+        <f>COUNTIF(Bugs!J2:J85,A22)</f>
         <v/>
       </c>
     </row>
@@ -780,7 +780,7 @@
         </is>
       </c>
       <c r="B25" s="5">
-        <f>COUNTIF(Bugs!H2:H84,"*"&amp;A25&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H85,"*"&amp;A25&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -791,7 +791,7 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF(Bugs!H2:H84,"*"&amp;A26&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H85,"*"&amp;A26&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -802,7 +802,7 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF(Bugs!H2:H84,"*"&amp;A27&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H85,"*"&amp;A27&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -850,7 +850,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M84"/>
+  <dimension ref="A1:M85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -6400,6 +6400,75 @@
       <c r="M84" s="7" t="inlineStr">
         <is>
           <t>UI-EVDTME-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="7" t="inlineStr">
+        <is>
+          <t>BUG-84</t>
+        </is>
+      </c>
+      <c r="B85" s="7" t="inlineStr">
+        <is>
+          <t>Auction configuration</t>
+        </is>
+      </c>
+      <c r="C85" s="7" t="inlineStr">
+        <is>
+          <t>A traffic-light range entered in the wrong order is refused with the message "Traffic light type is required"</t>
+        </is>
+      </c>
+      <c r="D85" s="7" t="inlineStr">
+        <is>
+          <t>When a buyer sets up a traffic-light auction and enters the GREEN limit above the YELLOW limit, Save is correctly refused, but the only message says the traffic light TYPE is required. The type is already chosen and both limits are filled; the actual problem is their order. A buyer is told to fix the wrong thing.</t>
+        </is>
+      </c>
+      <c r="E85" s="7" t="inlineStr">
+        <is>
+          <t>1. Create a single-stage event, Event Type Auction, strategy Traffic Light, award the entire lot.
+2. Enter GREEN "Gross total less than" 100 and YELLOW 50 (green above yellow).
+3. Press Save.</t>
+        </is>
+      </c>
+      <c r="F85" s="7" t="inlineStr">
+        <is>
+          <t>Save is refused with a message about the range (e.g. "Green must be lower than yellow").</t>
+        </is>
+      </c>
+      <c r="G85" s="7" t="inlineStr">
+        <is>
+          <t>Save is refused and the drawer shows "Traffic light type is required". The same message appears for a missing value, so the buyer cannot tell what is wrong.</t>
+        </is>
+      </c>
+      <c r="H85" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I85" s="10" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J85" s="7" t="inlineStr">
+        <is>
+          <t>Wrong message</t>
+        </is>
+      </c>
+      <c r="K85" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced live on fresh create screens on PROCOL DEMO (6 Oct 2026) with two inverted pairs (100/50, 6000/3000); valid pairs (3000/6000, 50/100) save. Cause in client-dashboard: auctionConfiguration.jsx:681-707 sets one flag (errors.trafficLight) for "missing" and "lower above upper", and configuration.jsx:338-344 shows trafficLightValueRequired for it.</t>
+        </is>
+      </c>
+      <c r="L85" s="7" t="inlineStr">
+        <is>
+          <t>6 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M85" s="7" t="inlineStr">
+        <is>
+          <t>UI-AUC-005</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
BUG-84 (wrong traffic-light message); refused configuration judged by the block assertion
Synced from procol-qa-platform 34f450c.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
+++ b/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
@@ -591,7 +591,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>COUNTA(Bugs!A2:A84)</f>
+        <f>COUNTA(Bugs!A2:A85)</f>
         <v/>
       </c>
     </row>
@@ -610,7 +610,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF(Bugs!I2:I84,A7)</f>
+        <f>COUNTIF(Bugs!I2:I85,A7)</f>
         <v/>
       </c>
     </row>
@@ -621,7 +621,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF(Bugs!I2:I84,A8)</f>
+        <f>COUNTIF(Bugs!I2:I85,A8)</f>
         <v/>
       </c>
     </row>
@@ -632,7 +632,7 @@
         </is>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIF(Bugs!I2:I84,A9)</f>
+        <f>COUNTIF(Bugs!I2:I85,A9)</f>
         <v/>
       </c>
     </row>
@@ -643,7 +643,7 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIF(Bugs!I2:I84,A10)</f>
+        <f>COUNTIF(Bugs!I2:I85,A10)</f>
         <v/>
       </c>
     </row>
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF(Bugs!J2:J84,A13)</f>
+        <f>COUNTIF(Bugs!J2:J85,A13)</f>
         <v/>
       </c>
     </row>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF(Bugs!J2:J84,A14)</f>
+        <f>COUNTIF(Bugs!J2:J85,A14)</f>
         <v/>
       </c>
     </row>
@@ -684,7 +684,7 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF(Bugs!J2:J84,A15)</f>
+        <f>COUNTIF(Bugs!J2:J85,A15)</f>
         <v/>
       </c>
     </row>
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF(Bugs!J2:J84,A16)</f>
+        <f>COUNTIF(Bugs!J2:J85,A16)</f>
         <v/>
       </c>
     </row>
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF(Bugs!J2:J84,A17)</f>
+        <f>COUNTIF(Bugs!J2:J85,A17)</f>
         <v/>
       </c>
     </row>
@@ -717,7 +717,7 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF(Bugs!J2:J84,A18)</f>
+        <f>COUNTIF(Bugs!J2:J85,A18)</f>
         <v/>
       </c>
     </row>
@@ -728,7 +728,7 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF(Bugs!J2:J84,A19)</f>
+        <f>COUNTIF(Bugs!J2:J85,A19)</f>
         <v/>
       </c>
     </row>
@@ -739,7 +739,7 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF(Bugs!J2:J84,A20)</f>
+        <f>COUNTIF(Bugs!J2:J85,A20)</f>
         <v/>
       </c>
     </row>
@@ -750,7 +750,7 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF(Bugs!J2:J84,A21)</f>
+        <f>COUNTIF(Bugs!J2:J85,A21)</f>
         <v/>
       </c>
     </row>
@@ -761,7 +761,7 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF(Bugs!J2:J84,A22)</f>
+        <f>COUNTIF(Bugs!J2:J85,A22)</f>
         <v/>
       </c>
     </row>
@@ -780,7 +780,7 @@
         </is>
       </c>
       <c r="B25" s="5">
-        <f>COUNTIF(Bugs!H2:H84,"*"&amp;A25&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H85,"*"&amp;A25&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -791,7 +791,7 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF(Bugs!H2:H84,"*"&amp;A26&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H85,"*"&amp;A26&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -802,7 +802,7 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF(Bugs!H2:H84,"*"&amp;A27&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H85,"*"&amp;A27&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -850,7 +850,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M84"/>
+  <dimension ref="A1:M85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -6400,6 +6400,75 @@
       <c r="M84" s="7" t="inlineStr">
         <is>
           <t>UI-EVDTME-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="7" t="inlineStr">
+        <is>
+          <t>BUG-84</t>
+        </is>
+      </c>
+      <c r="B85" s="7" t="inlineStr">
+        <is>
+          <t>Auction configuration</t>
+        </is>
+      </c>
+      <c r="C85" s="7" t="inlineStr">
+        <is>
+          <t>A traffic-light range entered in the wrong order is refused with the message "Traffic light type is required"</t>
+        </is>
+      </c>
+      <c r="D85" s="7" t="inlineStr">
+        <is>
+          <t>When a buyer sets up a traffic-light auction and enters the GREEN limit above the YELLOW limit, Save is correctly refused, but the only message says the traffic light TYPE is required. The type is already chosen and both limits are filled; the actual problem is their order. A buyer is told to fix the wrong thing.</t>
+        </is>
+      </c>
+      <c r="E85" s="7" t="inlineStr">
+        <is>
+          <t>1. Create a single-stage event, Event Type Auction, strategy Traffic Light, award the entire lot.
+2. Enter GREEN "Gross total less than" 100 and YELLOW 50 (green above yellow).
+3. Press Save.</t>
+        </is>
+      </c>
+      <c r="F85" s="7" t="inlineStr">
+        <is>
+          <t>Save is refused with a message about the range (e.g. "Green must be lower than yellow").</t>
+        </is>
+      </c>
+      <c r="G85" s="7" t="inlineStr">
+        <is>
+          <t>Save is refused and the drawer shows "Traffic light type is required". The same message appears for a missing value, so the buyer cannot tell what is wrong.</t>
+        </is>
+      </c>
+      <c r="H85" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I85" s="10" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J85" s="7" t="inlineStr">
+        <is>
+          <t>Wrong message</t>
+        </is>
+      </c>
+      <c r="K85" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced live on fresh create screens on PROCOL DEMO (6 Oct 2026) with two inverted pairs (100/50, 6000/3000); valid pairs (3000/6000, 50/100) save. Cause in client-dashboard: auctionConfiguration.jsx:681-707 sets one flag (errors.trafficLight) for "missing" and "lower above upper", and configuration.jsx:338-344 shows trafficLightValueRequired for it.</t>
+        </is>
+      </c>
+      <c r="L85" s="7" t="inlineStr">
+        <is>
+          <t>6 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M85" s="7" t="inlineStr">
+        <is>
+          <t>UI-AUC-005</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
BUG-85: the RFP-vs-RFQ end check compares a fixed end timestamp with a duration (refused although the RFP ends first; never fires the other way). Schedule step: one block per stage — every stage stays on Duration on a multi-stage event, each block's own end is read back before Save and reported (a 3-minute end that did not take was reported as saved). The user's 10-item RFP+RFQ flow now publishes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
+++ b/docs/bugs/Procol_bugs_found_2026-10-03.xlsx
@@ -591,7 +591,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>COUNTA(Bugs!A2:A85)</f>
+        <f>COUNTA(Bugs!A2:A86)</f>
         <v/>
       </c>
     </row>
@@ -610,7 +610,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF(Bugs!I2:I85,A7)</f>
+        <f>COUNTIF(Bugs!I2:I86,A7)</f>
         <v/>
       </c>
     </row>
@@ -621,7 +621,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF(Bugs!I2:I85,A8)</f>
+        <f>COUNTIF(Bugs!I2:I86,A8)</f>
         <v/>
       </c>
     </row>
@@ -632,7 +632,7 @@
         </is>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIF(Bugs!I2:I85,A9)</f>
+        <f>COUNTIF(Bugs!I2:I86,A9)</f>
         <v/>
       </c>
     </row>
@@ -643,7 +643,7 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIF(Bugs!I2:I85,A10)</f>
+        <f>COUNTIF(Bugs!I2:I86,A10)</f>
         <v/>
       </c>
     </row>
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF(Bugs!J2:J85,A13)</f>
+        <f>COUNTIF(Bugs!J2:J86,A13)</f>
         <v/>
       </c>
     </row>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF(Bugs!J2:J85,A14)</f>
+        <f>COUNTIF(Bugs!J2:J86,A14)</f>
         <v/>
       </c>
     </row>
@@ -684,7 +684,7 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF(Bugs!J2:J85,A15)</f>
+        <f>COUNTIF(Bugs!J2:J86,A15)</f>
         <v/>
       </c>
     </row>
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF(Bugs!J2:J85,A16)</f>
+        <f>COUNTIF(Bugs!J2:J86,A16)</f>
         <v/>
       </c>
     </row>
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF(Bugs!J2:J85,A17)</f>
+        <f>COUNTIF(Bugs!J2:J86,A17)</f>
         <v/>
       </c>
     </row>
@@ -717,7 +717,7 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF(Bugs!J2:J85,A18)</f>
+        <f>COUNTIF(Bugs!J2:J86,A18)</f>
         <v/>
       </c>
     </row>
@@ -728,7 +728,7 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF(Bugs!J2:J85,A19)</f>
+        <f>COUNTIF(Bugs!J2:J86,A19)</f>
         <v/>
       </c>
     </row>
@@ -739,7 +739,7 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF(Bugs!J2:J85,A20)</f>
+        <f>COUNTIF(Bugs!J2:J86,A20)</f>
         <v/>
       </c>
     </row>
@@ -750,7 +750,7 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF(Bugs!J2:J85,A21)</f>
+        <f>COUNTIF(Bugs!J2:J86,A21)</f>
         <v/>
       </c>
     </row>
@@ -761,7 +761,7 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF(Bugs!J2:J85,A22)</f>
+        <f>COUNTIF(Bugs!J2:J86,A22)</f>
         <v/>
       </c>
     </row>
@@ -780,7 +780,7 @@
         </is>
       </c>
       <c r="B25" s="5">
-        <f>COUNTIF(Bugs!H2:H85,"*"&amp;A25&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H86,"*"&amp;A25&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -791,7 +791,7 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF(Bugs!H2:H85,"*"&amp;A26&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H86,"*"&amp;A26&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -802,7 +802,7 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF(Bugs!H2:H85,"*"&amp;A27&amp;"*")</f>
+        <f>COUNTIF(Bugs!H2:H86,"*"&amp;A27&amp;"*")</f>
         <v/>
       </c>
     </row>
@@ -850,7 +850,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M85"/>
+  <dimension ref="A1:M86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -6469,6 +6469,75 @@
       <c r="M85" s="7" t="inlineStr">
         <is>
           <t>UI-AUC-005</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="7" t="inlineStr">
+        <is>
+          <t>BUG-85</t>
+        </is>
+      </c>
+      <c r="B86" s="7" t="inlineStr">
+        <is>
+          <t>Event scheduling (eRFX)</t>
+        </is>
+      </c>
+      <c r="C86" s="7" t="inlineStr">
+        <is>
+          <t>Publish is refused with "RFP duration exceeds RFQ end time" when the technical stage uses a fixed end time, even though it ends before the RFQ</t>
+        </is>
+      </c>
+      <c r="D86" s="7" t="inlineStr">
+        <is>
+          <t>On a project with a technical (RFP) stage and an RFQ stage, the app checks that the technical stage ends no later than the RFQ. The check compares each stage's stored end value directly, but that value is a length in seconds when the end is set as a Duration and a clock timestamp when it is set as a Fixed time. With the technical stage on Fixed time and the RFQ on Duration, a timestamp is compared with a duration, so publish is always refused. In the other direction (technical on Duration, RFQ on Fixed time) the check can never fire, so a technical stage that really runs past the RFQ is let through.</t>
+        </is>
+      </c>
+      <c r="E86" s="7" t="inlineStr">
+        <is>
+          <t>1. Create an eRFX project with a Technical stage and an RFQ stage, a template, line items, an evaluator and one participant.
+2. Open the schedule. Technical Stage: End time = Fixed time, 3 minutes from now. RFQ: End time = Duration, 30 Mins.
+3. Save Schedule and Publish.</t>
+        </is>
+      </c>
+      <c r="F86" s="7" t="inlineStr">
+        <is>
+          <t>Publish succeeds: the technical stage ends (e.g. 04:58 PM) before the RFQ (05:25 PM).</t>
+        </is>
+      </c>
+      <c r="G86" s="7" t="inlineStr">
+        <is>
+          <t>Publish is refused with "RFP duration exceeds RFQ end time. Please adjust." With both stages on Duration (30 Mins each) the same event publishes.</t>
+        </is>
+      </c>
+      <c r="H86" s="7" t="inlineStr">
+        <is>
+          <t>PROCOL DEMO</t>
+        </is>
+      </c>
+      <c r="I86" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J86" s="7" t="inlineStr">
+        <is>
+          <t>Business rule</t>
+        </is>
+      </c>
+      <c r="K86" s="7" t="inlineStr">
+        <is>
+          <t>Reproduced on two fresh events on PROCOL DEMO (8 Oct 2026, one run by the user, one by spine.ai with the panel captured before Save: technical ends 04:58 PM, RFQ ends 05:25 PM, refused). Cause in client-dashboard: projectCreation.jsx:1609-1622 compares stageConfig[].eventEndTime, which projectScheduler.jsx:99 sets to endTimeValue — a duration for EVENT_TIME_SCHEDULE_TYPE.relative and a timestamp for absolute (projectScheduler/helpers.js:24-27).</t>
+        </is>
+      </c>
+      <c r="L86" s="7" t="inlineStr">
+        <is>
+          <t>8 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M86" s="7" t="inlineStr">
+        <is>
+          <t>UI flow: RFP+RFQ with a short schedule</t>
         </is>
       </c>
     </row>

</xml_diff>